<commit_message>
Append v0.9 delivery and Excel handoff to iteration workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,11 +14,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'使用与维护'!$A$5:$B$17</definedName>
   </definedNames>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H11" headerRowCount="1">
-  <autoFilter ref="A5:H11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H13" headerRowCount="1">
+  <autoFilter ref="A5:H13"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L41" headerRowCount="1">
-  <autoFilter ref="A5:L41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L47" headerRowCount="1">
+  <autoFilter ref="A5:L47"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -264,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H9" headerRowCount="1">
-  <autoFilter ref="A5:H9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H8" headerRowCount="1">
+  <autoFilter ref="A5:H8"/>
   <tableColumns count="8">
     <tableColumn id="1" name="顺序"/>
     <tableColumn id="2" name="优先级"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 6 个阶段、36 项内容  |  当前功能版本 v0.8  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 8 个阶段、42 项内容  |  当前功能版本 v0.9  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -870,6 +870,78 @@
       <c r="H11" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/a45d069</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>文档补充</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>功能迭代 Excel 与维护机制</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>工作簿生成并重读、序号/链接/计划状态校验，GitHub 下载散列核对</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/07a46db</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>v0.9</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>统一审批待办与任务信息</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>36 项业务测试、33 项浏览器场景；生产产物同构路径验证通过</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/5f5bb2b</t>
         </is>
       </c>
     </row>
@@ -886,6 +958,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId8"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -899,7 +973,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
@@ -911,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3096,6 +3170,354 @@
       <c r="L41" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.8.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="88" customHeight="1">
+      <c r="A42" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>文档补充</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>项目管理</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>可持续维护的功能迭代 Excel</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>按顺序回顾新增内容并支持面试准备</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>仓库 deliverables/qingbao-feature-history.xlsx</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>打开阶段总览、历史明细、下一步计划及维护说明</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>工作簿生成并重读、序号/链接/计划状态校验，GitHub 下载散列核对</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>阶段内按演示逻辑排序；计划不标为已完成</t>
+        </is>
+      </c>
+      <c r="L42" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/07a46db/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="88" customHeight="1">
+      <c r="A43" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>v0.9</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>统一审批</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>费用申请、报销和付款统一待办</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>减少审批人跨模块寻找任务的入口切换</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>主管/财务 → 审批中心</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>林晓提交申请和报销，赵航在同页打开并处理</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>36 项业务测试、33 项浏览器场景；生产产物同构路径验证通过</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>按当前具体人员；无真实账号认证或批量审批</t>
+        </is>
+      </c>
+      <c r="L43" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.9.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="88" customHeight="1">
+      <c r="A44" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>v0.9</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>任务进度</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>当前节点、处理人、流程版本及进度</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>在列表解释当前责任和审批所处阶段</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>审批中心 → 当前阶段/审批进度</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>赵航通过后切许明，查看下一节点及 1/2 进度</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>36 项业务测试、33 项浏览器场景；生产产物同构路径验证通过</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>旧单据显示历史固定流程，不补写快照</t>
+        </is>
+      </c>
+      <c r="L44" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.9.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="88" customHeight="1">
+      <c r="A45" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>v0.9</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>查找与排序</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>类型筛选、关键词搜索及提交时间排序</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>快速定位本人可处理的单据</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>审批中心 → 类型/搜索/提交时间</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>筛选费用申请，搜索姓名，再切最早/最新排序</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>36 项业务测试、33 项浏览器场景；生产产物同构路径验证通过</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>未知历史提交时间排最后，不用费用日期代替</t>
+        </is>
+      </c>
+      <c r="L45" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.9.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="88" customHeight="1">
+      <c r="A46" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>v0.9</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>待办一致性</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>角标刷新、身份切换清筛选及付款保留</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>减少筛选误解和漏掉付款登记</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>侧栏审批中心角标/概览/模拟身份</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>处理申请观察角标，财务审核后查看付款任务</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>36 项业务测试、33 项浏览器场景；生产产物同构路径验证通过</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>筛选只影响列表；付款登记完成才从财务待办移出</t>
+        </is>
+      </c>
+      <c r="L46" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.9.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="88" customHeight="1">
+      <c r="A47" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>v0.9</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>导出与异常</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>当前筛选 CSV 导出与损坏存储提示</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>支持复核待办且避免导出假完整列表</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>审批中心 → 导出当前列表</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>筛选申请并导出 CSV，核对仅有当前范围</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>36 项业务测试、33 项浏览器场景；生产产物同构路径验证通过</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>CSV 防公式注入；申请存储损坏时明确提示不完整并拦截导出</t>
+        </is>
+      </c>
+      <c r="L47" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.9.md</t>
         </is>
       </c>
     </row>
@@ -3142,6 +3564,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId42"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3155,7 +3583,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId43"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3167,7 +3595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3190,14 +3618,14 @@
     <row r="2" ht="38" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>以下是建议及待办，尚未交付。下一阶段建议优先开发统一审批待办，本次仅整理记录表。</t>
+          <t>以下是建议及待办，尚未交付。已完成项已移入历史新增明细，不继续混在计划中。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：统一审批入口 → 进度信息完善 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
+          <t>建议顺序：我的已处理记录 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
         </is>
       </c>
     </row>
@@ -3249,12 +3677,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>统一审批待办</t>
+          <t>我的已处理记录</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -3264,22 +3692,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>费用申请与报销需要分别查找和处理</t>
+          <t>当前待办处理后移出，审批人需回看自己的处理动作</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>将当前身份可处理的申请、报销集中在审批中心，按类型筛选并跳转详情</t>
+          <t>依据具名审批记录呈现本人已处理单据、结果及处理时间，并可回看详情</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>只显示本人当前节点；两类单据能打开和处理；通过后待办与角标同步；旧单据兼容</t>
+          <t>严格区分本人处理与仅同角色处理；多次处理和退回重提有明确口径；不伪造旧记录责任人</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>可在现有免费云环境自主开发</t>
+          <t>需先定义历史记录可归属范围及兼容策略</t>
         </is>
       </c>
     </row>
@@ -3294,32 +3722,32 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>待办与历史进度信息完善</t>
+          <t>真实可用性测试</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>待排期</t>
+          <t>待用户参与</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>列表中需要快速理解当前节点及处理进度</t>
+          <t>自动化测试不能证明真实用户理解和使用顺畅</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>显示单据类型、当前处理人、流程版本与处理状态，按提交时间排序</t>
+          <t>使用已准备任务，收集员工、主管、财务参与者的真实操作反馈</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>展示内容与审批快照一致；旧记录明确标为旧流程；手机可读</t>
+          <t>记录真实任务完成情况、困惑点与改进建议；无参与者前不写研究结论</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>统一待办完成后，按实际使用反馈确定范围</t>
+          <t>需要用户协助招募实际参与者；AI 不能代替真实访谈</t>
         </is>
       </c>
     </row>
@@ -3329,75 +3757,35 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>真实可用性测试</t>
+          <t>复杂审批能力评估</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>待用户参与</t>
+          <t>暂缓</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>自动化测试不能证明真实用户理解和使用顺畅</t>
+          <t>尚无证据证明会签、或签、加签和嵌套条件为当前作品优先需求</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>使用已准备任务，收集员工、主管、财务参与者的真实操作反馈</t>
+          <t>先依据组织与审批树试用反馈，再决定是否扩展</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>记录真实任务完成情况、困惑点与改进建议；无参与者前不写研究结论</t>
+          <t>明确业务场景、异常策略与范围后再排开发</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>需要用户协助招募实际参与者；AI 不能代替真实访谈</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="100" customHeight="1">
-      <c r="A9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>复杂审批能力评估</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>暂缓</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>尚无证据证明会签、或签、加签和嵌套条件为当前作品优先需求</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>先依据组织与审批树试用反馈，再决定是否扩展</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>明确业务场景、异常策略与范围后再排开发</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>不在当前 Excel 中记为已完成</t>
         </is>
@@ -3596,12 +3984,12 @@
     <row r="16" ht="50" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>本次记录表交付</t>
+          <t>本轮更新</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>新增历史回溯、阶段总览、后续计划及维护说明；仅整理文档和 Excel，本次没有开发统一审批待办。</t>
+          <t>v0.9 完成统一审批待办、任务进度、筛选排序与导出，历史记录追加并更新后续计划；上轮 Excel 文档交付已补记。</t>
         </is>
       </c>
     </row>
@@ -3613,7 +4001,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.8-final</t>
+          <t>https://jameyan42.github.io/-/?v=0.9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append graphical organization and finance roles to feature workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$47</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H13" headerRowCount="1">
-  <autoFilter ref="A5:H13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H14" headerRowCount="1">
+  <autoFilter ref="A5:H14"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L47" headerRowCount="1">
-  <autoFilter ref="A5:L47"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L54" headerRowCount="1">
+  <autoFilter ref="A5:L54"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 8 个阶段、42 项内容  |  当前功能版本 v0.9  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 9 个阶段、49 项内容  |  当前功能版本 v0.10  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -942,6 +942,42 @@
       <c r="H13" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/5f5bb2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="74" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>v0.10</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>图形组织与财务岗位分工</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>42 项业务测试、38 项浏览器场景通过；修正后相关5项重跑及生产产物全链路通过</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/a1cd75d</t>
         </is>
       </c>
     </row>
@@ -960,6 +996,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId9"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -973,7 +1010,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>
@@ -985,7 +1022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3518,6 +3555,412 @@
       <c r="L47" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.9.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="88" customHeight="1">
+      <c r="A48" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>v0.10</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>组织画布</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>图形节点连接线、缩放与展开折叠</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>用类似思维导图的布局理解组织上下级</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>管理员 → 组织架构 → 汇报树/部门树</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>查看 CFO 及四部门，折叠、缩放、适应画布</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>42 项业务测试、38 项浏览器场景通过；修正后相关5项重跑及生产产物全链路通过</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>画布内部滚动；尚不支持拖拽节点改上级</t>
+        </is>
+      </c>
+      <c r="L48" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.10.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="88" customHeight="1">
+      <c r="A49" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>v0.10</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>组织维护</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>点选侧栏编辑岗位上级及快捷添加</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>减少管理人员切换表单的操作</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>组织画布节点/右侧资料栏</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>点部门总编辑岗位，在卡片上添加下级或子部门</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>42 项业务测试、38 项浏览器场景通过；修正后相关5项重跑及生产产物全链路通过</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>已有姓名及部门名称保留；循环或失效引用拦截</t>
+        </is>
+      </c>
+      <c r="L49" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.10.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="88" customHeight="1">
+      <c r="A50" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>v0.10</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>示例与兼容</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>CFO 及法报预算资金税务示例组织</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>贴近用户提出的财务组织结构</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>组织架构；旧组织可追加 CFO 示例</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>查看 CFO—部门总—员工层级</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>42 项业务测试、38 项浏览器场景通过；修正后相关5项重跑及生产产物全链路通过</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>新安装21人8部门；旧组织只追加，不替换原关系</t>
+        </is>
+      </c>
+      <c r="L50" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.10.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="88" customHeight="1">
+      <c r="A51" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>v0.10</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>流程分工</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>部门负责人—财务—总账—付款模板</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>区分业务审批、财务审核、总账复核和付款职责</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>管理员 → 审批流程 → 财务分工模板</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>载入草稿，配置总账及付款人，填写原因发布</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>42 项业务测试、38 项浏览器场景通过；修正后相关5项重跑及生产产物全链路通过</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>不静默更改运行配置；旧单据保留原路径；CFO不自动必经</t>
+        </is>
+      </c>
+      <c r="L51" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.10.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="88" customHeight="1">
+      <c r="A52" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>v0.10</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>总账复核</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>总账角色、科目核算归属与复核记录</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>通过前明确会计核算信息及责任</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>总账高璇 → 审批中心</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>填写6602科目和法报中心核算归属后通过</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>42 项业务测试、38 项浏览器场景通过；修正后相关5项重跑及生产产物全链路通过</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>未填或有未解决风险不能通过；不生成凭证或自动入账</t>
+        </is>
+      </c>
+      <c r="L52" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.10.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="88" customHeight="1">
+      <c r="A53" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>v0.10</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>付款工作台</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>独立付款岗位、待付已付筛选与搜索</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>集中处理已复核的报销并回看付款结果</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>付款杜川 → 付款工作台</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>登记模拟参考号后到已付款查询</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>42 项业务测试、38 项浏览器场景通过；修正后相关5项重跑及生产产物全链路通过</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>无银行接口或批量付款；管理员只读；旧单据仍由原财务登记</t>
+        </is>
+      </c>
+      <c r="L53" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.10.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="88" customHeight="1">
+      <c r="A54" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>v0.10</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>历史与保护</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>新快照、未来付款责任保护及总账备份校验</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>防止流程升级或人员停用破坏在途责任</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>组织维护/报销详情/数据管理</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>新旧流程并存，导出恢复总账记录与独立付款人</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>42 项业务测试、38 项浏览器场景通过；修正后相关5项重跑及生产产物全链路通过</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>schema 2新报销有独立付款责任；schema 1旧路径不自动迁移</t>
+        </is>
+      </c>
+      <c r="L54" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.10.md</t>
         </is>
       </c>
     </row>
@@ -3570,6 +4013,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId49"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3583,7 +4033,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId43"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId50"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3737,7 +4187,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>使用已准备任务，收集员工、主管、财务参与者的真实操作反馈</t>
+          <t>结合图形组织、部门总/财务/总账/付款路径，使用已准备任务收集真实参与者操作反馈</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -3989,7 +4439,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.9 完成统一审批待办、任务进度、筛选排序与导出，历史记录追加并更新后续计划；上轮 Excel 文档交付已补记。</t>
+          <t>v0.10 完成图形组织画布、节点维护、财务分工模板、总账复核和付款工作台；历史记录持续追加，开发完成系统弹窗尚未配置。</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4451,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.9</t>
+          <t>https://jameyan42.github.io/-/?v=0.10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append processed records release to feature history workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$14</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$54</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$59</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H14" headerRowCount="1">
-  <autoFilter ref="A5:H14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H15" headerRowCount="1">
+  <autoFilter ref="A5:H15"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L54" headerRowCount="1">
-  <autoFilter ref="A5:L54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L59" headerRowCount="1">
+  <autoFilter ref="A5:L59"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 9 个阶段、49 项内容  |  当前功能版本 v0.10  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 10 个阶段、54 项内容  |  当前功能版本 v0.11  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -978,6 +978,42 @@
       <c r="H14" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/a1cd75d</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="74" customHeight="1">
+      <c r="A15" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>我的已处理记录与历史摘要</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>48项业务测试、44项浏览器场景通过；生产同构路径退回重提、历史摘要及手机验证通过</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/09e9e3c</t>
         </is>
       </c>
     </row>
@@ -997,6 +1033,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId10"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1010,7 +1047,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1022,7 +1059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3961,6 +3998,296 @@
       <c r="L54" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.10.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="88" customHeight="1">
+      <c r="A55" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>审批已办</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>待办/已办双视图及精确人员归属</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>审批人可回看本人处理而不混入同角色其他人员</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>审批中心 → 我已处理</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>处理一笔申请后查看本人记录，再切其他主管</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>48项业务测试、44项浏览器场景通过；生产同构路径退回重提、历史摘要及手机验证通过</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>旧日志无人员标识不推断；初次升级可能为空</t>
+        </is>
+      </c>
+      <c r="L55" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.11.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="88" customHeight="1">
+      <c r="A56" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>历史摘要</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>按每次操作保留结果、原事项金额及版本时间</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>退回重提后仍能解释过去的处理结果</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>我已处理 → 处理时摘要/处理后与当前状态</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>200元原事项退回，修改600元重提后通过，对比两条记录</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>48项业务测试、44项浏览器场景通过；生产同构路径退回重提、历史摘要及手机验证通过</t>
+        </is>
+      </c>
+      <c r="K56" s="5" t="inlineStr">
+        <is>
+          <t>按处理次数非单据去重；提交快照时间仅作轮次参考</t>
+        </is>
+      </c>
+      <c r="L56" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.11.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="88" customHeight="1">
+      <c r="A57" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>岗位留痕</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>总账核算与付款摘要分别留存</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>总账与付款人员可回看自己的实际处理内容</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>总账/付款人员 → 我已处理</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>分别查看科目归属和付款参考号</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>48项业务测试、44项浏览器场景通过；生产同构路径退回重提、历史摘要及手机验证通过</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>点击当前单据打开最新状态；原摘要不冒充当前字段</t>
+        </is>
+      </c>
+      <c r="L57" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.11.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="88" customHeight="1">
+      <c r="A58" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>记录浏览</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>类型结果筛选、搜索排序与20条分页</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>在记录增长时便于定位本人已办操作</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>我已处理 → 筛选/搜索/处理时间/翻页</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>筛选退回、搜索备注，翻页后重新筛选回到首页</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>48项业务测试、44项浏览器场景通过；生产同构路径退回重提、历史摘要及手机验证通过</t>
+        </is>
+      </c>
+      <c r="K58" s="5" t="inlineStr">
+        <is>
+          <t>不按处理次数累加支出金额；无日期区间筛选</t>
+        </is>
+      </c>
+      <c r="L58" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.11.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="88" customHeight="1">
+      <c r="A59" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>v0.11</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>导出备份</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>筛选全量CSV与具名元数据备份校验</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>跨页导出及恢复后仍保留可归属的处理记录</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>我已处理导出/数据管理</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>25条分页结果全部导出，恢复备份后回看</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>48项业务测试、44项浏览器场景通过；生产同构路径退回重提、历史摘要及手机验证通过</t>
+        </is>
+      </c>
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>CSV防公式注入；损坏申请存储拦截假完整导出；本地日志不防篡改</t>
+        </is>
+      </c>
+      <c r="L59" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.11.md</t>
         </is>
       </c>
     </row>
@@ -4020,6 +4347,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId54"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4033,7 +4365,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId50"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId55"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4075,7 +4407,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：我的已处理记录 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
+          <t>建议顺序：组织画布查找与定位 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4464,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>我的已处理记录</t>
+          <t>组织画布查找与定位</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -4142,22 +4474,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>当前待办处理后移出，审批人需回看自己的处理动作</t>
+          <t>组织规模增大后图形画布需要更快找到人员及部门</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>依据具名审批记录呈现本人已处理单据、结果及处理时间，并可回看详情</t>
+          <t>评估按姓名、岗位、部门检索并定位节点，保持原组织关系和折叠语义清晰</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>严格区分本人处理与仅同角色处理；多次处理和退回重提有明确口径；不伪造旧记录责任人</t>
+          <t>搜索定位不修改组织；能解释隐藏和折叠的节点；手机可操作</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>需先定义历史记录可归属范围及兼容策略</t>
+          <t>先收集用户实际操作反馈，避免增加无验证价值的控件</t>
         </is>
       </c>
     </row>
@@ -4439,7 +4771,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.10 完成图形组织画布、节点维护、财务分工模板、总账复核和付款工作台；历史记录持续追加，开发完成系统弹窗尚未配置。</t>
+          <t>v0.11 完成本人已处理记录、每次操作历史摘要、总账付款留痕、分页和筛选全量导出；计划中的已处理记录已移入完成历史。</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4783,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.10</t>
+          <t>https://jameyan42.github.io/-/?v=0.11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append organization search release to maintained feature workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$59</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H15" headerRowCount="1">
-  <autoFilter ref="A5:H15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H16" headerRowCount="1">
+  <autoFilter ref="A5:H16"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L59" headerRowCount="1">
-  <autoFilter ref="A5:L59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L63" headerRowCount="1">
+  <autoFilter ref="A5:L63"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 10 个阶段、54 项内容  |  当前功能版本 v0.11  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 11 个阶段、58 项内容  |  当前功能版本 v0.12  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1014,6 +1014,42 @@
       <c r="H15" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/09e9e3c</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="74" customHeight="1">
+      <c r="A16" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>v0.12</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>组织画布查找与路径定位</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>53项业务测试、49项浏览器场景通过；生产路径折叠定位、配置不变和手机验证通过</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/dab7d76</t>
         </is>
       </c>
     </row>
@@ -1034,6 +1070,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId11"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1047,7 +1084,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1059,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4288,6 +4325,238 @@
       <c r="L59" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.11.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="88" customHeight="1">
+      <c r="A60" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>v0.12</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>组织检索</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>姓名岗位部门角色搜索及范围与停用标记</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>在组织变大时更快找到人员或部门</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>组织架构 → 查找组织节点</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>搜索叶禾、CFO、总账或法报中心，限定人员/部门</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>53项业务测试、49项浏览器场景通过；生产路径折叠定位、配置不变和手机验证通过</t>
+        </is>
+      </c>
+      <c r="K60" s="5" t="inlineStr">
+        <is>
+          <t>包含匹配；无拼音、模糊纠错或组合条件</t>
+        </is>
+      </c>
+      <c r="L60" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.12.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="88" customHeight="1">
+      <c r="A61" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>v0.12</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>画布定位</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>展开祖先、可读缩放与节点居中</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>目标被折叠或位于画布之外时仍可定位</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>组织搜索结果</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>先折叠CFO，再点叶禾结果，观察侧栏和高亮</t>
+        </is>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>53项业务测试、49项浏览器场景通过；生产路径折叠定位、配置不变和手机验证通过</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="inlineStr">
+        <is>
+          <t>只展开上级，保留其他折叠；部门结果切到归属图</t>
+        </is>
+      </c>
+      <c r="L61" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.12.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="88" customHeight="1">
+      <c r="A62" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>v0.12</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>关系导航</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>汇报归属路径与回到选中节点</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>保留关系语境，手动平移后可快速返回</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>组织画布路径导航/定位选中节点</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>点击沈岚祖先，或平移后定位当前选择</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>53项业务测试、49项浏览器场景通过；生产路径折叠定位、配置不变和手机验证通过</t>
+        </is>
+      </c>
+      <c r="K62" s="5" t="inlineStr">
+        <is>
+          <t>清除搜索保留选择和视图，不修改组织与审批</t>
+        </is>
+      </c>
+      <c r="L62" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.12.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="88" customHeight="1">
+      <c r="A63" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>v0.12</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>编辑保护</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>搜索切页切身份的未保存资料提醒</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>避免维护资料时因定位或换页面丢失修改</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>组织资料侧栏/搜索/导航/角色</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr">
+        <is>
+          <t>修改岗位后搜索或切页，取消提醒保留字段</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>53项业务测试、49项浏览器场景通过；生产路径折叠定位、配置不变和手机验证通过</t>
+        </is>
+      </c>
+      <c r="K63" s="5" t="inlineStr">
+        <is>
+          <t>仅前端编辑保护；无生产认证或版本并发控制</t>
+        </is>
+      </c>
+      <c r="L63" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.12.md</t>
         </is>
       </c>
     </row>
@@ -4352,6 +4621,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L60" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L61" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L62" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId58"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4365,7 +4638,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId55"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId59"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4407,7 +4680,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：组织画布查找与定位 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
+          <t>建议顺序：已处理记录日期区间筛选 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4737,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>组织画布查找与定位</t>
+          <t>已处理记录日期区间筛选</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -4474,22 +4747,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>组织规模增大后图形画布需要更快找到人员及部门</t>
+          <t>处理历史增长后需要回看某段时间内本人操作</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>评估按姓名、岗位、部门检索并定位节点，保持原组织关系和折叠语义清晰</t>
+          <t>评估起止日期、常用时间段与现有筛选导出的联动</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>搜索定位不修改组织；能解释隐藏和折叠的节点；手机可操作</t>
+          <t>明确本地日期时区与起止包含口径，倒置范围提示，跨页导出与筛选一致</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>先收集用户实际操作反馈，避免增加无验证价值的控件</t>
+          <t>先确定产品口径并结合实际使用反馈，不将日期筛选写为已完成</t>
         </is>
       </c>
     </row>
@@ -4771,7 +5044,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.11 完成本人已处理记录、每次操作历史摘要、总账付款留痕、分页和筛选全量导出；计划中的已处理记录已移入完成历史。</t>
+          <t>v0.12 完成组织多字段检索、折叠路径展开定位、路径导航与未保存保护；组织查找定位已从计划移入完成历史。</t>
         </is>
       </c>
     </row>
@@ -4783,7 +5056,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.11</t>
+          <t>https://jameyan42.github.io/-/?v=0.12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record date filtering stage and refresh 62-entry feature workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$63</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$67</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H16" headerRowCount="1">
-  <autoFilter ref="A5:H16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H17" headerRowCount="1">
+  <autoFilter ref="A5:H17"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L63" headerRowCount="1">
-  <autoFilter ref="A5:L63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L67" headerRowCount="1">
+  <autoFilter ref="A5:L67"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 11 个阶段、58 项内容  |  当前功能版本 v0.12  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 12 个阶段、62 项内容  |  当前功能版本 v0.13  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1050,6 +1050,42 @@
       <c r="H16" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/dab7d76</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="74" customHeight="1">
+      <c r="A17" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>v0.13</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>已处理记录日期范围与导出口径</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>58项业务测试、54项浏览器场景通过；同构生产实际审批、日期/CSV、存储不变与手机验证通过</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/95797d8</t>
         </is>
       </c>
     </row>
@@ -1071,6 +1107,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId12"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1084,7 +1121,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1096,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4557,6 +4594,238 @@
       <c r="L63" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.12.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="88" customHeight="1">
+      <c r="A64" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>v0.13</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>日期查询</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>起止日期、单边范围与常用时间段</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>按某段时间回看本人处理记录</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>审批中心 → 我已处理</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>选择今天、近7天、本月、上月或填写起止日期</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>58项业务测试、54项浏览器场景通过；同构生产实际审批、日期/CSV、存储不变与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K64" s="5" t="inlineStr">
+        <is>
+          <t>按处理时间，非报销发生日；默认不限</t>
+        </is>
+      </c>
+      <c r="L64" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.13.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="88" customHeight="1">
+      <c r="A65" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>v0.13</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>日期口径</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>本地时区双端包含与全部/匹配计数区分</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>明确边界并避免将筛选数误当全部处理数</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>日期范围说明及记录概览</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>筛选上月，比较匹配次数和本人全部次数</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>58项业务测试、54项浏览器场景通过；同构生产实际审批、日期/CSV、存储不变与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K65" s="5" t="inlineStr">
+        <is>
+          <t>浏览器本地时区；本月至今天，近7天含今天</t>
+        </is>
+      </c>
+      <c r="L65" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.13.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="88" customHeight="1">
+      <c r="A66" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>v0.13</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>异常保护</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>非法/倒置日期提示、禁导出及未计算状态</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>避免无效日期静默产生错误结果</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>日期范围控件</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>开始日期晚于结束日期，再纠正或清除</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>58项业务测试、54项浏览器场景通过；同构生产实际审批、日期/CSV、存储不变与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="inlineStr">
+        <is>
+          <t>日期仅视图状态，不写入业务记录</t>
+        </is>
+      </c>
+      <c r="L66" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.13.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="88" customHeight="1">
+      <c r="A67" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>v0.13</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>筛选导出</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>日期联合筛选、分页重置与CSV附范围时区</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>保证页面和所有匹配页导出口径一致</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>我已处理 → 导出筛选结果</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>多页记录筛选后导出全部，核对本地日期/起止/时区</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>58项业务测试、54项浏览器场景通过；同构生产实际审批、日期/CSV、存储不变与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K67" s="5" t="inlineStr">
+        <is>
+          <t>CSV保留原始ISO处理时间；无统一服务器时区</t>
+        </is>
+      </c>
+      <c r="L67" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.13.md</t>
         </is>
       </c>
     </row>
@@ -4625,6 +4894,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L61" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L62" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId62"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4638,7 +4911,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId59"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId63"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4680,7 +4953,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：已处理记录日期区间筛选 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
+          <t>建议顺序：员工报销进度总览 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
         </is>
       </c>
     </row>
@@ -4737,7 +5010,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>已处理记录日期区间筛选</t>
+          <t>员工报销进度总览</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -4747,22 +5020,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>处理历史增长后需要回看某段时间内本人操作</t>
+          <t>员工希望理解报销停在哪个节点及下一处理人</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>评估起止日期、常用时间段与现有筛选导出的联动</t>
+          <t>评估本人报销状态分组、当前节点和下一责任人提示</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>明确本地日期时区与起止包含口径，倒置范围提示，跨页导出与筛选一致</t>
+          <t>仅展示本人单据；兼容新旧流程和待付款状态，不猜测缺失处理人</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>先确定产品口径并结合实际使用反馈，不将日期筛选写为已完成</t>
+          <t>先明确可见范围与异常状态，结合实际反馈决定范围；尚未开发</t>
         </is>
       </c>
     </row>
@@ -5044,7 +5317,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.12 完成组织多字段检索、折叠路径展开定位、路径导航与未保存保护；组织查找定位已从计划移入完成历史。</t>
+          <t>v0.13 完成已处理记录日期范围、快捷区间、时区与错误提示、分页及导出联动；日期筛选已从计划移入完成历史。</t>
         </is>
       </c>
     </row>
@@ -5056,7 +5329,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.12</t>
+          <t>https://jameyan42.github.io/-/?v=0.13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record expense progress stage and refresh 66-entry feature workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$67</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$71</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H17" headerRowCount="1">
-  <autoFilter ref="A5:H17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H18" headerRowCount="1">
+  <autoFilter ref="A5:H18"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L67" headerRowCount="1">
-  <autoFilter ref="A5:L67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L71" headerRowCount="1">
+  <autoFilter ref="A5:L71"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 12 个阶段、62 项内容  |  当前功能版本 v0.13  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 13 个阶段、66 项内容  |  当前功能版本 v0.14  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1086,6 +1086,42 @@
       <c r="H17" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/95797d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="74" customHeight="1">
+      <c r="A18" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>v0.14</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>员工报销进度与退回完善闭环</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>64项业务测试、58项浏览器场景通过；生产同构实际提交/退回/重提、手机路径与只读存储验证通过</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/c46792e</t>
         </is>
       </c>
     </row>
@@ -1108,6 +1144,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId13"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1121,7 +1158,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1133,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4826,6 +4863,238 @@
       <c r="L67" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.13.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="88" customHeight="1">
+      <c r="A68" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>v0.14</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>员工进度</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>本人报销三类分组与申请金额概览</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>员工快速了解哪些单据流转中、需完善或已登记付款</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>员工 → 报销进度/工作台入口</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>切换流转中、待我完善、已登记付款，对比全部数量与匹配数</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>64项业务测试、58项浏览器场景通过；生产同构实际提交/退回/重提、手机路径与只读存储验证通过</t>
+        </is>
+      </c>
+      <c r="K68" s="5" t="inlineStr">
+        <is>
+          <t>仅本人报销；金额是申请金额，非期间支出，付款不等于银行到账</t>
+        </is>
+      </c>
+      <c r="L68" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.14.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="88" customHeight="1">
+      <c r="A69" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>v0.14</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>责任路径</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>提交快照当前节点与具名路径，兼容总账和独立付款</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>回答谁正在处理，保留提交时职责</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>报销进度 → 单据卡片</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>观察已通过/当前/后续节点，叶禾单据显示总账高璇和付款杜川</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>64项业务测试、58项浏览器场景通过；生产同构实际提交/退回/重提、手机路径与只读存储验证通过</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="inlineStr">
+        <is>
+          <t>旧单只显示原角色，不推测姓名；人员不可用提示管理员，不自动改派</t>
+        </is>
+      </c>
+      <c r="L69" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.14.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="88" customHeight="1">
+      <c r="A70" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>v0.14</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>退回完善</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>退回说明、草稿撤回完善与修改重提入口</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>让员工知道自己下一步该做什么</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>待我完善 → 查看并完善 → 详情编辑</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>主管退回写原因，员工查看并修正重提，回流转中</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>64项业务测试、58项浏览器场景通过；生产同构实际提交/退回/重提、手机路径与只读存储验证通过</t>
+        </is>
+      </c>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>重提生成新快照，历史仍在详情；无催办消息或SLA</t>
+        </is>
+      </c>
+      <c r="L70" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.14.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="88" customHeight="1">
+      <c r="A71" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>v0.14</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>查找与归属</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>进度搜索分页、切身份重置及详情本人校验</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>在记录增多时定位本人单据并避免混入他人记录</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>报销进度 → 搜索/分组/分页</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>搜索事项或待处理人，跨页后改筛选回第一页，切换员工</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>64项业务测试、58项浏览器场景通过；生产同构实际提交/退回/重提、手机路径与只读存储验证通过</t>
+        </is>
+      </c>
+      <c r="K71" s="5" t="inlineStr">
+        <is>
+          <t>每页10条；新单按ID，旧单唯一姓名且部门匹配；模拟身份非生产认证</t>
+        </is>
+      </c>
+      <c r="L71" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.14.md</t>
         </is>
       </c>
     </row>
@@ -4898,6 +5167,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId66"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4911,7 +5184,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId63"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId67"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4953,7 +5226,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：员工报销进度总览 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
+          <t>建议顺序：费用申请进度整合 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
         </is>
       </c>
     </row>
@@ -5010,7 +5283,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>员工报销进度总览</t>
+          <t>费用申请进度整合</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -5020,22 +5293,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>员工希望理解报销停在哪个节点及下一处理人</t>
+          <t>员工还需理解事前申请的预留余额、核销和结束状态</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>评估本人报销状态分组、当前节点和下一责任人提示</t>
+          <t>评估费用申请个人进度与报销关联，区分待审批、批准预留、部分核销及结束</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>仅展示本人单据；兼容新旧流程和待付款状态，不猜测缺失处理人</t>
+          <t>明确申请余额口径和关联单据状态，不将预留当支出；本人归属与新旧流程兼容</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>先明确可见范围与异常状态，结合实际反馈决定范围；尚未开发</t>
+          <t>需先明确状态和可见范围，结合实际反馈决定范围；尚未开发</t>
         </is>
       </c>
     </row>
@@ -5317,7 +5590,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.13 完成已处理记录日期范围、快捷区间、时区与错误提示、分页及导出联动；日期筛选已从计划移入完成历史。</t>
+          <t>v0.14 完成员工报销进度分组、当前责任人与快照路径、退回完善及查找分页；员工报销进度已移入完成历史。</t>
         </is>
       </c>
     </row>
@@ -5329,7 +5602,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.13</t>
+          <t>https://jameyan42.github.io/-/?v=0.14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record travel feature stage and refresh 70-entry workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$71</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$75</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H18" headerRowCount="1">
-  <autoFilter ref="A5:H18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H19" headerRowCount="1">
+  <autoFilter ref="A5:H19"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L71" headerRowCount="1">
-  <autoFilter ref="A5:L71"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L75" headerRowCount="1">
+  <autoFilter ref="A5:L75"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 13 个阶段、66 项内容  |  当前功能版本 v0.14  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 14 个阶段、70 项内容  |  当前功能版本 v0.15  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1122,6 +1122,42 @@
       <c r="H18" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/c46792e</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="74" customHeight="1">
+      <c r="A19" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>v0.15</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>差旅行程、费用明细与示例标准</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>71项业务测试、63项浏览器场景通过；生产同构申请2000/明细1500/付款/结束释放、手机及PDF验证通过</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/86e760a</t>
         </is>
       </c>
     </row>
@@ -1145,6 +1181,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId14"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1158,7 +1195,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1170,7 +1207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5095,6 +5132,238 @@
       <c r="L71" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.14.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="88" customHeight="1">
+      <c r="A72" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>v0.15</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>出差申请</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>行程、目的地日期和城市职级档的出差申请</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>将事前费用申请细化为可核对的出差场景</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>员工 → 费用申请 → 这是出差行程申请</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>杭州至上海21～23日申请2000元，主管批准后预留</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>71项业务测试、63项浏览器场景通过；生产同构申请2000/明细1500/付款/结束释放、手机及PDF验证通过</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>同一计划月份、最多31天；城市/职级档手选，旧申请不补造行程</t>
+        </is>
+      </c>
+      <c r="L72" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.15.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="88" customHeight="1">
+      <c r="A73" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>v0.15</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>差旅明细</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>五类费用行增减与分币自动合计、草稿和详情保留</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>区分交通住宿餐补，解释报销总额来源</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>新建报销 → 启用差旅费用明细</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>住宿1000/2晚、餐补300/3天、交通200，合计1500</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>71项业务测试、63项浏览器场景通过；生产同构申请2000/明细1500/付款/结束释放、手机及PDF验证通过</t>
+        </is>
+      </c>
+      <c r="K73" s="5" t="inlineStr">
+        <is>
+          <t>1～20行；整单附件，非逐票OCR；差旅草稿元数据需完整</t>
+        </is>
+      </c>
+      <c r="L73" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.15.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="88" customHeight="1">
+      <c r="A74" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>v0.15</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>差旅标准</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>固定示例标准检查、超标说明和只读制度页</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>让住宿餐补超标有明确依据和人工判断入口</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>差旅标准 / 明细预审 / 报销详情</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>住宿1100/2晚触发500元/晚预警，填理由后交审核</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>71项业务测试、63项浏览器场景通过；生产同构申请2000/明细1500/付款/结束释放、手机及PDF验证通过</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr">
+        <is>
+          <t>自定义示例制度，不代表真实公司或法定标准；有说明不豁免旧规则</t>
+        </is>
+      </c>
+      <c r="L74" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.15.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="88" customHeight="1">
+      <c r="A75" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>v0.15</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>申请报销联动</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>载入批准行程、一致性校验及备份兼容</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>使差旅行程、额度、明细和付款核销形成闭环</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>报销关联申请 / 数据管理备份</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>批准申请自动载入行程；报1500付完后结束申请释放500；坏合计备份不覆盖</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>71项业务测试、63项浏览器场景通过；生产同构申请2000/明细1500/付款/结束释放、手机及PDF验证通过</t>
+        </is>
+      </c>
+      <c r="K75" s="5" t="inlineStr">
+        <is>
+          <t>行程需与批准申请一致；预算仍按原报销日期月份，跨月和多票暂不支持</t>
+        </is>
+      </c>
+      <c r="L75" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.15.md</t>
         </is>
       </c>
     </row>
@@ -5171,6 +5440,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L73" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L74" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L75" r:id="rId70"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5184,7 +5457,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId67"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId71"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5590,7 +5863,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.14 完成员工报销进度分组、当前责任人与快照路径、退回完善及查找分页；员工报销进度已移入完成历史。</t>
+          <t>v0.15 完成出差行程申请、五类费用明细、住宿餐补示例标准与申请报销一致性/备份兼容；费用申请进度整合仍为计划。</t>
         </is>
       </c>
     </row>
@@ -5602,7 +5875,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.14</t>
+          <t>https://jameyan42.github.io/-/?v=0.15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record request progress stage and refresh 74-entry workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$75</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$79</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H19" headerRowCount="1">
-  <autoFilter ref="A5:H19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H20" headerRowCount="1">
+  <autoFilter ref="A5:H20"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L75" headerRowCount="1">
-  <autoFilter ref="A5:L75"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L79" headerRowCount="1">
+  <autoFilter ref="A5:L79"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 14 个阶段、70 项内容  |  当前功能版本 v0.15  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 15 个阶段、74 项内容  |  当前功能版本 v0.16  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1158,6 +1158,42 @@
       <c r="H19" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/86e760a</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>v0.16</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>费用申请进度、额度分解与关联报销</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>78项业务测试、68项浏览器场景通过；同构生产申请/关联/撤回/结束、CSV、只读存储与手机验证通过</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/387790e</t>
         </is>
       </c>
     </row>
@@ -1182,6 +1218,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId15"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1195,7 +1232,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1207,7 +1244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5364,6 +5401,238 @@
       <c r="L75" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.15.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="88" customHeight="1">
+      <c r="A76" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>v0.16</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>申请进度</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>本人费用申请状态及当前具体审批路径</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>让员工理解事前申请由谁处理及审批结果</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>员工 → 申请进度</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>提交1000元申请，查看赵航及当前节点，批准后转额度视图</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>78项业务测试、68项浏览器场景通过；同构生产申请/关联/撤回/结束、CSV、只读存储与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K76" s="5" t="inlineStr">
+        <is>
+          <t>旧申请仅原角色；模拟身份非生产认证，驳回不可编辑重提</t>
+        </is>
+      </c>
+      <c r="L76" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.16.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="88" customHeight="1">
+      <c r="A77" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>v0.16</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>额度追踪</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>占用在途已付未使用可关联及预留分开</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>避免把未使用额度误当可用或重复计原申请额</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>申请进度概览与卡片</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>批准1000，关联600，显示在途600/可关联400；关闭后可关联和预留归零</t>
+        </is>
+      </c>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>78项业务测试、68项浏览器场景通过；同构生产申请/关联/撤回/结束、CSV、只读存储与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K77" s="5" t="inlineStr">
+        <is>
+          <t>已付为模拟登记；关闭仍保留历史未使用额，预算沿用原口径</t>
+        </is>
+      </c>
+      <c r="L77" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.16.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="88" customHeight="1">
+      <c r="A78" s="5" t="n">
+        <v>73</v>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>v0.16</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>关联流转</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>本人关联报销展开、详情跳转和结束入口</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>从申请追踪报销进度与额度回补</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>申请卡片 → 关联报销 / 查看申请</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>撤回关联600恢复申请额度至1000；原详情限制在途时不能结束</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>78项业务测试、68项浏览器场景通过；同构生产申请/关联/撤回/结束、CSV、只读存储与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K78" s="5" t="inlineStr">
+        <is>
+          <t>不新增绕过规则的快捷结束，不发送催办，不修改审批路径</t>
+        </is>
+      </c>
+      <c r="L78" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.16.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="88" customHeight="1">
+      <c r="A79" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>v0.16</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>查询导出</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>状态月份搜索分页与全匹配CSV及存储异常保护</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>多申请时定位记录并核对所有匹配页</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>申请进度筛选和导出</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>翻到第二页后改月份回第一页，导出全部匹配；切身份清条件</t>
+        </is>
+      </c>
+      <c r="J79" s="5" t="inlineStr">
+        <is>
+          <t>78项业务测试、68项浏览器场景通过；同构生产申请/关联/撤回/结束、CSV、只读存储与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K79" s="5" t="inlineStr">
+        <is>
+          <t>每页10条，过滤不写业务数据；损坏存储关闭导出，不显示假完整结果</t>
+        </is>
+      </c>
+      <c r="L79" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.16.md</t>
         </is>
       </c>
     </row>
@@ -5444,6 +5713,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L73" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L74" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L75" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L76" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L77" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L78" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L79" r:id="rId74"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5457,7 +5730,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId71"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId75"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5499,7 +5772,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：费用申请进度整合 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
+          <t>建议顺序：多票据附件与逐票OCR评估 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
         </is>
       </c>
     </row>
@@ -5556,7 +5829,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>费用申请进度整合</t>
+          <t>多票据附件与逐票OCR评估</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -5566,22 +5839,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>员工还需理解事前申请的预留余额、核销和结束状态</t>
+          <t>当前只有整单附件和单张OCR，无法逐票核对多个费用来源</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>评估费用申请个人进度与报销关联，区分待审批、批准预留、部分核销及结束</t>
+          <t>先评估多票据清单、每票候选核对、合计去重和备份隐私，不直接承诺全部实现</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>明确申请余额口径和关联单据状态，不将预留当支出；本人归属与新旧流程兼容</t>
+          <t>明确图片保留和备份范围、取消失败回退、人工核对、明细合计与重复提示后再开发</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>需先明确状态和可见范围，结合实际反馈决定范围；尚未开发</t>
+          <t>先评审数据模型及本地存储容量，结合实际使用反馈；尚未开发</t>
         </is>
       </c>
     </row>
@@ -5863,7 +6136,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.15 完成出差行程申请、五类费用明细、住宿餐补示例标准与申请报销一致性/备份兼容；费用申请进度整合仍为计划。</t>
+          <t>v0.16 完成个人申请进度、当前审批路径、额度分解、关联报销跳转和筛选全量导出；费用申请进度整合已移入完成历史。</t>
         </is>
       </c>
     </row>
@@ -5875,7 +6148,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.15</t>
+          <t>https://jameyan42.github.io/-/?v=0.16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record attachment stage and refresh 78-entry workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$79</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$83</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H20" headerRowCount="1">
-  <autoFilter ref="A5:H20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H21" headerRowCount="1">
+  <autoFilter ref="A5:H21"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L79" headerRowCount="1">
-  <autoFilter ref="A5:L79"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L83" headerRowCount="1">
+  <autoFilter ref="A5:L83"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 15 个阶段、74 项内容  |  当前功能版本 v0.16  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 16 个阶段、78 项内容  |  当前功能版本 v0.17  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1194,6 +1194,42 @@
       <c r="H20" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/387790e</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="74" customHeight="1">
+      <c r="A21" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>v0.17</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>报销多附件、原文件留存与备份</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>85项业务测试、73项浏览器场景通过；生产同构原件上传/预览下载/备份恢复字节一致、629KB PDF和手机验证通过</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/6c4b06a</t>
         </is>
       </c>
     </row>
@@ -1219,6 +1255,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId16"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1232,7 +1269,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1244,7 +1281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5633,6 +5670,238 @@
       <c r="L79" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.16.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="88" customHeight="1">
+      <c r="A80" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>v0.17</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>报销附件</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>多选文件与酒店水单等五类材料分类、本地原件留存</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>让报销单附带可核对的证明材料</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>新建/编辑报销 → 报销附件 / 证明材料</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>添加虚构酒店水单PDF和行程图片，保存草稿刷新重开</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>85项业务测试、73项浏览器场景通过；生产同构原件上传/预览下载/备份恢复字节一致、629KB PDF和手机验证通过</t>
+        </is>
+      </c>
+      <c r="K80" s="5" t="inlineStr">
+        <is>
+          <t>PDF/PNG/JPG/WebP；5份/单、1MB/文件、1.5MB/单；原件只存本浏览器</t>
+        </is>
+      </c>
+      <c r="L80" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.17.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="88" customHeight="1">
+      <c r="A81" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>v0.17</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>材料核对</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>审核只读、图片预览及原文件下载、台账索引</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>审核人能看到材料内容并保留下载副本</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>报销详情 → 报销附件 / 发票台账</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>切主管展开图片预览，下载PDF，台账搜新附件名称</t>
+        </is>
+      </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>85项业务测试、73项浏览器场景通过；生产同构原件上传/预览下载/备份恢复字节一致、629KB PDF和手机验证通过</t>
+        </is>
+      </c>
+      <c r="K81" s="5" t="inlineStr">
+        <is>
+          <t>PDF下载后查看；证明材料不替代发票，分类手工声明，非逐票OCR或验真</t>
+        </is>
+      </c>
+      <c r="L81" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.17.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="88" customHeight="1">
+      <c r="A82" s="5" t="n">
+        <v>77</v>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>v0.17</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>附件编辑</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>草稿保留、移除确认与保存后生效、失败重试</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>避免上传或修改材料时意外丢失文件</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>编辑报销附件区</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>取消已存附件移除提醒，确认移除后保存才更新原单</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>85项业务测试、73项浏览器场景通过；生产同构原件上传/预览下载/备份恢复字节一致、629KB PDF和手机验证通过</t>
+        </is>
+      </c>
+      <c r="K82" s="5" t="inlineStr">
+        <is>
+          <t>仅可编辑状态可维护；旧OCR名称入口本身仍只存名称，不补造旧原件</t>
+        </is>
+      </c>
+      <c r="L82" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.17.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="88" customHeight="1">
+      <c r="A83" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>v0.17</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>备份与容量</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>含原件备份恢复、文件校验及存储失败回退</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>换浏览器可携带文件，错误备份或容量异常避免覆盖旧数据</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>数据管理备份 / 上传及保存错误提示</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>恢复备份后下载文件字节一致；模拟容量失败保留原状态</t>
+        </is>
+      </c>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>85项业务测试、73项浏览器场景通过；生产同构原件上传/预览下载/备份恢复字节一致、629KB PDF和手机验证通过</t>
+        </is>
+      </c>
+      <c r="K83" s="5" t="inlineStr">
+        <is>
+          <t>备份上限5MB，总存储有容量保护；失败回退不抵御崩溃/并发，非生产归档</t>
+        </is>
+      </c>
+      <c r="L83" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.17.md</t>
         </is>
       </c>
     </row>
@@ -5717,6 +5986,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L77" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L78" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L79" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L80" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L81" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L82" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L83" r:id="rId78"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5730,7 +6003,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId75"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId79"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5772,7 +6045,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：多票据附件与逐票OCR评估 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
+          <t>建议顺序：逐票OCR核对与明细绑定评估 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
         </is>
       </c>
     </row>
@@ -5829,7 +6102,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>多票据附件与逐票OCR评估</t>
+          <t>逐票OCR核对与明细绑定评估</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -5839,22 +6112,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>当前只有整单附件和单张OCR，无法逐票核对多个费用来源</t>
+          <t>多附件已可留存，但发票识别仍为原单张入口，未逐票关联明细</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>先评估多票据清单、每票候选核对、合计去重和备份隐私，不直接承诺全部实现</t>
+          <t>评估从已存发票附件发起识别、多号码冲突提示、每票人工核对及明细关联</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>明确图片保留和备份范围、取消失败回退、人工核对、明细合计与重复提示后再开发</t>
+          <t>明确票据/明细对应、金额合计和重复规则，保留失败取消回退；不让OCR自动提交报销</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>先评审数据模型及本地存储容量，结合实际使用反馈；尚未开发</t>
+          <t>多附件阶段已交付；逐票OCR尚未开发，先评审模型与实际操作反馈</t>
         </is>
       </c>
     </row>
@@ -6136,7 +6409,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.16 完成个人申请进度、当前审批路径、额度分解、关联报销跳转和筛选全量导出；费用申请进度整合已移入完成历史。</t>
+          <t>v0.17 完成多附件分类、原件本地留存、图片预览/下载、草稿编辑及含原件备份恢复；逐票OCR仍为计划。</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6421,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.16</t>
+          <t>https://jameyan42.github.io/-/?v=0.17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record payment workbench stage and refresh 82-entry workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$83</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$87</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H21" headerRowCount="1">
-  <autoFilter ref="A5:H21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H22" headerRowCount="1">
+  <autoFilter ref="A5:H22"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L83" headerRowCount="1">
-  <autoFilter ref="A5:L83"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L87" headerRowCount="1">
+  <autoFilter ref="A5:L87"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 16 个阶段、78 项内容  |  当前功能版本 v0.17  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 17 个阶段、82 项内容  |  当前功能版本 v0.18  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1230,6 +1230,42 @@
       <c r="H21" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/6c4b06a</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>v0.18</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>付款清单、批量模拟登记与参考号判重</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>91项业务测试、77项浏览器场景通过；同构生产两笔真实流程→总账→批量模拟400元/个人记录/CSV/刷新/手机验证通过</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/479b80b</t>
         </is>
       </c>
     </row>
@@ -1256,6 +1292,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId17"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1269,7 +1306,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1281,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5902,6 +5939,238 @@
       <c r="L83" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.17.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="88" customHeight="1">
+      <c r="A84" s="5" t="n">
+        <v>79</v>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>v0.18</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>批量付款登记</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>20笔内勾选、逐笔参考号预览和确认后整批模拟登记</t>
+        </is>
+      </c>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>让付款人员集中核对多笔待付款单据，保留每笔留痕</t>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>付款工作台 → 勾选 → 批量模拟登记</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>两笔各200元，核对总额400及两个独立参考号，确认后回看个人已处理</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>91项业务测试、77项浏览器场景通过；同构生产两笔真实流程→总账→批量模拟400元/个人记录/CSV/刷新/手机验证通过</t>
+        </is>
+      </c>
+      <c r="K84" s="5" t="inlineStr">
+        <is>
+          <t>仅模拟，不连接银行；3～48位前缀，每笔独立参考号，非真实银行批次</t>
+        </is>
+      </c>
+      <c r="L84" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.18.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="88" customHeight="1">
+      <c r="A85" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>v0.18</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>重复检查</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>新单笔及批量参考号跨已付款记录判重</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>避免重复登记已用参考号，失败不部分修改单据</t>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>单笔付款详情 / 批量核对提交</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>复用已付款参考号，忽略大小写和首尾空格仍被拦</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>91项业务测试、77项浏览器场景通过；同构生产两笔真实流程→总账→批量模拟400元/个人记录/CSV/刷新/手机验证通过</t>
+        </is>
+      </c>
+      <c r="K85" s="5" t="inlineStr">
+        <is>
+          <t>仅当前浏览器新登记生效，旧重复不改；不支持一个银行交易匹配多报销</t>
+        </is>
+      </c>
+      <c r="L85" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.18.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="88" customHeight="1">
+      <c r="A86" s="5" t="n">
+        <v>81</v>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>v0.18</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>付款清单</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>当前筛选CSV含责任人、总账和付款信息</t>
+        </is>
+      </c>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>核对待付或已付清单，保留查询范围与金额来源</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>付款工作台 → 导出筛选付款清单</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>按部门关键词或状态筛选后导出，核对杜川/总账科目/参考号</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>91项业务测试、77项浏览器场景通过；同构生产两笔真实流程→总账→批量模拟400元/个人记录/CSV/刷新/手机验证通过</t>
+        </is>
+      </c>
+      <c r="K86" s="5" t="inlineStr">
+        <is>
+          <t>导出所有匹配记录，不限勾选；不是实际银行付款文件</t>
+        </is>
+      </c>
+      <c r="L86" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.18.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="88" customHeight="1">
+      <c r="A87" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>v0.18</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>保存与权限</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>付款状态总账风险重校验和容量失败保留重试</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>避免无权限、未复核或存储失败造成部分登记</t>
+        </is>
+      </c>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>批量提交 / 单笔付款提交</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>管理员不可勾选，总账未完不入待付；模拟容量不足保留表单和原数据</t>
+        </is>
+      </c>
+      <c r="J87" s="5" t="inlineStr">
+        <is>
+          <t>91项业务测试、77项浏览器场景通过；同构生产两笔真实流程→总账→批量模拟400元/个人记录/CSV/刷新/手机验证通过</t>
+        </is>
+      </c>
+      <c r="K87" s="5" t="inlineStr">
+        <is>
+          <t>原型单键保存，无后端事务或并发幂等；旧财务付款兼容</t>
+        </is>
+      </c>
+      <c r="L87" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.18.md</t>
         </is>
       </c>
     </row>
@@ -5990,6 +6259,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L81" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L82" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L83" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L84" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L85" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L86" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L87" r:id="rId82"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6003,7 +6276,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId79"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId83"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6409,7 +6682,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.17 完成多附件分类、原件本地留存、图片预览/下载、草稿编辑及含原件备份恢复；逐票OCR仍为计划。</t>
+          <t>v0.18 完成付款清单导出、批量核对与模拟登记、独立参考号和重复检查及失败保护；逐票OCR仍为计划。</t>
         </is>
       </c>
     </row>
@@ -6421,7 +6694,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.17</t>
+          <t>https://jameyan42.github.io/-/?v=0.18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record message center stage and refresh 86-entry workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$23</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$87</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$91</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H22" headerRowCount="1">
-  <autoFilter ref="A5:H22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H23" headerRowCount="1">
+  <autoFilter ref="A5:H23"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L87" headerRowCount="1">
-  <autoFilter ref="A5:L87"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L91" headerRowCount="1">
+  <autoFilter ref="A5:L91"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 17 个阶段、82 项内容  |  当前功能版本 v0.18  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 18 个阶段、86 项内容  |  当前功能版本 v0.19  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1266,6 +1266,42 @@
       <c r="H22" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/479b80b</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="74" customHeight="1">
+      <c r="A23" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>v0.19</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>站内消息、人员已读与业务跳转</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>98项业务测试、82项浏览器场景通过；同构生产提交/消息退回重提/新未读/付款结果/已读备份恢复、导航滚动与手机验证通过</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/fb69f1f</t>
         </is>
       </c>
     </row>
@@ -1293,6 +1329,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId18"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1306,7 +1343,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1318,7 +1355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6171,6 +6208,238 @@
       <c r="L87" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.18.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="88" customHeight="1">
+      <c r="A88" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>v0.19</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>站内消息</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>当前人员待办与本人退回付款申请结果提示</t>
+        </is>
+      </c>
+      <c r="F88" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>集中查看当前需要处理及本人单据进展</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>消息中心 / 导航未读角标</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>主管查看具名待办，从消息退回；员工看到原因与模拟付款结果</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>98项业务测试、82项浏览器场景通过；同构生产提交/消息退回重提/新未读/付款结果/已读备份恢复、导航滚动与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K88" s="5" t="inlineStr">
+        <is>
+          <t>每单当前一条提示，旧记录初次出现不代表刚送达；无外部或桌面推送</t>
+        </is>
+      </c>
+      <c r="L88" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.19.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="88" customHeight="1">
+      <c r="A89" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>v0.19</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>阅读状态</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>人员隔离已读、稳定事件键和新节点新未读</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>读过的任务不冒充已审批，后续流转仍可提示</t>
+        </is>
+      </c>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>消息中心标记已读 / 查看单据</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>读消息不改业务；退回重提后同一单据产生新未读，刷新仍保留已读</t>
+        </is>
+      </c>
+      <c r="J89" s="5" t="inlineStr">
+        <is>
+          <t>98项业务测试、82项浏览器场景通过；同构生产提交/消息退回重提/新未读/付款结果/已读备份恢复、导航滚动与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K89" s="5" t="inlineStr">
+        <is>
+          <t>已读按本浏览器人员ID，非生产身份权限；每人1000条及总容量保护</t>
+        </is>
+      </c>
+      <c r="L89" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.19.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="88" customHeight="1">
+      <c r="A90" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>v0.19</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>查找与处理</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>类别未读关键词分页、跨页批读与单据跳转</t>
+        </is>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>快速找到任务，直接进入原审批或编辑入口</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>消息筛选 / 将筛选结果标读 / 查看单据</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>25条跨页全部标读，跳转原详情处理；桌面长菜单可滚动且切页保留位置</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>98项业务测试、82项浏览器场景通过；同构生产提交/消息退回重提/新未读/付款结果/已读备份恢复、导航滚动与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K90" s="5" t="inlineStr">
+        <is>
+          <t>每页20条；只改阅读状态，业务规则仍走原入口，不自动催办</t>
+        </is>
+      </c>
+      <c r="L90" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.19.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="88" customHeight="1">
+      <c r="A91" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>v0.19</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>备份与异常</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>新旧已读备份兼容、损坏及配额失败不覆盖</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>换浏览器可携带已读，异常明确显示未知或部分结果</t>
+        </is>
+      </c>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>数据管理备份 / 消息异常提示</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>新备份恢复已读，旧备份保留已有标记；存储坏值保留且仍可查看业务</t>
+        </is>
+      </c>
+      <c r="J91" s="5" t="inlineStr">
+        <is>
+          <t>98项业务测试、82项浏览器场景通过；同构生产提交/消息退回重提/新未读/付款结果/已读备份恢复、导航滚动与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K91" s="5" t="inlineStr">
+        <is>
+          <t>无服务端消息投递、跨设备实时同步或崩溃事务保证，未知业务时间不猜</t>
+        </is>
+      </c>
+      <c r="L91" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.19.md</t>
         </is>
       </c>
     </row>
@@ -6263,6 +6532,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L85" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L86" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L87" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L88" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L89" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L90" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L91" r:id="rId86"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6276,7 +6549,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId83"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId87"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6682,7 +6955,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.18 完成付款清单导出、批量核对与模拟登记、独立参考号和重复检查及失败保护；逐票OCR仍为计划。</t>
+          <t>v0.19 完成站内状态提示、人员已读、新节点未读、筛选跳转/批读和已读备份异常保护；逐票OCR及开发完成系统弹窗未完成。</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6967,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.18</t>
+          <t>https://jameyan42.github.io/-/?v=0.19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record v0.20 enterprise workflows in iteration workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,11 +14,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$91</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$97</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$8</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'使用与维护'!$A$5:$B$17</definedName>
   </definedNames>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H23" headerRowCount="1">
-  <autoFilter ref="A5:H23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H24" headerRowCount="1">
+  <autoFilter ref="A5:H24"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L91" headerRowCount="1">
-  <autoFilter ref="A5:L91"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L97" headerRowCount="1">
+  <autoFilter ref="A5:L97"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -264,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H8" headerRowCount="1">
-  <autoFilter ref="A5:H8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H12" headerRowCount="1">
+  <autoFilter ref="A5:H12"/>
   <tableColumns count="8">
     <tableColumn id="1" name="顺序"/>
     <tableColumn id="2" name="优先级"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 18 个阶段、86 项内容  |  当前功能版本 v0.19  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-23  |  已交付 19 个阶段、92 项内容  |  当前功能版本 v0.20  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1302,6 +1302,42 @@
       <c r="H23" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/fb69f1f</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="74" customHeight="1">
+      <c r="A24" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>v0.20</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>供应商、合同初筛与对公支付全链路</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>110项业务测试、89项浏览器场景全部通过；同构生产新建供应商/10000元合同人工复核/4000元对公完整审批及模拟付款/剩余6000元、备份恢复与手机验证通过</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/43d925d</t>
         </is>
       </c>
     </row>
@@ -1330,6 +1366,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId19"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1343,7 +1380,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1355,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6440,6 +6477,354 @@
       <c r="L91" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.19.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="88" customHeight="1">
+      <c r="A92" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>v0.20</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>供应商档案</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>同名虚构收款账户、唯一标识与启停</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>区分供应商收款与员工报销收款，维护后续付款基础档案</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>供应商管理（管理员）</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>新增虚构供应商与DEMO账号；改账户后核对旧对公单快照未变</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>110项业务测试、89项浏览器场景全部通过；同构生产新建供应商/10000元合同人工复核/4000元对公完整审批及模拟付款/剩余6000元、备份恢复与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K92" s="5" t="inlineStr">
+        <is>
+          <t>不连接银行、工商或供应商外部数据库；停用仅阻止新提交，无删除</t>
+        </is>
+      </c>
+      <c r="L92" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.20.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="88" customHeight="1">
+      <c r="A93" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>v0.20</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>合同规则初筛</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>正文/TXT导入、原文风险片段与缺失条款提示</t>
+        </is>
+      </c>
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>把付款依据的疑点交给人工核对，并保留透明规则</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>合同审查 → 员工提交 / 预览规则初筛</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>载入虚构正文；用全额预付、无限责任及单方解除片段查看提示</t>
+        </is>
+      </c>
+      <c r="J93" s="5" t="inlineStr">
+        <is>
+          <t>110项业务测试、89项浏览器场景全部通过；同构生产新建供应商/10000元合同人工复核/4000元对公完整审批及模拟付款/剩余6000元、备份恢复与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K93" s="5" t="inlineStr">
+        <is>
+          <t>本地关键词规则，非AI或法律意见；PDF/DOCX不提取，真实模型未接</t>
+        </is>
+      </c>
+      <c r="L93" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.20.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="88" customHeight="1">
+      <c r="A94" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>v0.20</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>合同人工复核</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>人工确认与意见、要求修改及版本修订</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>避免规则提示自动代替审批，固定付款依据版本</t>
+        </is>
+      </c>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>合同审查 → 财务/管理员查看合同</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>阅读全文填复核意见并确认；要求修改后员工修订重新初筛</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr">
+        <is>
+          <t>110项业务测试、89项浏览器场景全部通过；同构生产新建供应商/10000元合同人工复核/4000元对公完整审批及模拟付款/剩余6000元、备份恢复与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K94" s="5" t="inlineStr">
+        <is>
+          <t>已复核合同不可直接修订，需另建；无电子签章/补充协议/法律准确率数据</t>
+        </is>
+      </c>
+      <c r="L94" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.20.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="88" customHeight="1">
+      <c r="A95" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>v0.20</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>对公支付链路</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>独立对公单与具名业务、财务、总账、付款办理</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>完成供应商合同付款的企业费用主链路</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>对公支付单；先在审批流程发布财务分工</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>林晓按本人已复核合同提交；许明、周宁、高璇、杜川按指定节点办理</t>
+        </is>
+      </c>
+      <c r="J95" s="5" t="inlineStr">
+        <is>
+          <t>110项业务测试、89项浏览器场景全部通过；同构生产新建供应商/10000元合同人工复核/4000元对公完整审批及模拟付款/剩余6000元、备份恢复与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K95" s="5" t="inlineStr">
+        <is>
+          <t>复用已发布报销分支，数据和历史独立；未并入原消息/审批/报销付款台，无履约附件或真实转账</t>
+        </is>
+      </c>
+      <c r="L95" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.20.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="88" customHeight="1">
+      <c r="A96" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>v0.20</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>合同额度与快照</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>分币累计占用、退回释放、账户路径冻结及参考号跨业务判重</t>
+        </is>
+      </c>
+      <c r="F96" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>防止单浏览器顺序超额提交及主数据改动影响在途</t>
+        </is>
+      </c>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>合同详情额度 / 对公收款及路径快照 / 报销与对公付款</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>10000元合同支付4000元后可用6000元；超额拦截，退回重提重算；重复参考号拦截</t>
+        </is>
+      </c>
+      <c r="J96" s="5" t="inlineStr">
+        <is>
+          <t>110项业务测试、89项浏览器场景全部通过；同构生产新建供应商/10000元合同人工复核/4000元对公完整审批及模拟付款/剩余6000元、备份恢复与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K96" s="5" t="inlineStr">
+        <is>
+          <t>合同额度不进入原部门报销预算；无并发事务或银行幂等，多币种/多法人未实现</t>
+        </is>
+      </c>
+      <c r="L96" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.20.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="88" customHeight="1">
+      <c r="A97" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>v0.20</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>46318</v>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>企业数据与交付</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>企业业务备份兼容、容量损坏保护与筛选分页CSV</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>迁移完整演示记录，异常不把空数据当成成功保存</t>
+        </is>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>企业业务列表 / 数据管理 / 演示指南08</t>
+        </is>
+      </c>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>新备份恢复企业业务、旧备份保留；模拟写入失败保留原值与表单；筛选导出全部页</t>
+        </is>
+      </c>
+      <c r="J97" s="5" t="inlineStr">
+        <is>
+          <t>110项业务测试、89项浏览器场景全部通过；同构生产新建供应商/10000元合同人工复核/4000元对公完整审批及模拟付款/剩余6000元、备份恢复与手机验证通过</t>
+        </is>
+      </c>
+      <c r="K97" s="5" t="inlineStr">
+        <is>
+          <t>各类200条/整体80万字符，本地存储非生产鉴权；有企业业务时保护旧重置，未做真实用户验证</t>
+        </is>
+      </c>
+      <c r="L97" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.20.md</t>
         </is>
       </c>
     </row>
@@ -6536,6 +6921,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L89" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L90" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L91" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L92" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L93" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L94" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L95" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L97" r:id="rId92"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6549,7 +6940,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId87"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId93"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6561,7 +6952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6591,7 +6982,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：逐票OCR核对与明细绑定评估 → 真实可用性反馈；复杂审批能力等待需求验证。</t>
+          <t>建议顺序：对公履约附件与统一待办 → 预算模型评估；真实AI按用户选择暂缓，先做本地规则。</t>
         </is>
       </c>
     </row>
@@ -6648,7 +7039,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>逐票OCR核对与明细绑定评估</t>
+          <t>对公履约附件与付款依据</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -6658,22 +7049,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>多附件已可留存，但发票识别仍为原单张入口，未逐票关联明细</t>
+          <t>对公单已有合同依据，但还不能留存验收单/发票等原文件</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>评估从已存发票附件发起识别、多号码冲突提示、每票人工核对及明细关联</t>
+          <t>复用附件校验与存储边界，区分验收、发票和付款凭证，保护已有合同及对公记录</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>明确票据/明细对应、金额合计和重复规则，保留失败取消回退；不让OCR自动提交报销</t>
+          <t>指定人员可查看原文件，备份可恢复，容量失败不覆盖；不把上传视作验真</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>多附件阶段已交付；逐票OCR尚未开发，先评审模型与实际操作反馈</t>
+          <t>先评估企业数据容量与文件存储方式，不接真实财务资料</t>
         </is>
       </c>
     </row>
@@ -6688,32 +7079,32 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>真实可用性测试</t>
+          <t>对公统一待办及消息</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>待用户参与</t>
+          <t>待排期</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>自动化测试不能证明真实用户理解和使用顺畅</t>
+          <t>当前对公需到独立页面，原审批中心/消息仅汇集员工费用</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>结合图形组织、部门总/财务/总账/付款路径，使用已准备任务收集真实参与者操作反馈</t>
+          <t>明确定义corporate单据类型和个人处理历史，复用跳转而不伪装报销</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>记录真实任务完成情况、困惑点与改进建议；无参与者前不写研究结论</t>
+          <t>不同类型与人员范围准确，处理结果独立，已读不改业务，新事件提示一致</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>需要用户协助招募实际参与者；AI 不能代替真实访谈</t>
+          <t>对公闭环已完成；需定义消息与历史兼容模型</t>
         </is>
       </c>
     </row>
@@ -6728,30 +7119,190 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
+          <t>多法人及部门预算评估</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>待排期</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>当前只有单企业CNY及合同额度，未统一对公预算</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>先明确法人、预算维度、申请预留/合同/对公避免重复占用的口径</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>有可审查的业务模型及虚构场景后再开发，不提前宣称企业规模能力</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>需要需求验证；当前不接真实会计系统</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="100" customHeight="1">
+      <c r="A9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>真实AI合同审查接入</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>待排期</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>本地规则不能理解复杂法律语义，当前无模型服务端适配器</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>后端保管密钥、模型选择、费用/合同范围授权、结构化风险及原文证据核验、人工兜底</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>先完成可审查接口及模拟测试，必要授权后才真实调用；不把模型输出当法律结论</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>用户已选择先本地规则，真实AI稍后；真实服务需新账号权限及费用/数据范围确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>逐票OCR核对与明细绑定评估</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>建议下一阶段</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>多附件已可留存，但发票识别仍为原单张入口，未逐票关联明细</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>评估从已存发票附件发起识别、多号码冲突提示、每票人工核对及明细关联</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>明确票据/明细对应、金额合计和重复规则，保留失败取消回退；不让OCR自动提交报销</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>多附件阶段已交付；逐票OCR尚未开发，先评审模型与实际操作反馈</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="100" customHeight="1">
+      <c r="A11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>真实可用性测试</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>待用户参与</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>自动化测试不能证明真实用户理解和使用顺畅</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>结合图形组织、部门总/财务/总账/付款路径，使用已准备任务收集真实参与者操作反馈</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>记录真实任务完成情况、困惑点与改进建议；无参与者前不写研究结论</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>需要用户协助招募实际参与者；AI 不能代替真实访谈</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="100" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
           <t>复杂审批能力评估</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>暂缓</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>尚无证据证明会签、或签、加签和嵌套条件为当前作品优先需求</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>先依据组织与审批树试用反馈，再决定是否扩展</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>明确业务场景、异常策略与范围后再排开发</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>不在当前 Excel 中记为已完成</t>
         </is>
@@ -6955,7 +7506,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.19 完成站内状态提示、人员已读、新节点未读、筛选跳转/批读和已读备份异常保护；逐票OCR及开发完成系统弹窗未完成。</t>
+          <t>v0.20 完成供应商、合同规则初筛/人工复核、独立对公支付、合同额度/快照及备份保护；真实AI、对公附件和统一消息待后续。</t>
         </is>
       </c>
     </row>
@@ -6967,7 +7518,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.19</t>
+          <t>https://jameyan42.github.io/-/?v=0.20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record v0.21 rule prechecks in iteration workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,11 +14,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$97</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$102</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'使用与维护'!$A$5:$B$17</definedName>
   </definedNames>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H24" headerRowCount="1">
-  <autoFilter ref="A5:H24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H25" headerRowCount="1">
+  <autoFilter ref="A5:H25"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L97" headerRowCount="1">
-  <autoFilter ref="A5:L97"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L102" headerRowCount="1">
+  <autoFilter ref="A5:L102"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -264,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H12" headerRowCount="1">
-  <autoFilter ref="A5:H12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H13" headerRowCount="1">
+  <autoFilter ref="A5:H13"/>
   <tableColumns count="8">
     <tableColumn id="1" name="顺序"/>
     <tableColumn id="2" name="优先级"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -604,14 +604,14 @@
     <row r="2" ht="38" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>依据 Git 提交与阶段验收回溯；日期为功能源码提交日，不是每项功能的独立完成时间。</t>
+          <t>依据 Git 提交与阶段验收回溯；日期沿用阶段验收口径，v0.21起按上海日期记录；不是每项功能的独立完成时间。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-23  |  已交付 19 个阶段、92 项内容  |  当前功能版本 v0.20  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 20 个阶段、97 项内容  |  当前功能版本 v0.21  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1338,6 +1338,42 @@
       <c r="H24" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/43d925d</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="74" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>v0.21</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>报销与对公可配置规则预审及风险依据</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>120项业务测试、94项浏览器场景全部通过；同构生产报销原文件拦截/提醒付款、对公2000阈值拦截/提醒处理/9000当前与v3旧快照、配置及两类快照备份恢复/390px通过</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/5b678a0</t>
         </is>
       </c>
     </row>
@@ -1367,6 +1403,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId20"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1380,7 +1417,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1392,7 +1429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6825,6 +6862,296 @@
       <c r="L97" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.20.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="88" customHeight="1">
+      <c r="A98" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>v0.21</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>审核风险提示</t>
+        </is>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>报销与对公结构化风险、触发依据及核对建议</t>
+        </is>
+      </c>
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>把字段及关联记录转为审核人可核查的风险线索</t>
+        </is>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>报销管理/对公支付单列表与详情</t>
+        </is>
+      </c>
+      <c r="I98" s="5" t="inlineStr">
+        <is>
+          <t>查看原文件、疑似重复、大额或账户变更提示，核对对应字段与关联单号</t>
+        </is>
+      </c>
+      <c r="J98" s="5" t="inlineStr">
+        <is>
+          <t>120项业务测试、94项浏览器场景全部通过；同构生产报销原文件拦截/提醒付款、对公2000阈值拦截/提醒处理/9000当前与v3旧快照、配置及两类快照备份恢复/390px通过</t>
+        </is>
+      </c>
+      <c r="K98" s="5" t="inlineStr">
+        <is>
+          <t>规则匹配不代表业务违规或发票验真；无AI或外部上传</t>
+        </is>
+      </c>
+      <c r="L98" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.21.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="88" customHeight="1">
+      <c r="A99" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>v0.21</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>预审规则配置</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>10条补充规则启停、提醒/拦截、阈值和版本</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>将提醒和必须修正的情形分开，保留财务配置空间</t>
+        </is>
+      </c>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>财务 → 规则配置 → 报销/对公补充规则</t>
+        </is>
+      </c>
+      <c r="I99" s="5" t="inlineStr">
+        <is>
+          <t>设置原文件检查、时效、大额和占用比例，填写原因保存后观察当前提示</t>
+        </is>
+      </c>
+      <c r="J99" s="5" t="inlineStr">
+        <is>
+          <t>120项业务测试、94项浏览器场景全部通过；同构生产报销原文件拦截/提醒付款、对公2000阈值拦截/提醒处理/9000当前与v3旧快照、配置及两类快照备份恢复/390px通过</t>
+        </is>
+      </c>
+      <c r="K99" s="5" t="inlineStr">
+        <is>
+          <t>固定规则目录，无任意脚本或条件组；新增默认提醒，原报销制度及对公固定校验保留</t>
+        </is>
+      </c>
+      <c r="L99" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.21.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="88" customHeight="1">
+      <c r="A100" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>v0.21</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>审批与付款校验</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>处理前重算、财务总账付款拦截与批量整批校验</t>
+        </is>
+      </c>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>防止页面展示提示却在后续处理入口放行</t>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>报销单笔/批量付款；对公指定节点办理</t>
+        </is>
+      </c>
+      <c r="I100" s="5" t="inlineStr">
+        <is>
+          <t>原文件设拦截不能付款；对公4000元命中2000元阈值，退回或调整可配规则后人工处理</t>
+        </is>
+      </c>
+      <c r="J100" s="5" t="inlineStr">
+        <is>
+          <t>120项业务测试、94项浏览器场景全部通过；同构生产报销原文件拦截/提醒付款、对公2000阈值拦截/提醒处理/9000当前与v3旧快照、配置及两类快照备份恢复/390px通过</t>
+        </is>
+      </c>
+      <c r="K100" s="5" t="inlineStr">
+        <is>
+          <t>主管仍可转交财务，提醒不阻止继续；无银行转账或服务端并发保证</t>
+        </is>
+      </c>
+      <c r="L100" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.21.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="88" customHeight="1">
+      <c r="A101" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>v0.21</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>处理依据追溯</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>每次处理保留规则参数和风险快照，与当前检查分开</t>
+        </is>
+      </c>
+      <c r="F101" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>避免用现在的规则推断过去审批依据</t>
+        </is>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>报销/对公详情 → 处理时预审快照</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>2000元阈值下处理，改9000元后比较当前结果与旧版本参数</t>
+        </is>
+      </c>
+      <c r="J101" s="5" t="inlineStr">
+        <is>
+          <t>120项业务测试、94项浏览器场景全部通过；同构生产报销原文件拦截/提醒付款、对公2000阈值拦截/提醒处理/9000当前与v3旧快照、配置及两类快照备份恢复/390px通过</t>
+        </is>
+      </c>
+      <c r="K101" s="5" t="inlineStr">
+        <is>
+          <t>保存系统计算结果不等于审核人逐项确认；不补造旧历史，日志非不可篡改</t>
+        </is>
+      </c>
+      <c r="L101" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.21.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="88" customHeight="1">
+      <c r="A102" s="5" t="n">
+        <v>97</v>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>v0.21</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>规则存储与兼容</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>配置及结果备份、写入失败不替换与坏规则暂停通过</t>
+        </is>
+      </c>
+      <c r="F102" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>迁移演示现场，异常时不默认放行</t>
+        </is>
+      </c>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>规则配置 / 数据管理 / 单据详情异常提示</t>
+        </is>
+      </c>
+      <c r="I102" s="5" t="inlineStr">
+        <is>
+          <t>新备份恢复配置和两类快照；模拟配额失败保留表单；坏规则仍可退回但不能通过或完整备份</t>
+        </is>
+      </c>
+      <c r="J102" s="5" t="inlineStr">
+        <is>
+          <t>120项业务测试、94项浏览器场景全部通过；同构生产报销原文件拦截/提醒付款、对公2000阈值拦截/提醒处理/9000当前与v3旧快照、配置及两类快照备份恢复/390px通过</t>
+        </is>
+      </c>
+      <c r="K102" s="5" t="inlineStr">
+        <is>
+          <t>旧政策使用内置补充提醒，旧记录无快照仍可恢复；无真实审核准确率或业务收益证明</t>
+        </is>
+      </c>
+      <c r="L102" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.21.md</t>
         </is>
       </c>
     </row>
@@ -6927,6 +7254,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L95" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L97" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L98" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L99" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L100" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L101" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L102" r:id="rId97"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6940,7 +7272,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId93"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId98"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6952,7 +7284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6982,7 +7314,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：对公履约附件与统一待办 → 预算模型评估；真实AI按用户选择暂缓，先做本地规则。</t>
+          <t>建议顺序：对公履约附件与统一待办 → 预算模型评估；规则预审已交付，后续按使用反馈扩展；真实AI按用户选择暂缓。</t>
         </is>
       </c>
     </row>
@@ -7305,6 +7637,46 @@
       <c r="H12" s="5" t="inlineStr">
         <is>
           <t>不在当前 Excel 中记为已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="100" customHeight="1">
+      <c r="A13" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>规则适用范围与疑点核对闭环</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>待排期</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>当前为统一固定规则目录，无组织适用范围或逐项核对状态</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>先验证提醒/拦截理解，再评估按部门类型配置及疑点逐项处置</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>明确规则冲突、审批节点及历史迁移口径后开发；不把已保存预审快照当作逐项核实</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>当前规则预审已交付；需真实任务反馈决定范围</t>
         </is>
       </c>
     </row>
@@ -7362,7 +7734,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>记录口径更新于 2026-10-23</t>
+          <t>记录口径更新于 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -7410,7 +7782,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>按 Git 功能提交顺序分阶段；同阶段按功能/演示逻辑编号。2026-10-22/23 为源码提交日，不将其当作独立功能时间或上线时间。</t>
+          <t>按 Git 功能提交顺序分阶段；同阶段按功能/演示逻辑编号。早期日期沿用源码提交记录，v0.21起按上海日期记录；不将阶段日期当作每项独立完成或上线时间。</t>
         </is>
       </c>
     </row>
@@ -7506,7 +7878,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.20 完成供应商、合同规则初筛/人工复核、独立对公支付、合同额度/快照及备份保护；真实AI、对公附件和统一消息待后续。</t>
+          <t>v0.21 完成报销/对公10条补充规则、风险依据、提醒/拦截、处理时快照及配置异常保护；真实AI暂停，对公附件与统一待办待后续。</t>
         </is>
       </c>
     </row>
@@ -7518,7 +7890,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.20</t>
+          <t>https://jameyan42.github.io/-/?v=0.21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record v0.22 structured invoice delivery in workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$26</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$102</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$107</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H25" headerRowCount="1">
-  <autoFilter ref="A5:H25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H26" headerRowCount="1">
+  <autoFilter ref="A5:H26"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L102" headerRowCount="1">
-  <autoFilter ref="A5:L102"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L107" headerRowCount="1">
+  <autoFilter ref="A5:L107"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 20 个阶段、97 项内容  |  当前功能版本 v0.21  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 21 个阶段、102 项内容  |  当前功能版本 v0.22  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1374,6 +1374,42 @@
       <c r="H25" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/5b678a0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="74" customHeight="1">
+      <c r="A26" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>v0.22</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>票面结构化与抬头金额核对</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>131项业务测试通过、100项浏览器场景整套通过，导出修正后相关6项重跑通过；生产同构真实OCR抬头/日期/265元、200申请不覆盖、对公跨单线索、CSV/JSON/备份恢复及手机通过</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/defe80a</t>
         </is>
       </c>
     </row>
@@ -1404,6 +1440,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId21"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1417,7 +1454,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1429,7 +1466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7152,6 +7189,296 @@
       <c r="L102" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.21.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="88" customHeight="1">
+      <c r="A103" s="5" t="n">
+        <v>98</v>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>v0.22</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>票面OCR提取</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>明确标签购销方税号、日期代码及金额税额候选</t>
+        </is>
+      </c>
+      <c r="F103" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>从单一号码金额扩展为可核对的票面字段</t>
+        </is>
+      </c>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>报销快速OCR / 报销与对公结构化采集</t>
+        </is>
+      </c>
+      <c r="I103" s="5" t="inlineStr">
+        <is>
+          <t>载入新虚构样票，实际本地OCR识别星河科技、2026-10-24与265.00元</t>
+        </is>
+      </c>
+      <c r="J103" s="5" t="inlineStr">
+        <is>
+          <t>131项业务测试通过、100项浏览器场景整套通过，导出修正后相关6项重跑通过；生产同构真实OCR抬头/日期/265元、200申请不覆盖、对公跨单线索、CSV/JSON/备份恢复及手机通过</t>
+        </is>
+      </c>
+      <c r="K103" s="5" t="inlineStr">
+        <is>
+          <t>真实引擎但无通用准确率；冲突留空，仅人民币正数图片，PDF/红票/外币/二维码暂不支持</t>
+        </is>
+      </c>
+      <c r="L103" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.22.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="88" customHeight="1">
+      <c r="A104" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>v0.22</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>多票结构化采集</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>每单5张、人工确认修订、字段卡片及申请金额独立</t>
+        </is>
+      </c>
+      <c r="F104" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>把候选转成系统可保存展示的数据，不把多票金额自动覆盖申请</t>
+        </is>
+      </c>
+      <c r="H104" s="5" t="inlineStr">
+        <is>
+          <t>新建/编辑报销及对公 → 结构化发票采集；单据详情</t>
+        </is>
+      </c>
+      <c r="I104" s="5" t="inlineStr">
+        <is>
+          <t>265票面申请200元，确认后卡片保留265、原申请仍200；未加入候选阻止保存</t>
+        </is>
+      </c>
+      <c r="J104" s="5" t="inlineStr">
+        <is>
+          <t>131项业务测试通过、100项浏览器场景整套通过，导出修正后相关6项重跑通过；生产同构真实OCR抬头/日期/265元、200申请不覆盖、对公跨单线索、CSV/JSON/备份恢复及手机通过</t>
+        </is>
+      </c>
+      <c r="K104" s="5" t="inlineStr">
+        <is>
+          <t>采集区仅留字段和来源名，不关联原图；原快速单票填入仍可替换金额，对公原附件未实现</t>
+        </is>
+      </c>
+      <c r="L104" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.22.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="88" customHeight="1">
+      <c r="A105" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>v0.22</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>财务基准与票面预审</t>
+        </is>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>统一抬头税号及购买方/合计/重复/税额四条规则</t>
+        </is>
+      </c>
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>让审核人看到一致性差异及原字段依据，员工不能改本单核对基准</t>
+        </is>
+      </c>
+      <c r="H105" s="5" t="inlineStr">
+        <is>
+          <t>财务规则配置 / 单据当前预审及处理快照</t>
+        </is>
+      </c>
+      <c r="I105" s="5" t="inlineStr">
+        <is>
+          <t>错误抬头设拦截，265与200差异提醒，同票号跨报销对公均有线索</t>
+        </is>
+      </c>
+      <c r="J105" s="5" t="inlineStr">
+        <is>
+          <t>131项业务测试通过、100项浏览器场景整套通过，导出修正后相关6项重跑通过；生产同构真实OCR抬头/日期/265元、200申请不覆盖、对公跨单线索、CSV/JSON/备份恢复及手机通过</t>
+        </is>
+      </c>
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t>不是官方真伪或税号工商核验；不做简称模糊匹配，空税号不声称一致，部分报销可合理</t>
+        </is>
+      </c>
+      <c r="L105" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.22.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="88" customHeight="1">
+      <c r="A106" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>v0.22</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>票面数据展示导出</t>
+        </is>
+      </c>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>逐张结构化台账、JSON及CSV、长号码文本保护</t>
+        </is>
+      </c>
+      <c r="F106" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>票面金额与申请金额分列，导出可保留20位票号</t>
+        </is>
+      </c>
+      <c r="H106" s="5" t="inlineStr">
+        <is>
+          <t>发票台账下方票面台账 / 详情JSON下载</t>
+        </is>
+      </c>
+      <c r="I106" s="5" t="inlineStr">
+        <is>
+          <t>跨报销对公查看每张票，点击原单；CSV数字号码前置文本标记，JSON保留原字段</t>
+        </is>
+      </c>
+      <c r="J106" s="5" t="inlineStr">
+        <is>
+          <t>131项业务测试通过、100项浏览器场景整套通过，导出修正后相关6项重跑通过；生产同构真实OCR抬头/日期/265元、200申请不覆盖、对公跨单线索、CSV/JSON/备份恢复及手机通过</t>
+        </is>
+      </c>
+      <c r="K106" s="5" t="inlineStr">
+        <is>
+          <t>按本浏览器模拟可见范围，无生产权限；CSV文本前缀不改变系统保存值</t>
+        </is>
+      </c>
+      <c r="L106" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.22.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="88" customHeight="1">
+      <c r="A107" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>v0.22</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>兼容与异常保护</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>票面基准备份、旧10条规则兼容及坏字段/容量失败回退</t>
+        </is>
+      </c>
+      <c r="F107" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>迁移票面字段与处理依据，不补造旧字段或旧基准</t>
+        </is>
+      </c>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>数据管理 / 票据采集错误提示 / 历史预审</t>
+        </is>
+      </c>
+      <c r="I107" s="5" t="inlineStr">
+        <is>
+          <t>新备份恢复票面和14条规则；旧10条运行补齐默认提醒；失败保留原单和采集清单</t>
+        </is>
+      </c>
+      <c r="J107" s="5" t="inlineStr">
+        <is>
+          <t>131项业务测试通过、100项浏览器场景整套通过，导出修正后相关6项重跑通过；生产同构真实OCR抬头/日期/265元、200申请不覆盖、对公跨单线索、CSV/JSON/备份恢复及手机通过</t>
+        </is>
+      </c>
+      <c r="K107" s="5" t="inlineStr">
+        <is>
+          <t>本地数据、非不可篡改凭证；不补造老抬头/原金额或原件，真实用户效果未验证</t>
+        </is>
+      </c>
+      <c r="L107" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.22.md</t>
         </is>
       </c>
     </row>
@@ -7259,6 +7586,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L100" r:id="rId95"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L101" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L102" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L105" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L106" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L107" r:id="rId102"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7272,7 +7604,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId98"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId103"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7531,7 +7863,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>逐票OCR核对与明细绑定评估</t>
+          <t>票面与原附件及明细绑定</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -7541,22 +7873,22 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>多附件已可留存，但发票识别仍为原单张入口，未逐票关联明细</t>
+          <t>逐票结构化及跨单查重已交付，但票面记录尚未关联原文件和具体费用明细</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>评估从已存发票附件发起识别、多号码冲突提示、每票人工核对及明细关联</t>
+          <t>评估从已存附件发起识别、文件与字段关联、票据到费用行的分摊及重复引用</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>明确票据/明细对应、金额合计和重复规则，保留失败取消回退；不让OCR自动提交报销</t>
+          <t>可追溯原文件与人工核对字段，明细分摊不重计，失败取消回退；不自动提交或验真</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>多附件阶段已交付；逐票OCR尚未开发，先评审模型与实际操作反馈</t>
+          <t>结构化阶段已交付；逐原件/费用明细绑定仍未开发</t>
         </is>
       </c>
     </row>
@@ -7878,7 +8210,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.21 完成报销/对公10条补充规则、风险依据、提醒/拦截、处理时快照及配置异常保护；真实AI暂停，对公附件与统一待办待后续。</t>
+          <t>v0.22 完成多票结构化、购销方及金额税额OCR候选、财务抬头基准、四条票面规则与台账/JSON/CSV；真伪验证与原文件绑定未接。</t>
         </is>
       </c>
     </row>
@@ -7890,7 +8222,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.21</t>
+          <t>https://jameyan42.github.io/-/?v=0.22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record v0.23 delivery in feature history workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,11 +14,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$107</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$112</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'使用与维护'!$A$5:$B$17</definedName>
   </definedNames>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H26" headerRowCount="1">
-  <autoFilter ref="A5:H26"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H27" headerRowCount="1">
+  <autoFilter ref="A5:H27"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L107" headerRowCount="1">
-  <autoFilter ref="A5:L107"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L112" headerRowCount="1">
+  <autoFilter ref="A5:L112"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -264,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H13" headerRowCount="1">
-  <autoFilter ref="A5:H13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H12" headerRowCount="1">
+  <autoFilter ref="A5:H12"/>
   <tableColumns count="8">
     <tableColumn id="1" name="顺序"/>
     <tableColumn id="2" name="优先级"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 21 个阶段、102 项内容  |  当前功能版本 v0.22  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 22 个阶段、107 项内容  |  当前功能版本 v0.23  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1410,6 +1410,42 @@
       <c r="H26" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/defe80a</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="74" customHeight="1">
+      <c r="A27" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>v0.23</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>原件关联与对公履约附件</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>135项业务测试、103项浏览器场景整套通过；生产同构留存原件真实OCR、对公材料全审批/模拟付款、恢复原件下载字节一致、手机及PDF通过</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/caef12f</t>
         </is>
       </c>
     </row>
@@ -1441,6 +1477,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId22"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1454,7 +1491,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1466,7 +1503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7479,6 +7516,296 @@
       <c r="L107" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.22.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="88" customHeight="1">
+      <c r="A108" s="5" t="n">
+        <v>103</v>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>v0.23</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>票据与原件</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>票面显式关联原件、从留存图片OCR及PDF手工核对</t>
+        </is>
+      </c>
+      <c r="F108" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>字段可追溯到本单具体原件，不按文件名猜测</t>
+        </is>
+      </c>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>报销/对公编辑 → 附件区 → 结构化发票采集</t>
+        </is>
+      </c>
+      <c r="I108" s="5" t="inlineStr">
+        <is>
+          <t>先上传发票原件、选择关联、运行本地OCR并人工确认</t>
+        </is>
+      </c>
+      <c r="J108" s="5" t="inlineStr">
+        <is>
+          <t>135项业务测试、103项浏览器场景整套通过；生产同构留存原件真实OCR、对公材料全审批/模拟付款、恢复原件下载字节一致、手机及PDF通过</t>
+        </is>
+      </c>
+      <c r="K108" s="5" t="inlineStr">
+        <is>
+          <t>一原件限一票，PDF不识别，多票文件需拆分；仅选图OCR仍只存字段</t>
+        </is>
+      </c>
+      <c r="L108" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.23.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="88" customHeight="1">
+      <c r="A109" s="5" t="n">
+        <v>104</v>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>v0.23</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>对公材料</t>
+        </is>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>对公发票、验收单、合同附件等多份材料留存</t>
+        </is>
+      </c>
+      <c r="F109" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr">
+        <is>
+          <t>审核付款依据时可查看履约材料，与合同额度链路相连</t>
+        </is>
+      </c>
+      <c r="H109" s="5" t="inlineStr">
+        <is>
+          <t>对公支付单 → 新建/重提 → 对公附件</t>
+        </is>
+      </c>
+      <c r="I109" s="5" t="inlineStr">
+        <is>
+          <t>上传发票和验收单，完成指定主管/财务/总账/付款后查看保留原件</t>
+        </is>
+      </c>
+      <c r="J109" s="5" t="inlineStr">
+        <is>
+          <t>135项业务测试、103项浏览器场景整套通过；生产同构留存原件真实OCR、对公材料全审批/模拟付款、恢复原件下载字节一致、手机及PDF通过</t>
+        </is>
+      </c>
+      <c r="K109" s="5" t="inlineStr">
+        <is>
+          <t>本地单份1 MB、每单5份/1.5 MB，上传不证明已验收或发票真实</t>
+        </is>
+      </c>
+      <c r="L109" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.23.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="88" customHeight="1">
+      <c r="A110" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>v0.23</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>审核证据</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr">
+        <is>
+          <t>票面卡片原件预览/下载及字段JSON范围说明</t>
+        </is>
+      </c>
+      <c r="F110" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>审核人直接找到对应原件，区分字段导出和文件备份</t>
+        </is>
+      </c>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>报销/对公详情 → 结构化发票 → 关联原件</t>
+        </is>
+      </c>
+      <c r="I110" s="5" t="inlineStr">
+        <is>
+          <t>展开原图并下载，核对字节与上传一致；字段JSON含ID引用而无文件</t>
+        </is>
+      </c>
+      <c r="J110" s="5" t="inlineStr">
+        <is>
+          <t>135项业务测试、103项浏览器场景整套通过；生产同构留存原件真实OCR、对公材料全审批/模拟付款、恢复原件下载字节一致、手机及PDF通过</t>
+        </is>
+      </c>
+      <c r="K110" s="5" t="inlineStr">
+        <is>
+          <t>图片预览，PDF下载查看；只读是演示交互，非生产权限保障</t>
+        </is>
+      </c>
+      <c r="L110" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.23.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="88" customHeight="1">
+      <c r="A111" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>v0.23</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>关联保护</t>
+        </is>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>拦截已关联文件误删/改类，移除票面保留原件</t>
+        </is>
+      </c>
+      <c r="F111" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>防止已确认字段的证据丢失和隐式级联删除</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>报销/对公编辑 → 原件分类/移除及票面修订</t>
+        </is>
+      </c>
+      <c r="I111" s="5" t="inlineStr">
+        <is>
+          <t>尝试移除被拦；票面编辑选不关联确认后改类；移除字段后文件仍在</t>
+        </is>
+      </c>
+      <c r="J111" s="5" t="inlineStr">
+        <is>
+          <t>135项业务测试、103项浏览器场景整套通过；生产同构留存原件真实OCR、对公材料全审批/模拟付款、恢复原件下载字节一致、手机及PDF通过</t>
+        </is>
+      </c>
+      <c r="K111" s="5" t="inlineStr">
+        <is>
+          <t>修改仅保存单据后生效，不替代不可篡改归档或跨页面并发控制</t>
+        </is>
+      </c>
+      <c r="L111" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.23.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="88" customHeight="1">
+      <c r="A112" s="5" t="n">
+        <v>107</v>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>v0.23</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>备份与容量</t>
+        </is>
+      </c>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>原件引用校验、对公容量分层及重提/审批/恢复保留</t>
+        </is>
+      </c>
+      <c r="F112" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>迁移后仍可定位原件，坏引用及配额失败不覆盖原值</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>数据管理 / 对公提交错误 / 原件关联校验</t>
+        </is>
+      </c>
+      <c r="I112" s="5" t="inlineStr">
+        <is>
+          <t>恢复有效备份下载原件；坏ID拒绝；容量失败保留表单后重试</t>
+        </is>
+      </c>
+      <c r="J112" s="5" t="inlineStr">
+        <is>
+          <t>135项业务测试、103项浏览器场景整套通过；生产同构留存原件真实OCR、对公材料全审批/模拟付款、恢复原件下载字节一致、手机及PDF通过</t>
+        </is>
+      </c>
+      <c r="K112" s="5" t="inlineStr">
+        <is>
+          <t>旧无引用记录不补造，企业元数据80万/含文件220万字符，受浏览器总配额限制</t>
+        </is>
+      </c>
+      <c r="L112" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.23.md</t>
         </is>
       </c>
     </row>
@@ -7591,6 +7918,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L105" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L106" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L107" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L108" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L109" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L110" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L111" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L112" r:id="rId107"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7604,7 +7936,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId103"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId108"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7616,7 +7948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7646,7 +7978,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：对公履约附件与统一待办 → 预算模型评估；规则预审已交付，后续按使用反馈扩展；真实AI按用户选择暂缓。</t>
+          <t>建议顺序：对公统一待办与消息 → 费用行分摊及预算模型评估；规则预审已交付，后续按使用反馈扩展；真实AI按用户选择暂缓。</t>
         </is>
       </c>
     </row>
@@ -7703,32 +8035,32 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>对公履约附件与付款依据</t>
+          <t>对公统一待办及消息</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>建议下一阶段</t>
+          <t>待排期</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>对公单已有合同依据，但还不能留存验收单/发票等原文件</t>
+          <t>当前对公需到独立页面，原审批中心/消息仅汇集员工费用</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>复用附件校验与存储边界，区分验收、发票和付款凭证，保护已有合同及对公记录</t>
+          <t>明确定义corporate单据类型和个人处理历史，复用跳转而不伪装报销</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>指定人员可查看原文件，备份可恢复，容量失败不覆盖；不把上传视作验真</t>
+          <t>不同类型与人员范围准确，处理结果独立，已读不改业务，新事件提示一致</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>先评估企业数据容量与文件存储方式，不接真实财务资料</t>
+          <t>对公闭环已完成；需定义消息与历史兼容模型</t>
         </is>
       </c>
     </row>
@@ -7738,12 +8070,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>对公统一待办及消息</t>
+          <t>多法人及部门预算评估</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -7753,22 +8085,22 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>当前对公需到独立页面，原审批中心/消息仅汇集员工费用</t>
+          <t>当前只有单企业CNY及合同额度，未统一对公预算</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>明确定义corporate单据类型和个人处理历史，复用跳转而不伪装报销</t>
+          <t>先明确法人、预算维度、申请预留/合同/对公避免重复占用的口径</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>不同类型与人员范围准确，处理结果独立，已读不改业务，新事件提示一致</t>
+          <t>有可审查的业务模型及虚构场景后再开发，不提前宣称企业规模能力</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>对公闭环已完成；需定义消息与历史兼容模型</t>
+          <t>需要需求验证；当前不接真实会计系统</t>
         </is>
       </c>
     </row>
@@ -7783,7 +8115,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>多法人及部门预算评估</t>
+          <t>真实AI合同审查接入</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -7793,22 +8125,22 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>当前只有单企业CNY及合同额度，未统一对公预算</t>
+          <t>本地规则不能理解复杂法律语义，当前无模型服务端适配器</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>先明确法人、预算维度、申请预留/合同/对公避免重复占用的口径</t>
+          <t>后端保管密钥、模型选择、费用/合同范围授权、结构化风险及原文证据核验、人工兜底</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>有可审查的业务模型及虚构场景后再开发，不提前宣称企业规模能力</t>
+          <t>先完成可审查接口及模拟测试，必要授权后才真实调用；不把模型输出当法律结论</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>需要需求验证；当前不接真实会计系统</t>
+          <t>用户已选择先本地规则，真实AI稍后；真实服务需新账号权限及费用/数据范围确认</t>
         </is>
       </c>
     </row>
@@ -7818,37 +8150,37 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>真实AI合同审查接入</t>
+          <t>票面与费用明细分摊</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>待排期</t>
+          <t>建议下一阶段</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>本地规则不能理解复杂法律语义，当前无模型服务端适配器</t>
+          <t>原件关联与从已存图片OCR已交付，尚未按具体费用行分摊票面金额</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>后端保管密钥、模型选择、费用/合同范围授权、结构化风险及原文证据核验、人工兜底</t>
+          <t>评估票据到费用行的分摊、合并票据拆分及金额不重复计入</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>先完成可审查接口及模拟测试，必要授权后才真实调用；不把模型输出当法律结论</t>
+          <t>明确票据/费用行/申请金额关系，分摊不重计，修改与撤回可回退</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>用户已选择先本地规则，真实AI稍后；真实服务需新账号权限及费用/数据范围确认</t>
+          <t>v0.23完成原文件引用；费用明细分摊尚未开发</t>
         </is>
       </c>
     </row>
@@ -7863,32 +8195,32 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>票面与原附件及明细绑定</t>
+          <t>真实可用性测试</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>建议下一阶段</t>
+          <t>待用户参与</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>逐票结构化及跨单查重已交付，但票面记录尚未关联原文件和具体费用明细</t>
+          <t>自动化测试不能证明真实用户理解和使用顺畅</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>评估从已存附件发起识别、文件与字段关联、票据到费用行的分摊及重复引用</t>
+          <t>结合图形组织、部门总/财务/总账/付款路径，使用已准备任务收集真实参与者操作反馈</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>可追溯原文件与人工核对字段，明细分摊不重计，失败取消回退；不自动提交或验真</t>
+          <t>记录真实任务完成情况、困惑点与改进建议；无参与者前不写研究结论</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>结构化阶段已交付；逐原件/费用明细绑定仍未开发</t>
+          <t>需要用户协助招募实际参与者；AI 不能代替真实访谈</t>
         </is>
       </c>
     </row>
@@ -7898,37 +8230,37 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>真实可用性测试</t>
+          <t>复杂审批能力评估</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>待用户参与</t>
+          <t>暂缓</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>自动化测试不能证明真实用户理解和使用顺畅</t>
+          <t>尚无证据证明会签、或签、加签和嵌套条件为当前作品优先需求</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>结合图形组织、部门总/财务/总账/付款路径，使用已准备任务收集真实参与者操作反馈</t>
+          <t>先依据组织与审批树试用反馈，再决定是否扩展</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>记录真实任务完成情况、困惑点与改进建议；无参与者前不写研究结论</t>
+          <t>明确业务场景、异常策略与范围后再排开发</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>需要用户协助招募实际参与者；AI 不能代替真实访谈</t>
+          <t>不在当前 Excel 中记为已完成</t>
         </is>
       </c>
     </row>
@@ -7943,70 +8275,30 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>复杂审批能力评估</t>
+          <t>规则适用范围与疑点核对闭环</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>待排期</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>尚无证据证明会签、或签、加签和嵌套条件为当前作品优先需求</t>
+          <t>当前为统一固定规则目录，无组织适用范围或逐项核对状态</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>先依据组织与审批树试用反馈，再决定是否扩展</t>
+          <t>先验证提醒/拦截理解，再评估按部门类型配置及疑点逐项处置</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>明确业务场景、异常策略与范围后再排开发</t>
+          <t>明确规则冲突、审批节点及历史迁移口径后开发；不把已保存预审快照当作逐项核实</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>不在当前 Excel 中记为已完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="100" customHeight="1">
-      <c r="A13" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>规则适用范围与疑点核对闭环</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>待排期</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>当前为统一固定规则目录，无组织适用范围或逐项核对状态</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>先验证提醒/拦截理解，再评估按部门类型配置及疑点逐项处置</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>明确规则冲突、审批节点及历史迁移口径后开发；不把已保存预审快照当作逐项核实</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>当前规则预审已交付；需真实任务反馈决定范围</t>
         </is>
@@ -8210,7 +8502,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.22 完成多票结构化、购销方及金额税额OCR候选、财务抬头基准、四条票面规则与台账/JSON/CSV；真伪验证与原文件绑定未接。</t>
+          <t>v0.23完成报销/对公原件关联、从留存图片OCR、对公发票/验收材料、审核预览下载、误删改类保护及含文件备份；明细分摊与官方验真未接。</t>
         </is>
       </c>
     </row>
@@ -8222,7 +8514,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.22</t>
+          <t>https://jameyan42.github.io/-/?v=0.23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record v0.24 delivery in feature history workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,11 +14,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$28</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$112</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$117</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'使用与维护'!$A$5:$B$17</definedName>
   </definedNames>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H27" headerRowCount="1">
-  <autoFilter ref="A5:H27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H28" headerRowCount="1">
+  <autoFilter ref="A5:H28"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L112" headerRowCount="1">
-  <autoFilter ref="A5:L112"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L117" headerRowCount="1">
+  <autoFilter ref="A5:L117"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -264,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H12" headerRowCount="1">
-  <autoFilter ref="A5:H12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H11" headerRowCount="1">
+  <autoFilter ref="A5:H11"/>
   <tableColumns count="8">
     <tableColumn id="1" name="顺序"/>
     <tableColumn id="2" name="优先级"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 22 个阶段、107 项内容  |  当前功能版本 v0.23  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 23 个阶段、112 项内容  |  当前功能版本 v0.24  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1446,6 +1446,42 @@
       <c r="H27" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/caef12f</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="74" customHeight="1">
+      <c r="A28" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>v0.24</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>对公统一待办、已处理与消息</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>142项业务测试、108项浏览器场景整套通过；生产同构审批/消息四岗对公全流程、独立处理CSV、本人结果提示、操作/已读及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/5a3f24d</t>
         </is>
       </c>
     </row>
@@ -1478,6 +1514,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId23"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1491,7 +1528,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1503,7 +1540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7806,6 +7843,296 @@
       <c r="L112" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.23.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="88" customHeight="1">
+      <c r="A113" s="5" t="n">
+        <v>108</v>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>v0.24</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>统一审批</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>对公支付以独立类型纳入统一待办，可从原页面直接办理</t>
+        </is>
+      </c>
+      <c r="F113" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>指定人员不再切换独立业务页面找单，保持类型与路径边界</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>审批中心 → 待我处理 → 对公支付</t>
+        </is>
+      </c>
+      <c r="I113" s="5" t="inlineStr">
+        <is>
+          <t>赵航无待办、许明有待办；打开原对公详情，财务/总账/付款沿用指定路径办理</t>
+        </is>
+      </c>
+      <c r="J113" s="5" t="inlineStr">
+        <is>
+          <t>142项业务测试、108项浏览器场景整套通过；生产同构审批/消息四岗对公全流程、独立处理CSV、本人结果提示、操作/已读及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K113" s="5" t="inlineStr">
+        <is>
+          <t>只整合对公支付任务，合同复核、供应商变更及对公批量付款未纳入</t>
+        </is>
+      </c>
+      <c r="L113" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.24.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="88" customHeight="1">
+      <c r="A114" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>v0.24</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>个人处理记录</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>对公新操作保存处理时摘要、日期筛选/导出和历史人员只读回看</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>重提修改不覆盖原事项金额，原处理人能回顾而不能代办新节点</t>
+        </is>
+      </c>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>审批中心 → 我已处理 → 对公支付</t>
+        </is>
+      </c>
+      <c r="I114" s="5" t="inlineStr">
+        <is>
+          <t>退回后改金额重提，保留旧100元和新200元记录；总账/付款CSV各有独立摘要</t>
+        </is>
+      </c>
+      <c r="J114" s="5" t="inlineStr">
+        <is>
+          <t>142项业务测试、108项浏览器场景整套通过；生产同构审批/消息四岗对公全流程、独立处理CSV、本人结果提示、操作/已读及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K114" s="5" t="inlineStr">
+        <is>
+          <t>旧文本不补造；处理次数不是单据数或支出额；本地记录不防篡改</t>
+        </is>
+      </c>
+      <c r="L114" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.24.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="88" customHeight="1">
+      <c r="A115" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>v0.24</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>站内消息</t>
+        </is>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>对公具名待办及本人进展、类型筛选与跨页已读</t>
+        </is>
+      </c>
+      <c r="F115" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>统一提醒入口，区分读过和业务办完，新节点仍提示</t>
+        </is>
+      </c>
+      <c r="H115" s="5" t="inlineStr">
+        <is>
+          <t>消息中心 → 单据类型对公支付</t>
+        </is>
+      </c>
+      <c r="I115" s="5" t="inlineStr">
+        <is>
+          <t>标已读后待办还在；消息退回重提生成新未读，员工查看原因及模拟付款结果</t>
+        </is>
+      </c>
+      <c r="J115" s="5" t="inlineStr">
+        <is>
+          <t>142项业务测试、108项浏览器场景整套通过；生产同构审批/消息四岗对公全流程、独立处理CSV、本人结果提示、操作/已读及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K115" s="5" t="inlineStr">
+        <is>
+          <t>当前状态派生，无服务端投递、外部推送、系统通知或开发完成弹窗</t>
+        </is>
+      </c>
+      <c r="L115" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.24.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="88" customHeight="1">
+      <c r="A116" s="5" t="n">
+        <v>111</v>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>v0.24</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>列表效率</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>统一待办每页20条及全匹配CSV、筛选和页码联动</t>
+        </is>
+      </c>
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>多人多类型任务下避免单页过长，导出不漏其他匹配页</t>
+        </is>
+      </c>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>审批中心 → 待我处理 → 搜索/类型/排序/分页/导出</t>
+        </is>
+      </c>
+      <c r="I116" s="5" t="inlineStr">
+        <is>
+          <t>25条虚构对公待办显示20+5，导出25条；搜索重置第一页，手机无整页横向溢出</t>
+        </is>
+      </c>
+      <c r="J116" s="5" t="inlineStr">
+        <is>
+          <t>142项业务测试、108项浏览器场景整套通过；生产同构审批/消息四岗对公全流程、独立处理CSV、本人结果提示、操作/已读及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K116" s="5" t="inlineStr">
+        <is>
+          <t>概览与筛选数量分开；对公合同额度仍独立于原报销预算</t>
+        </is>
+      </c>
+      <c r="L116" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.24.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="88" customHeight="1">
+      <c r="A117" s="5" t="n">
+        <v>112</v>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>v0.24</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>兼容与异常保护</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>对公操作/已读备份兼容、坏集合部分提示与导出保护</t>
+        </is>
+      </c>
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>保留旧记录，避免损坏数据时把部分任务误认为全部</t>
+        </is>
+      </c>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>数据管理 / 审批与消息异常提示</t>
+        </is>
+      </c>
+      <c r="I117" s="5" t="inlineStr">
+        <is>
+          <t>恢复操作和已读；坏操作拒绝；配额失败不增加处理次数；坏对公存储保留且角标未知</t>
+        </is>
+      </c>
+      <c r="J117" s="5" t="inlineStr">
+        <is>
+          <t>142项业务测试、108项浏览器场景整套通过；生产同构审批/消息四岗对公全流程、独立处理CSV、本人结果提示、操作/已读及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K117" s="5" t="inlineStr">
+        <is>
+          <t>恢复需有效备份；无跨设备并发或断电事务，身份是模拟机制</t>
+        </is>
+      </c>
+      <c r="L117" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.24.md</t>
         </is>
       </c>
     </row>
@@ -7923,6 +8250,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L110" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L111" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L112" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L113" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L114" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L115" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L116" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L117" r:id="rId112"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7936,7 +8268,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId108"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId113"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7948,7 +8280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7978,7 +8310,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：对公统一待办与消息 → 费用行分摊及预算模型评估；规则预审已交付，后续按使用反馈扩展；真实AI按用户选择暂缓。</t>
+          <t>建议顺序：费用行分摊及预算模型评估 → 规则疑点处置与真实可用性验证；规则预审已交付，后续按使用反馈扩展；真实AI按用户选择暂缓。</t>
         </is>
       </c>
     </row>
@@ -8030,12 +8362,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>对公统一待办及消息</t>
+          <t>多法人及部门预算评估</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -8045,22 +8377,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>当前对公需到独立页面，原审批中心/消息仅汇集员工费用</t>
+          <t>当前只有单企业CNY及合同额度，未统一对公预算</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>明确定义corporate单据类型和个人处理历史，复用跳转而不伪装报销</t>
+          <t>先明确法人、预算维度、申请预留/合同/对公避免重复占用的口径</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>不同类型与人员范围准确，处理结果独立，已读不改业务，新事件提示一致</t>
+          <t>有可审查的业务模型及虚构场景后再开发，不提前宣称企业规模能力</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>对公闭环已完成；需定义消息与历史兼容模型</t>
+          <t>需要需求验证；当前不接真实会计系统</t>
         </is>
       </c>
     </row>
@@ -8075,7 +8407,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>多法人及部门预算评估</t>
+          <t>真实AI合同审查接入</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -8085,22 +8417,22 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>当前只有单企业CNY及合同额度，未统一对公预算</t>
+          <t>本地规则不能理解复杂法律语义，当前无模型服务端适配器</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>先明确法人、预算维度、申请预留/合同/对公避免重复占用的口径</t>
+          <t>后端保管密钥、模型选择、费用/合同范围授权、结构化风险及原文证据核验、人工兜底</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>有可审查的业务模型及虚构场景后再开发，不提前宣称企业规模能力</t>
+          <t>先完成可审查接口及模拟测试，必要授权后才真实调用；不把模型输出当法律结论</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>需要需求验证；当前不接真实会计系统</t>
+          <t>用户已选择先本地规则，真实AI稍后；真实服务需新账号权限及费用/数据范围确认</t>
         </is>
       </c>
     </row>
@@ -8110,37 +8442,37 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>真实AI合同审查接入</t>
+          <t>票面与费用明细分摊</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>待排期</t>
+          <t>建议下一阶段</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>本地规则不能理解复杂法律语义，当前无模型服务端适配器</t>
+          <t>原件关联与从已存图片OCR已交付，尚未按具体费用行分摊票面金额</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后端保管密钥、模型选择、费用/合同范围授权、结构化风险及原文证据核验、人工兜底</t>
+          <t>评估票据到费用行的分摊、合并票据拆分及金额不重复计入</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>先完成可审查接口及模拟测试，必要授权后才真实调用；不把模型输出当法律结论</t>
+          <t>明确票据/费用行/申请金额关系，分摊不重计，修改与撤回可回退</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>用户已选择先本地规则，真实AI稍后；真实服务需新账号权限及费用/数据范围确认</t>
+          <t>v0.23完成原文件引用；费用明细分摊尚未开发</t>
         </is>
       </c>
     </row>
@@ -8155,32 +8487,32 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>票面与费用明细分摊</t>
+          <t>真实可用性测试</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>建议下一阶段</t>
+          <t>待用户参与</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>原件关联与从已存图片OCR已交付，尚未按具体费用行分摊票面金额</t>
+          <t>自动化测试不能证明真实用户理解和使用顺畅</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>评估票据到费用行的分摊、合并票据拆分及金额不重复计入</t>
+          <t>结合图形组织、部门总/财务/总账/付款路径，使用已准备任务收集真实参与者操作反馈</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>明确票据/费用行/申请金额关系，分摊不重计，修改与撤回可回退</t>
+          <t>记录真实任务完成情况、困惑点与改进建议；无参与者前不写研究结论</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>v0.23完成原文件引用；费用明细分摊尚未开发</t>
+          <t>需要用户协助招募实际参与者；AI 不能代替真实访谈</t>
         </is>
       </c>
     </row>
@@ -8190,37 +8522,37 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>真实可用性测试</t>
+          <t>复杂审批能力评估</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>待用户参与</t>
+          <t>暂缓</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>自动化测试不能证明真实用户理解和使用顺畅</t>
+          <t>尚无证据证明会签、或签、加签和嵌套条件为当前作品优先需求</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>结合图形组织、部门总/财务/总账/付款路径，使用已准备任务收集真实参与者操作反馈</t>
+          <t>先依据组织与审批树试用反馈，再决定是否扩展</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>记录真实任务完成情况、困惑点与改进建议；无参与者前不写研究结论</t>
+          <t>明确业务场景、异常策略与范围后再排开发</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>需要用户协助招募实际参与者；AI 不能代替真实访谈</t>
+          <t>不在当前 Excel 中记为已完成</t>
         </is>
       </c>
     </row>
@@ -8235,70 +8567,30 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>复杂审批能力评估</t>
+          <t>规则适用范围与疑点核对闭环</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>暂缓</t>
+          <t>待排期</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>尚无证据证明会签、或签、加签和嵌套条件为当前作品优先需求</t>
+          <t>当前为统一固定规则目录，无组织适用范围或逐项核对状态</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>先依据组织与审批树试用反馈，再决定是否扩展</t>
+          <t>先验证提醒/拦截理解，再评估按部门类型配置及疑点逐项处置</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>明确业务场景、异常策略与范围后再排开发</t>
+          <t>明确规则冲突、审批节点及历史迁移口径后开发；不把已保存预审快照当作逐项核实</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>不在当前 Excel 中记为已完成</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="100" customHeight="1">
-      <c r="A12" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>规则适用范围与疑点核对闭环</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>待排期</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>当前为统一固定规则目录，无组织适用范围或逐项核对状态</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>先验证提醒/拦截理解，再评估按部门类型配置及疑点逐项处置</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>明确规则冲突、审批节点及历史迁移口径后开发；不把已保存预审快照当作逐项核实</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>当前规则预审已交付；需真实任务反馈决定范围</t>
         </is>
@@ -8502,7 +8794,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.23完成报销/对公原件关联、从留存图片OCR、对公发票/验收材料、审核预览下载、误删改类保护及含文件备份；明细分摊与官方验真未接。</t>
+          <t>v0.24完成对公统一待办、已处理摘要及日期CSV、消息类型筛选/跨页已读、统一待办分页和部分数据异常保护；合同复核待办、对公批量付款及费用分摊未接。</t>
         </is>
       </c>
     </row>
@@ -8514,7 +8806,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.23</t>
+          <t>https://jameyan42.github.io/-/?v=0.24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record v0.25 risk review delivery in feature workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$29</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$117</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$122</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H28" headerRowCount="1">
-  <autoFilter ref="A5:H28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H29" headerRowCount="1">
+  <autoFilter ref="A5:H29"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L117" headerRowCount="1">
-  <autoFilter ref="A5:L117"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L122" headerRowCount="1">
+  <autoFilter ref="A5:L122"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 23 个阶段、112 项内容  |  当前功能版本 v0.24  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 24 个阶段、117 项内容  |  当前功能版本 v0.25  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1482,6 +1482,42 @@
       <c r="H28" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/5a3f24d</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="74" customHeight="1">
+      <c r="A29" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>v0.25</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>风险逐项核对与依据变化提示</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>150项业务测试、113项浏览器场景整套通过，文案更新后相关15项重跑；生产同构报销两级/对公四岗核对、材料关联、CSV/记录及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/dfbfb08</t>
         </is>
       </c>
     </row>
@@ -1515,6 +1551,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId24"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1528,7 +1565,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1540,7 +1577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8133,6 +8170,296 @@
       <c r="L117" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.24.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="88" customHeight="1">
+      <c r="A118" s="5" t="n">
+        <v>113</v>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>v0.25</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>人工风险核对</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>报销及对公按命中疑点记录具名结论、说明和材料关联</t>
+        </is>
+      </c>
+      <c r="F118" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G118" s="5" t="inlineStr">
+        <is>
+          <t>后续节点知道前一人核对了什么、还缺什么材料</t>
+        </is>
+      </c>
+      <c r="H118" s="5" t="inlineStr">
+        <is>
+          <t>报销/对公详情 → 风险逐项核对</t>
+        </is>
+      </c>
+      <c r="I118" s="5" t="inlineStr">
+        <is>
+          <t>当前处理人选择疑点、写5～500字说明并关联本单材料，后续节点只读回看及追加</t>
+        </is>
+      </c>
+      <c r="J118" s="5" t="inlineStr">
+        <is>
+          <t>150项业务测试、113项浏览器场景整套通过，文案更新后相关15项重跑；生产同构报销两级/对公四岗核对、材料关联、CSV/记录及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K118" s="5" t="inlineStr">
+        <is>
+          <t>只是人工核对说明，未实现AI审核、履约确认或全项强制核对</t>
+        </is>
+      </c>
+      <c r="L118" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.25.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="88" customHeight="1">
+      <c r="A119" s="5" t="n">
+        <v>114</v>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>v0.25</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>依据有效性</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>规则、单据、原件字节和重提变化后提示重新核对</t>
+        </is>
+      </c>
+      <c r="F119" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr">
+        <is>
+          <t>避免旧说明被当作修改后材料或新规则下的判断</t>
+        </is>
+      </c>
+      <c r="H119" s="5" t="inlineStr">
+        <is>
+          <t>风险逐项核对 → 当前疑点及历史有效性</t>
+        </is>
+      </c>
+      <c r="I119" s="5" t="inlineStr">
+        <is>
+          <t>同名同大小文件换字节、改金额重提或更新规则，旧记录失效；正常节点推进仍有效</t>
+        </is>
+      </c>
+      <c r="J119" s="5" t="inlineStr">
+        <is>
+          <t>150项业务测试、113项浏览器场景整套通过，文案更新后相关15项重跑；生产同构报销两级/对公四岗核对、材料关联、CSV/记录及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K119" s="5" t="inlineStr">
+        <is>
+          <t>本地SHA-256变更标识不是签名或防篡改审计；政策变化整体要求重核</t>
+        </is>
+      </c>
+      <c r="L119" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.25.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="88" customHeight="1">
+      <c r="A120" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>v0.25</t>
+        </is>
+      </c>
+      <c r="C120" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>审批安全边界</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>核对与审批独立保存、拦截不豁免及未保存输入保护</t>
+        </is>
+      </c>
+      <c r="F120" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G120" s="5" t="inlineStr">
+        <is>
+          <t>避免写了已核对就绕过规则，防止误丢正在填写的说明</t>
+        </is>
+      </c>
+      <c r="H120" s="5" t="inlineStr">
+        <is>
+          <t>核对保存 / 关闭 / 审批与退回按钮</t>
+        </is>
+      </c>
+      <c r="I120" s="5" t="inlineStr">
+        <is>
+          <t>记录已核对后财务仍受缺票或大额拦截；先保存或放弃候选才能办理，配额失败保留输入</t>
+        </is>
+      </c>
+      <c r="J120" s="5" t="inlineStr">
+        <is>
+          <t>150项业务测试、113项浏览器场景整套通过，文案更新后相关15项重跑；生产同构报销两级/对公四岗核对、材料关联、CSV/记录及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K120" s="5" t="inlineStr">
+        <is>
+          <t>待补充和建议退回不自动流转；没有豁免审批或材料补交任务</t>
+        </is>
+      </c>
+      <c r="L120" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.25.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="88" customHeight="1">
+      <c r="A121" s="5" t="n">
+        <v>116</v>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>v0.25</t>
+        </is>
+      </c>
+      <c r="C121" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>核对历史与导出</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>当时规则依据、金额/日期/轮次和个人节点快照及CSV</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr">
+        <is>
+          <t>区分当时的核对与当前依据，历史追加不被改写</t>
+        </is>
+      </c>
+      <c r="H121" s="5" t="inlineStr">
+        <is>
+          <t>风险逐项核对 → 查看全部记录 / 导出CSV</t>
+        </is>
+      </c>
+      <c r="I121" s="5" t="inlineStr">
+        <is>
+          <t>主管和财务分别保存说明，查看旧金额和触发依据，CSV含有效性、材料名称及节点</t>
+        </is>
+      </c>
+      <c r="J121" s="5" t="inlineStr">
+        <is>
+          <t>150项业务测试、113项浏览器场景整套通过，文案更新后相关15项重跑；生产同构报销两级/对公四岗核对、材料关联、CSV/记录及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K121" s="5" t="inlineStr">
+        <is>
+          <t>不从旧审批备注补造核对，不构成所有旧字段或旧原件的完整归档</t>
+        </is>
+      </c>
+      <c r="L121" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.25.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="88" customHeight="1">
+      <c r="A122" s="5" t="n">
+        <v>117</v>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>v0.25</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D122" s="5" t="inlineStr">
+        <is>
+          <t>备份与异常保护</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>核对记录备份兼容、容量/坏格式保护和重提保留</t>
+        </is>
+      </c>
+      <c r="F122" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr">
+        <is>
+          <t>已有数据不被隐式清空，迁移后仍可查看核对依据</t>
+        </is>
+      </c>
+      <c r="H122" s="5" t="inlineStr">
+        <is>
+          <t>数据管理 / 核对保存错误提示</t>
+        </is>
+      </c>
+      <c r="I122" s="5" t="inlineStr">
+        <is>
+          <t>恢复报销及对公核对；坏快照拒绝不覆盖；重提保留旧记录且失效；记录不改消息事件</t>
+        </is>
+      </c>
+      <c r="J122" s="5" t="inlineStr">
+        <is>
+          <t>150项业务测试、113项浏览器场景整套通过，文案更新后相关15项重跑；生产同构报销两级/对公四岗核对、材料关联、CSV/记录及原件备份恢复、手机/PDF通过</t>
+        </is>
+      </c>
+      <c r="K122" s="5" t="inlineStr">
+        <is>
+          <t>每单100条/40万字符与浏览器配额限制，无跨标签并发或生产后端</t>
+        </is>
+      </c>
+      <c r="L122" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.25.md</t>
         </is>
       </c>
     </row>
@@ -8255,6 +8582,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L115" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L116" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L117" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L118" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L119" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L122" r:id="rId117"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8268,7 +8600,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId113"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId118"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8310,7 +8642,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：费用行分摊及预算模型评估 → 规则疑点处置与真实可用性验证；规则预审已交付，后续按使用反馈扩展；真实AI按用户选择暂缓。</t>
+          <t>建议顺序：费用行分摊及预算模型评估 → 制度适用/核对策略与真实可用性验证；规则预审已交付，后续按使用反馈扩展；真实AI按用户选择暂缓。</t>
         </is>
       </c>
     </row>
@@ -8567,7 +8899,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>规则适用范围与疑点核对闭环</t>
+          <t>规则适用范围与核对策略评估</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -8577,22 +8909,22 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>当前为统一固定规则目录，无组织适用范围或逐项核对状态</t>
+          <t>逐项核对留痕已交付，但仍为统一固定规则目录，无组织制度适用范围</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>先验证提醒/拦截理解，再评估按部门类型配置及疑点逐项处置</t>
+          <t>依据真实反馈评估按部门类型配置、关键节点强制确认及风险豁免策略</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>明确规则冲突、审批节点及历史迁移口径后开发；不把已保存预审快照当作逐项核实</t>
+          <t>明确规则冲突、审批责任、版本迁移及异常口径后开发，不把核对说明当作豁免</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>当前规则预审已交付；需真实任务反馈决定范围</t>
+          <t>v0.25已完成逐项核对与依据失效；组织适用和豁免机制尚未实现</t>
         </is>
       </c>
     </row>
@@ -8794,7 +9126,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.24完成对公统一待办、已处理摘要及日期CSV、消息类型筛选/跨页已读、统一待办分页和部分数据异常保护；合同复核待办、对公批量付款及费用分摊未接。</t>
+          <t>v0.25完成报销/对公风险逐项核对、材料关联、依据变化提示、核对历史/CSV及备份异常保护；核对不豁免拦截，制度适用、豁免及补交任务未接。</t>
         </is>
       </c>
     </row>
@@ -8806,7 +9138,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.24</t>
+          <t>https://jameyan42.github.io/-/?v=0.25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record budget and interview readiness milestone in feature workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$122</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$127</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H29" headerRowCount="1">
-  <autoFilter ref="A5:H29"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H30" headerRowCount="1">
+  <autoFilter ref="A5:H30"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L122" headerRowCount="1">
-  <autoFilter ref="A5:L122"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L127" headerRowCount="1">
+  <autoFilter ref="A5:L127"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 24 个阶段、117 项内容  |  当前功能版本 v0.25  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 25 个阶段、122 项内容  |  当前功能版本 v0.26  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1518,6 +1518,42 @@
       <c r="H29" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/dfbfb08</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="74" customHeight="1">
+      <c r="A30" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>v0.26</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>月度预算闭环与面试展示版收尾</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>157项业务测试、119项浏览器场景整套通过，预算/组织/财务分工17项及坏数据保护补充场景通过；生产同构1000申请→265真实OCR报销/四岗模拟付款→735释放、4125占用，明细/备份及两份PDF通过</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/86b9bad</t>
         </is>
       </c>
     </row>
@@ -1552,6 +1588,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId25"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1565,7 +1602,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1577,7 +1614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8460,6 +8497,296 @@
       <c r="L122" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.25.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="88" customHeight="1">
+      <c r="A123" s="5" t="n">
+        <v>118</v>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>v0.26</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>月度预算</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>部门/月独立额度、软预警或新增硬控及具名调整历史</t>
+        </is>
+      </c>
+      <c r="F123" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>补齐每月独立计划与配置变化的业务依据</t>
+        </is>
+      </c>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>预算管理 → 月份 → 调整本月额度与管控</t>
+        </is>
+      </c>
+      <c r="I123" s="5" t="inlineStr">
+        <is>
+          <t>配置产品部本月4860元/block，次月仍15000元默认；查看前后值、原因与人员</t>
+        </is>
+      </c>
+      <c r="J123" s="5" t="inlineStr">
+        <is>
+          <t>157项业务测试、119项浏览器场景整套通过，预算/组织/财务分工17项及坏数据保护补充场景通过；生产同构1000申请→265真实OCR报销/四岗模拟付款→735释放、4125占用，明细/备份及两份PDF通过</t>
+        </is>
+      </c>
+      <c r="K123" s="5" t="inlineStr">
+        <is>
+          <t>单企业部门/月度，不含多法人、费用类型或对公预算；旧默认仍保留</t>
+        </is>
+      </c>
+      <c r="L123" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.26.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="88" customHeight="1">
+      <c r="A124" s="5" t="n">
+        <v>119</v>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>v0.26</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>预算事前管控</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>报销正式提交/重提和申请最终批准的新增占用门槛</t>
+        </is>
+      </c>
+      <c r="F124" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G124" s="5" t="inlineStr">
+        <is>
+          <t>超额阻止新增，既有预留核销/付款不重复扣预算</t>
+        </is>
+      </c>
+      <c r="H124" s="5" t="inlineStr">
+        <is>
+          <t>新建报销 / 费用申请最终批准</t>
+        </is>
+      </c>
+      <c r="I124" s="5" t="inlineStr">
+        <is>
+          <t>1000元申请占满后额外1元被拦；265元关联核销仍可流转，降额不阻断既有预留转换</t>
+        </is>
+      </c>
+      <c r="J124" s="5" t="inlineStr">
+        <is>
+          <t>157项业务测试、119项浏览器场景整套通过，预算/组织/财务分工17项及坏数据保护补充场景通过；生产同构1000申请→265真实OCR报销/四岗模拟付款→735释放、4125占用，明细/备份及两份PDF通过</t>
+        </is>
+      </c>
+      <c r="K124" s="5" t="inlineStr">
+        <is>
+          <t>同浏览器比较，无服务端并发预算锁、冻结/追加审批或跨月摊销</t>
+        </is>
+      </c>
+      <c r="L124" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.26.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="88" customHeight="1">
+      <c r="A125" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>v0.26</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>预算执行解释</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>贡献明细下钻、原单跳转、20条分页及全匹配CSV</t>
+        </is>
+      </c>
+      <c r="F125" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>说明每一元占用来自哪笔申请或报销，避免重复计数</t>
+        </is>
+      </c>
+      <c r="H125" s="5" t="inlineStr">
+        <is>
+          <t>预算管理 → 占用明细 / 月度汇总CSV</t>
+        </is>
+      </c>
+      <c r="I125" s="5" t="inlineStr">
+        <is>
+          <t>申请1000转报销265+余额735，付款后结束释放735，初始产品部最终占用4125</t>
+        </is>
+      </c>
+      <c r="J125" s="5" t="inlineStr">
+        <is>
+          <t>157项业务测试、119项浏览器场景整套通过，预算/组织/财务分工17项及坏数据保护补充场景通过；生产同构1000申请→265真实OCR报销/四岗模拟付款→735释放、4125占用，明细/备份及两份PDF通过</t>
+        </is>
+      </c>
+      <c r="K125" s="5" t="inlineStr">
+        <is>
+          <t>批准总额只作说明，贡献只计剩余；对公仍使用独立合同额度</t>
+        </is>
+      </c>
+      <c r="L125" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.26.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="88" customHeight="1">
+      <c r="A126" s="5" t="n">
+        <v>121</v>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>v0.26</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t>预算迁移保护</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>月度配置新旧备份、容量/损坏与失败回退保护</t>
+        </is>
+      </c>
+      <c r="F126" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G126" s="5" t="inlineStr">
+        <is>
+          <t>旧配置不被静默覆盖，异常时不误判可用额度或增加占用</t>
+        </is>
+      </c>
+      <c r="H126" s="5" t="inlineStr">
+        <is>
+          <t>数据管理 / 预算异常提示 / 草稿与提交</t>
+        </is>
+      </c>
+      <c r="I126" s="5" t="inlineStr">
+        <is>
+          <t>旧备份保留当前月配置；坏数据暂停新增和导出，配置保存失败保留输入及原值</t>
+        </is>
+      </c>
+      <c r="J126" s="5" t="inlineStr">
+        <is>
+          <t>157项业务测试、119项浏览器场景整套通过，预算/组织/财务分工17项及坏数据保护补充场景通过；生产同构1000申请→265真实OCR报销/四岗模拟付款→735释放、4125占用，明细/备份及两份PDF通过</t>
+        </is>
+      </c>
+      <c r="K126" s="5" t="inlineStr">
+        <is>
+          <t>240个期间、500条调整/40万字符，未知数据需有效备份恢复，不能宣称生产安全保障</t>
+        </is>
+      </c>
+      <c r="L126" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.26.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="88" customHeight="1">
+      <c r="A127" s="5" t="n">
+        <v>122</v>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>v0.26</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>面试准备</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>直达准备页、10分钟路线、6个决策、12个问答与Markdown/PDF手册</t>
+        </is>
+      </c>
+      <c r="F127" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G127" s="5" t="inlineStr">
+        <is>
+          <t>把可操作业务闭环转成可讲清的产品分析和验证证据</t>
+        </is>
+      </c>
+      <c r="H127" s="5" t="inlineStr">
+        <is>
+          <t>面试准备 / ?view=interview / 下载手册</t>
+        </is>
+      </c>
+      <c r="I127" s="5" t="inlineStr">
+        <is>
+          <t>按角色跳转演练预算与报销，读决策及问答；7页手册和4页案例可离线准备</t>
+        </is>
+      </c>
+      <c r="J127" s="5" t="inlineStr">
+        <is>
+          <t>157项业务测试、119项浏览器场景整套通过，预算/组织/财务分工17项及坏数据保护补充场景通过；生产同构1000申请→265真实OCR报销/四岗模拟付款→735释放、4125占用，明细/备份及两份PDF通过</t>
+        </is>
+      </c>
+      <c r="K127" s="5" t="inlineStr">
+        <is>
+          <t>模板按本人实际参与修改，自动化不代表真实研究或收益；今天优先亲自演练答辩</t>
+        </is>
+      </c>
+      <c r="L127" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.26.md</t>
         </is>
       </c>
     </row>
@@ -8587,6 +8914,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L122" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L123" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L124" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L125" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L126" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L127" r:id="rId122"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8600,7 +8932,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId118"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId123"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8642,7 +8974,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>建议顺序：费用行分摊及预算模型评估 → 制度适用/核对策略与真实可用性验证；规则预审已交付，后续按使用反馈扩展；真实AI按用户选择暂缓。</t>
+          <t>建议顺序：今天先亲自演练与准备答辩 → 真实可用性验证；费用分摊、多法人及制度扩展按反馈排期；规则预审已交付，后续按使用反馈扩展；真实AI按用户选择暂缓。</t>
         </is>
       </c>
     </row>
@@ -8699,7 +9031,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>多法人及部门预算评估</t>
+          <t>多法人与预算维度扩展评估</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -8709,22 +9041,22 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>当前只有单企业CNY及合同额度，未统一对公预算</t>
+          <t>已完成单企业部门/月独立预算和新增硬控，尚无多法人、项目/费用类型预算及并发控制</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>先明确法人、预算维度、申请预留/合同/对公避免重复占用的口径</t>
+          <t>按真实任务反馈评估法人/项目/类型归属和跨主体口径，再设计后端预算事务</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>有可审查的业务模型及虚构场景后再开发，不提前宣称企业规模能力</t>
+          <t>明确主数据、占用释放、不重计、并发与历史迁移规则，再排开发</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>需要需求验证；当前不接真实会计系统</t>
+          <t>v0.26仅交付单企业部门/月度；今天先演练与答辩，扩展未计为已完成</t>
         </is>
       </c>
     </row>
@@ -9042,7 +9374,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>已存在于代码和交付记录；不代表已做真实客户验证、生产安全审计或取得业务收益。</t>
+          <t>已存在于代码和交付记录；每条为阶段新增或改进，不等于独立模块数量，也不代表真实客户验证、生产安全审计或业务收益。</t>
         </is>
       </c>
     </row>
@@ -9126,7 +9458,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.25完成报销/对公风险逐项核对、材料关联、依据变化提示、核对历史/CSV及备份异常保护；核对不豁免拦截，制度适用、豁免及补交任务未接。</t>
+          <t>v0.26完成部门月度预算、新增占用硬控/核销不重扣、贡献明细、备份保护及面试准备手册；已可做个人原型演示，不代表生产落地或真实收益。</t>
         </is>
       </c>
     </row>
@@ -9138,7 +9470,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.25</t>
+          <t>https://jameyan42.github.io/-/?v=0.26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record PDF OCR delivery and verification in iteration workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$31</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$127</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$131</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H30" headerRowCount="1">
-  <autoFilter ref="A5:H30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H31" headerRowCount="1">
+  <autoFilter ref="A5:H31"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L127" headerRowCount="1">
-  <autoFilter ref="A5:L127"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L131" headerRowCount="1">
+  <autoFilter ref="A5:L131"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 25 个阶段、122 项内容  |  当前功能版本 v0.26  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 26 个阶段、126 项内容  |  当前功能版本 v0.27  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1554,6 +1554,42 @@
       <c r="H30" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/86b9bad</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="74" customHeight="1">
+      <c r="A31" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>v0.27</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>PDF发票本地识别与选页预览</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>159项业务测试、125项浏览器场景整套通过，最终OCR/PDF14项回归通过；生产同构PDF第2页真实识别265元并完成四岗模拟付款、735释放及备份原字节一致</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/2dfe512</t>
         </is>
       </c>
     </row>
@@ -1589,6 +1625,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId26"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1602,7 +1639,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1614,7 +1651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8787,6 +8824,238 @@
       <c r="L127" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.26.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="88" customHeight="1">
+      <c r="A128" s="5" t="n">
+        <v>123</v>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>v0.27</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D128" s="5" t="inlineStr">
+        <is>
+          <t>PDF快速识别</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>扫描/电子PDF逐页预览、本地OCR及旋转裁剪</t>
+        </is>
+      </c>
+      <c r="F128" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G128" s="5" t="inlineStr">
+        <is>
+          <t>补齐常见发票格式在报销录入中的断点</t>
+        </is>
+      </c>
+      <c r="H128" s="5" t="inlineStr">
+        <is>
+          <t>员工→新建报销→发票OCR</t>
+        </is>
+      </c>
+      <c r="I128" s="5" t="inlineStr">
+        <is>
+          <t>下载虚构PDF，选第2页，识别265元，核对后才填入</t>
+        </is>
+      </c>
+      <c r="J128" s="5" t="inlineStr">
+        <is>
+          <t>159项业务测试、125项浏览器场景整套通过，最终OCR/PDF14项回归通过；生产同构PDF第2页真实识别265元并完成四岗模拟付款、735释放及备份原字节一致</t>
+        </is>
+      </c>
+      <c r="K128" s="5" t="inlineStr">
+        <is>
+          <t>6 MB/20页，每次一页；不自动合并金额，不代表验真</t>
+        </is>
+      </c>
+      <c r="L128" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.27.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="88" customHeight="1">
+      <c r="A129" s="5" t="n">
+        <v>124</v>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>v0.27</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>PDF结构化与原件</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>报销/对公从所选PDF及已留存PDF采集，来源保留页码及原件引用</t>
+        </is>
+      </c>
+      <c r="F129" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G129" s="5" t="inlineStr">
+        <is>
+          <t>让字段、原件和审核链路连续，避免二次转图与手工抄录</t>
+        </is>
+      </c>
+      <c r="H129" s="5" t="inlineStr">
+        <is>
+          <t>结构化发票采集→关联原件→识别</t>
+        </is>
+      </c>
+      <c r="I129" s="5" t="inlineStr">
+        <is>
+          <t>保留PDF原件，选页识别购销方/金额，确认后保存并下载备份核对字节</t>
+        </is>
+      </c>
+      <c r="J129" s="5" t="inlineStr">
+        <is>
+          <t>159项业务测试、125项浏览器场景整套通过，最终OCR/PDF14项回归通过；生产同构PDF第2页真实识别265元并完成四岗模拟付款、735释放及备份原字节一致</t>
+        </is>
+      </c>
+      <c r="K129" s="5" t="inlineStr">
+        <is>
+          <t>一原件一票面，合并多票须拆分；原件留存容量仍为1 MB/份、1.5 MB/单</t>
+        </is>
+      </c>
+      <c r="L129" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.27.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="88" customHeight="1">
+      <c r="A130" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>v0.27</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>PDF异常与本地资源</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>同源PDF.js/Worker/字体资源，加密/超页/坏文件回退及取消保护</t>
+        </is>
+      </c>
+      <c r="F130" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G130" s="5" t="inlineStr">
+        <is>
+          <t>识别失败不覆盖已填数据，不引入外部文件上传服务</t>
+        </is>
+      </c>
+      <c r="H130" s="5" t="inlineStr">
+        <is>
+          <t>选PDF异常提示 / 取消识别 / 手工填写</t>
+        </is>
+      </c>
+      <c r="I130" s="5" t="inlineStr">
+        <is>
+          <t>加密或21页PDF提示回退，取消读取后新表单不接收迟到候选</t>
+        </is>
+      </c>
+      <c r="J130" s="5" t="inlineStr">
+        <is>
+          <t>159项业务测试、125项浏览器场景整套通过，最终OCR/PDF14项回归通过；生产同构PDF第2页真实识别265元并完成四岗模拟付款、735释放及备份原字节一致</t>
+        </is>
+      </c>
+      <c r="K130" s="5" t="inlineStr">
+        <is>
+          <t>无真实密码处理，无生产安全扫描；OCR与渲染仍受浏览器性能及版式影响</t>
+        </is>
+      </c>
+      <c r="L130" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.27.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="88" customHeight="1">
+      <c r="A131" s="5" t="n">
+        <v>126</v>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>v0.27</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>PDF样票与产品复盘</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>两页扫描样票和电子/加密/超限夹具，文档/Excel/ZIP同步</t>
+        </is>
+      </c>
+      <c r="F131" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G131" s="5" t="inlineStr">
+        <is>
+          <t>提供可复现演示与范围取舍，支持面试解释</t>
+        </is>
+      </c>
+      <c r="H131" s="5" t="inlineStr">
+        <is>
+          <t>OCR区下载虚构PDF / docs / 功能Excel</t>
+        </is>
+      </c>
+      <c r="I131" s="5" t="inlineStr">
+        <is>
+          <t>使用第2页真实OCR跑申请核销审批闭环，说明为何逐页与人工确认</t>
+        </is>
+      </c>
+      <c r="J131" s="5" t="inlineStr">
+        <is>
+          <t>159项业务测试、125项浏览器场景整套通过，最终OCR/PDF14项回归通过；生产同构PDF第2页真实识别265元并完成四岗模拟付款、735释放及备份原字节一致</t>
+        </is>
+      </c>
+      <c r="K131" s="5" t="inlineStr">
+        <is>
+          <t>样票通过不代表通用准确率、真实调研或收益；面试主路线继续以理解业务为先</t>
+        </is>
+      </c>
+      <c r="L131" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.27.md</t>
         </is>
       </c>
     </row>
@@ -8919,6 +9188,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L125" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L126" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L127" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L128" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L129" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L130" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L131" r:id="rId126"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8932,7 +9205,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId123"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId127"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record travel screening delivery and enterprise trial backlog
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,11 +14,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$32</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$131</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$136</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'使用与维护'!$A$5:$B$17</definedName>
   </definedNames>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H31" headerRowCount="1">
-  <autoFilter ref="A5:H31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H32" headerRowCount="1">
+  <autoFilter ref="A5:H32"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L131" headerRowCount="1">
-  <autoFilter ref="A5:L131"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L136" headerRowCount="1">
+  <autoFilter ref="A5:L136"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -264,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H11" headerRowCount="1">
-  <autoFilter ref="A5:H11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H12" headerRowCount="1">
+  <autoFilter ref="A5:H12"/>
   <tableColumns count="8">
     <tableColumn id="1" name="顺序"/>
     <tableColumn id="2" name="优先级"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 26 个阶段、126 项内容  |  当前功能版本 v0.27  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 27 个阶段、131 项内容  |  当前功能版本 v0.28  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1590,6 +1590,42 @@
       <c r="H31" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/2dfe512</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="74" customHeight="1">
+      <c r="A32" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>v0.28</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>城市与人员职级差旅规则预审</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>168项业务测试、131项浏览器场景整套通过；生产同构住宿1100对500×2超100被拦、同日交通合并、退回修正并四岗模拟付款1390、处理快照和备份通过；全程不依赖OCR</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/34d80e9</t>
         </is>
       </c>
     </row>
@@ -1626,6 +1662,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId27"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1639,7 +1676,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1651,7 +1688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9056,6 +9093,296 @@
       <c r="L131" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.27.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="88" customHeight="1">
+      <c r="A132" s="5" t="n">
+        <v>127</v>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>v0.28</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D132" s="5" t="inlineStr">
+        <is>
+          <t>差旅制度配置</t>
+        </is>
+      </c>
+      <c r="E132" s="5" t="inlineStr">
+        <is>
+          <t>财务维护城市目录、城市档/职级矩阵、单城市特例、人员ID职级及5类提醒/拦截</t>
+        </is>
+      </c>
+      <c r="F132" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G132" s="5" t="inlineStr">
+        <is>
+          <t>把企业差旅制度转成可执行且可解释的标准</t>
+        </is>
+      </c>
+      <c r="H132" s="5" t="inlineStr">
+        <is>
+          <t>财务→差旅标准→发布</t>
+        </is>
+      </c>
+      <c r="I132" s="5" t="inlineStr">
+        <is>
+          <t>普通与管理档、上海与南京及上海独立标准分别匹配，员工不能自行选高档</t>
+        </is>
+      </c>
+      <c r="J132" s="5" t="inlineStr">
+        <is>
+          <t>168项业务测试、131项浏览器场景整套通过；生产同构住宿1100对500×2超100被拦、同日交通合并、退回修正并四岗模拟付款1390、处理快照和备份通过；全程不依赖OCR</t>
+        </is>
+      </c>
+      <c r="K132" s="5" t="inlineStr">
+        <is>
+          <t>两档城市/两档职级加城市特例；未接HR或后端权限</t>
+        </is>
+      </c>
+      <c r="L132" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.28.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="88" customHeight="1">
+      <c r="A133" s="5" t="n">
+        <v>128</v>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>v0.28</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>差旅费用预审</t>
+        </is>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>住宿/餐补计算、同日市内交通合并、缺酒店水单及未关联事前申请提示</t>
+        </is>
+      </c>
+      <c r="F133" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G133" s="5" t="inlineStr">
+        <is>
+          <t>减少重复查标准及计算额度，向财务集中提供风险依据</t>
+        </is>
+      </c>
+      <c r="H133" s="5" t="inlineStr">
+        <is>
+          <t>差旅报销明细 / 预审详情 / 审批中心</t>
+        </is>
+      </c>
+      <c r="I133" s="5" t="inlineStr">
+        <is>
+          <t>1100住宿对500×2显示100超额；50+40交通合并对80显示10超额；缺材料提示</t>
+        </is>
+      </c>
+      <c r="J133" s="5" t="inlineStr">
+        <is>
+          <t>168项业务测试、131项浏览器场景整套通过；生产同构住宿1100对500×2超100被拦、同日交通合并、退回修正并四岗模拟付款1390、处理快照和备份通过；全程不依赖OCR</t>
+        </is>
+      </c>
+      <c r="K133" s="5" t="inlineStr">
+        <is>
+          <t>未自动批准；水单只检查分类及留存，不读取真实入住内容</t>
+        </is>
+      </c>
+      <c r="L133" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.28.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="88" customHeight="1">
+      <c r="A134" s="5" t="n">
+        <v>129</v>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>v0.28</t>
+        </is>
+      </c>
+      <c r="C134" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D134" s="5" t="inlineStr">
+        <is>
+          <t>差旅标准快照</t>
+        </is>
+      </c>
+      <c r="E134" s="5" t="inlineStr">
+        <is>
+          <t>提交时标准/人员快照、处理时风险记录、在途不追改及退回重提新标准</t>
+        </is>
+      </c>
+      <c r="F134" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G134" s="5" t="inlineStr">
+        <is>
+          <t>制度变更后仍能复核原审核依据，例外路径明确</t>
+        </is>
+      </c>
+      <c r="H134" s="5" t="inlineStr">
+        <is>
+          <t>报销详情 / 处理时预审快照 / 退回修改</t>
+        </is>
+      </c>
+      <c r="I134" s="5" t="inlineStr">
+        <is>
+          <t>提高新制度不清除在途原拦截，退回重提捕获新标准，保留旧风险记录</t>
+        </is>
+      </c>
+      <c r="J134" s="5" t="inlineStr">
+        <is>
+          <t>168项业务测试、131项浏览器场景整套通过；生产同构住宿1100对500×2超100被拦、同日交通合并、退回修正并四岗模拟付款1390、处理快照和备份通过；全程不依赖OCR</t>
+        </is>
+      </c>
+      <c r="K134" s="5" t="inlineStr">
+        <is>
+          <t>无自动豁免和生效排程；旧无快照单保持原示例并提醒人工核实</t>
+        </is>
+      </c>
+      <c r="L134" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.28.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="88" customHeight="1">
+      <c r="A135" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>v0.28</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>差旅数据保护</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>制度配额失败/未发布切换保护、坏配置及快照提示、新旧备份校验</t>
+        </is>
+      </c>
+      <c r="F135" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G135" s="5" t="inlineStr">
+        <is>
+          <t>避免不完整数据被误当通过，配置和业务恢复可核对</t>
+        </is>
+      </c>
+      <c r="H135" s="5" t="inlineStr">
+        <is>
+          <t>差旅制度发布 / 数据管理 / 异常详情</t>
+        </is>
+      </c>
+      <c r="I135" s="5" t="inlineStr">
+        <is>
+          <t>写入失败保持原制度和输入，旧备份缺新制度时保留当前，非法快照拒绝恢复</t>
+        </is>
+      </c>
+      <c r="J135" s="5" t="inlineStr">
+        <is>
+          <t>168项业务测试、131项浏览器场景整套通过；生产同构住宿1100对500×2超100被拦、同日交通合并、退回修正并四岗模拟付款1390、处理快照和备份通过；全程不依赖OCR</t>
+        </is>
+      </c>
+      <c r="K135" s="5" t="inlineStr">
+        <is>
+          <t>仍为单浏览器原型，日志无防篡改和生产灾备保障</t>
+        </is>
+      </c>
+      <c r="L135" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.28.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="88" customHeight="1">
+      <c r="A136" s="5" t="n">
+        <v>131</v>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>v0.28</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D136" s="5" t="inlineStr">
+        <is>
+          <t>产品取舍与演示</t>
+        </is>
+      </c>
+      <c r="E136" s="5" t="inlineStr">
+        <is>
+          <t>暂停通用OCR扩展，补充差旅规则演示、设计复盘和Excel记录</t>
+        </is>
+      </c>
+      <c r="F136" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G136" s="5" t="inlineStr">
+        <is>
+          <t>围绕财务重复核算验证价值，避免把不稳定识别作为面试前提</t>
+        </is>
+      </c>
+      <c r="H136" s="5" t="inlineStr">
+        <is>
+          <t>差旅规则说明 / 面试案例 / 功能Excel / 演示ZIP</t>
+        </is>
+      </c>
+      <c r="I136" s="5" t="inlineStr">
+        <is>
+          <t>使用虚构附件和手工明细完成规则拦截、退回修正、总账及模拟付款</t>
+        </is>
+      </c>
+      <c r="J136" s="5" t="inlineStr">
+        <is>
+          <t>168项业务测试、131项浏览器场景整套通过；生产同构住宿1100对500×2超100被拦、同日交通合并、退回修正并四岗模拟付款1390、处理快照和备份通过；全程不依赖OCR</t>
+        </is>
+      </c>
+      <c r="K136" s="5" t="inlineStr">
+        <is>
+          <t>自动化不证明真实企业工时下降，需后续试点记录耗时、补材料次数及误报</t>
+        </is>
+      </c>
+      <c r="L136" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.28.md</t>
         </is>
       </c>
     </row>
@@ -9192,6 +9519,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L129" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L130" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L131" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L132" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L133" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L134" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L135" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L136" r:id="rId131"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9205,7 +9537,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId127"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId132"/>
   </tableParts>
 </worksheet>
 </file>
@@ -9217,7 +9549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9514,7 +9846,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>逐项核对留痕已交付，但仍为统一固定规则目录，无组织制度适用范围</t>
+          <t>已交付逐项核对及差旅城市/人员职级制度，尚无按组织部门的通用制度适用范围或豁免机制</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -9529,7 +9861,47 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>v0.25已完成逐项核对与依据失效；组织适用和豁免机制尚未实现</t>
+          <t>v0.25完成逐项核对、v0.28完成差旅城市职级制度；通用组织适用与豁免尚未实现</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="100" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>企业试点前的多人协作与权限基础</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>待设计与实施</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>用户希望真实企业试用，当前本地浏览器数据和模拟身份不足以正式给200人公司使用</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>先明确试点企业需求，再设计服务端数据、真实身份与范围权限、并发事务、文件授权及备份恢复</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>跨账号跨设备完成受权限保护的同一笔报销，重复请求不重复审批/占用，恢复演练和小范围虚构数据验收通过后再规划真实试点</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>新账号权限、费用或真实财务资料必须按既有授权边界单独确认；本轮仅完成差旅规则，无正式企业上线承诺</t>
         </is>
       </c>
     </row>
@@ -9731,7 +10103,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.26完成部门月度预算、新增占用硬控/核销不重扣、贡献明细、备份保护及面试准备手册；已可做个人原型演示，不代表生产落地或真实收益。</t>
+          <t>v0.28完成城市/人员职级差旅制度、透明预审、提交与处理快照、异常恢复和不依赖OCR的演示；企业多人权限仍待实施，不代表生产落地或真实收益。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record R001 v1 delivery and test evidence in feature history
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$33</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$136</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$142</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H32" headerRowCount="1">
-  <autoFilter ref="A5:H32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H33" headerRowCount="1">
+  <autoFilter ref="A5:H33"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L136" headerRowCount="1">
-  <autoFilter ref="A5:L136"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L142" headerRowCount="1">
+  <autoFilter ref="A5:L142"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 27 个阶段、131 项内容  |  当前功能版本 v0.28  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 28 个阶段、137 项内容  |  当前功能版本 R001 v1  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1626,6 +1626,42 @@
       <c r="H32" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/34d80e9</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="74" customHeight="1">
+      <c r="A33" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>R001 v1</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>独立住宿费超标审核R001 v1</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>R001严格类型检查、22项规则/数据测试（含T01–T10）、11项浏览器场景通过；整套190项业务/142项浏览器回归通过，最终R00122/11再次通过；生产独立HTML验证T03人工通过、T05驳回、新旧标准快照及手机布局</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/3797ed1</t>
         </is>
       </c>
     </row>
@@ -1663,6 +1699,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId28"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1676,7 +1713,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1688,7 +1725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L136"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9383,6 +9420,354 @@
       <c r="L136" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/阶段验收-v0.28.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="88" customHeight="1">
+      <c r="A137" s="5" t="n">
+        <v>132</v>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>R001 v1</t>
+        </is>
+      </c>
+      <c r="C137" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>R001独立录入</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>独立四页面入口、自动单号、三档职级/可输入未知城市、自动住宿晚数</t>
+        </is>
+      </c>
+      <c r="F137" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G137" s="5" t="inlineStr">
+        <is>
+          <t>以限定规则范围展示完整产品交互，沿用现有Vite而不重构其他业务</t>
+        </is>
+      </c>
+      <c r="H137" s="5" t="inlineStr">
+        <is>
+          <t>r001.html→住宿报销单录入</t>
+        </is>
+      </c>
+      <c r="I137" s="5" t="inlineStr">
+        <is>
+          <t>载入T03虚构示例，深圳普通员工3晚1800元，自动计算晚数并执行审核</t>
+        </is>
+      </c>
+      <c r="J137" s="5" t="inlineStr">
+        <is>
+          <t>R001严格类型检查、22项规则/数据测试（含T01–T10）、11项浏览器场景通过；整套190项业务/142项浏览器回归通过，最终R00122/11再次通过；生产独立HTML验证T03人工通过、T05驳回、新旧标准快照及手机布局</t>
+        </is>
+      </c>
+      <c r="K137" s="5" t="inlineStr">
+        <is>
+          <t>仅R001，境内人民币单城市连续住宿；模拟身份，无后端</t>
+        </is>
+      </c>
+      <c r="L137" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R001-v1验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="88" customHeight="1">
+      <c r="A138" s="5" t="n">
+        <v>133</v>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>R001 v1</t>
+        </is>
+      </c>
+      <c r="C138" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D138" s="5" t="inlineStr">
+        <is>
+          <t>R001纯审核规则</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t>独立TypeScript纯函数、分离模拟制度、整数分和公历日期计算</t>
+        </is>
+      </c>
+      <c r="F138" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G138" s="5" t="inlineStr">
+        <is>
+          <t>明确限额、超额及错误边界，结果可复算</t>
+        </is>
+      </c>
+      <c r="H138" s="5" t="inlineStr">
+        <is>
+          <t>src/r001/rule.ts / standards.ts / 自动审核结果</t>
+        </is>
+      </c>
+      <c r="I138" s="5" t="inlineStr">
+        <is>
+          <t>T01–T10验证相等/超标/缺标准/零晚/负数，0.31对0.30仅超1分</t>
+        </is>
+      </c>
+      <c r="J138" s="5" t="inlineStr">
+        <is>
+          <t>R001严格类型检查、22项规则/数据测试（含T01–T10）、11项浏览器场景通过；整套190项业务/142项浏览器回归通过，最终R00122/11再次通过；生产独立HTML验证T03人工通过、T05驳回、新旧标准快照及手机布局</t>
+        </is>
+      </c>
+      <c r="K138" s="5" t="inlineStr">
+        <is>
+          <t>只通过住宿金额本项，不验真、不执行整单审批或付款</t>
+        </is>
+      </c>
+      <c r="L138" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R001-v1验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="88" customHeight="1">
+      <c r="A139" s="5" t="n">
+        <v>134</v>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>R001 v1</t>
+        </is>
+      </c>
+      <c r="C139" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>R001人工复核</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>人工通过/驳回均必须填写原因，记录时间且保留原始自动结论</t>
+        </is>
+      </c>
+      <c r="F139" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="inlineStr">
+        <is>
+          <t>让系统提示与财务判断分开，历史结果不会覆盖</t>
+        </is>
+      </c>
+      <c r="H139" s="5" t="inlineStr">
+        <is>
+          <t>人工复核 / 自动审核结果</t>
+        </is>
+      </c>
+      <c r="I139" s="5" t="inlineStr">
+        <is>
+          <t>T03超300元可人工通过，T05超100元可人工驳回，两者原因/时间与原始结果可查看</t>
+        </is>
+      </c>
+      <c r="J139" s="5" t="inlineStr">
+        <is>
+          <t>R001严格类型检查、22项规则/数据测试（含T01–T10）、11项浏览器场景通过；整套190项业务/142项浏览器回归通过，最终R00122/11再次通过；生产独立HTML验证T03人工通过、T05驳回、新旧标准快照及手机布局</t>
+        </is>
+      </c>
+      <c r="K139" s="5" t="inlineStr">
+        <is>
+          <t>一次复核完成不重复改写；仅模拟财务身份，无生产权限或防篡改审计</t>
+        </is>
+      </c>
+      <c r="L139" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R001-v1验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="88" customHeight="1">
+      <c r="A140" s="5" t="n">
+        <v>135</v>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>R001 v1</t>
+        </is>
+      </c>
+      <c r="C140" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D140" s="5" t="inlineStr">
+        <is>
+          <t>R001标准快照</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>15条模拟标准、增加/修改与版本更新、历史匹配或缺失事实留存</t>
+        </is>
+      </c>
+      <c r="F140" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G140" s="5" t="inlineStr">
+        <is>
+          <t>修改新制度不悄悄重算旧单，支持清晰解释历史依据</t>
+        </is>
+      </c>
+      <c r="H140" s="5" t="inlineStr">
+        <is>
+          <t>模拟住宿标准 / 历史审核单据</t>
+        </is>
+      </c>
+      <c r="I140" s="5" t="inlineStr">
+        <is>
+          <t>深圳500改700，旧单限额1500超300不变，复制新单限额2100通过；新增城市也不补造旧标准</t>
+        </is>
+      </c>
+      <c r="J140" s="5" t="inlineStr">
+        <is>
+          <t>R001严格类型检查、22项规则/数据测试（含T01–T10）、11项浏览器场景通过；整套190项业务/142项浏览器回归通过，最终R00122/11再次通过；生产独立HTML验证T03人工通过、T05驳回、新旧标准快照及手机布局</t>
+        </is>
+      </c>
+      <c r="K140" s="5" t="inlineStr">
+        <is>
+          <t>单规则标准目录，管理者应仅录入境内模拟城市，不接公司制度系统</t>
+        </is>
+      </c>
+      <c r="L140" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R001-v1验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="88" customHeight="1">
+      <c r="A141" s="5" t="n">
+        <v>136</v>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>R001 v1</t>
+        </is>
+      </c>
+      <c r="C141" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>R001本地数据保护</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>独立存储键、恢复模拟数据、失败保留和已发生的页面冲突检测</t>
+        </is>
+      </c>
+      <c r="F141" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G141" s="5" t="inlineStr">
+        <is>
+          <t>保存失败不丢填写，恢复仅影响R001且不删除其他轻报数据</t>
+        </is>
+      </c>
+      <c r="H141" s="5" t="inlineStr">
+        <is>
+          <t>恢复R001模拟数据 / 保存失败提示</t>
+        </is>
+      </c>
+      <c r="I141" s="5" t="inlineStr">
+        <is>
+          <t>注入配额失败、坏JSON和旧页写入冲突，验证原值保留及恢复隔离</t>
+        </is>
+      </c>
+      <c r="J141" s="5" t="inlineStr">
+        <is>
+          <t>R001严格类型检查、22项规则/数据测试（含T01–T10）、11项浏览器场景通过；整套190项业务/142项浏览器回归通过，最终R00122/11再次通过；生产独立HTML验证T03人工通过、T05驳回、新旧标准快照及手机布局</t>
+        </is>
+      </c>
+      <c r="K141" s="5" t="inlineStr">
+        <is>
+          <t>200记录/300标准/约150万字符；本地冲突检测不是服务端原子事务</t>
+        </is>
+      </c>
+      <c r="L141" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R001-v1验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="88" customHeight="1">
+      <c r="A142" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>R001 v1</t>
+        </is>
+      </c>
+      <c r="C142" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D142" s="5" t="inlineStr">
+        <is>
+          <t>R001交付与验证</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>README启动/T03流程、CHANGELOG v1、独立HTML构建和真实测试记录</t>
+        </is>
+      </c>
+      <c r="F142" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G142" s="5" t="inlineStr">
+        <is>
+          <t>交付可运行、可复现、有边界的单规则作品</t>
+        </is>
+      </c>
+      <c r="H142" s="5" t="inlineStr">
+        <is>
+          <t>README / CHANGELOG / docs/R001-v1验收 / r001独立网页</t>
+        </is>
+      </c>
+      <c r="I142" s="5" t="inlineStr">
+        <is>
+          <t>本地HTTP启动并验证生产独立页面，四页手机和旧轻报首页通过，只有同源GET</t>
+        </is>
+      </c>
+      <c r="J142" s="5" t="inlineStr">
+        <is>
+          <t>R001严格类型检查、22项规则/数据测试（含T01–T10）、11项浏览器场景通过；整套190项业务/142项浏览器回归通过，最终R00122/11再次通过；生产独立HTML验证T03人工通过、T05驳回、新旧标准快照及手机布局</t>
+        </is>
+      </c>
+      <c r="K142" s="5" t="inlineStr">
+        <is>
+          <t>自动化不证明真实企业收益；未扩展其他费用模块，不依赖OCR</t>
+        </is>
+      </c>
+      <c r="L142" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R001-v1验收.md</t>
         </is>
       </c>
     </row>
@@ -9524,6 +9909,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L134" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L135" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L136" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L137" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L138" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L139" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L140" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L141" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L142" r:id="rId137"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9537,7 +9928,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId132"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId138"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10103,7 +10494,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v0.28完成城市/人员职级差旅制度、透明预审、提交与处理快照、异常恢复和不依赖OCR的演示；企业多人权限仍待实施，不代表生产落地或真实收益。</t>
+          <t>R001 v1仅交付独立住宿费审核、15条城市职级制度、整数分/日历、原始结果与独立人工复核及历史标准快照；不扩展其他业务，无真实企业收益或生产鉴权。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record R002 delivery and refresh feature history workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$142</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$148</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H33" headerRowCount="1">
-  <autoFilter ref="A5:H33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H34" headerRowCount="1">
+  <autoFilter ref="A5:H34"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L142" headerRowCount="1">
-  <autoFilter ref="A5:L142"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L148" headerRowCount="1">
+  <autoFilter ref="A5:L148"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 28 个阶段、137 项内容  |  当前功能版本 R001 v1  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-24  |  已交付 29 个阶段、143 项内容  |  当前功能版本 v2 / R002 v1  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1662,6 +1662,42 @@
       <c r="H33" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/3797ed1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="74" customHeight="1">
+      <c r="A34" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>v2 / R002 v1</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>发票重复报销审核R002及证据版本</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>基线190业务/142浏览器；最终225业务/154浏览器通过，含R00235项T01–T30及12项浏览器、原R00122/11；生产独立HTML T02驳回/重审证据/恢复隔离及390px四页通过</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/a059d16</t>
         </is>
       </c>
     </row>
@@ -1700,6 +1736,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId29"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1713,7 +1750,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1725,7 +1762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -9768,6 +9805,354 @@
       <c r="L142" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/R001-v1验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="88" customHeight="1">
+      <c r="A143" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>v2 / R002 v1</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>R002票面采集</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>单票单单字段、五种发票类型、长号码字符串与整数分金额</t>
+        </is>
+      </c>
+      <c r="F143" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="inlineStr">
+        <is>
+          <t>减少发票标识与金额录入丢失，清楚说明错误</t>
+        </is>
+      </c>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>R002 → 发票报销单录入</t>
+        </is>
+      </c>
+      <c r="I143" s="5" t="inlineStr">
+        <is>
+          <t>载入T02；用20位含前导零及100.01/100.001比较</t>
+        </is>
+      </c>
+      <c r="J143" s="5" t="inlineStr">
+        <is>
+          <t>基线190业务/142浏览器；最终225业务/154浏览器通过，含R00235项T01–T30及12项浏览器、原R00122/11；生产独立HTML T02驳回/重审证据/恢复隔离及390px四页通过</t>
+        </is>
+      </c>
+      <c r="K143" s="5" t="inlineStr">
+        <is>
+          <t>无OCR/税务真实性或官方格式认证</t>
+        </is>
+      </c>
+      <c r="L143" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R002-v2验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="88" customHeight="1">
+      <c r="A144" s="5" t="n">
+        <v>139</v>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>v2 / R002 v1</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D144" s="5" t="inlineStr">
+        <is>
+          <t>R002查重规则</t>
+        </is>
+      </c>
+      <c r="E144" s="5" t="inlineStr">
+        <is>
+          <t>代码＋号码/无代码数电号码查重、跨类型潜在冲突及四状态解释</t>
+        </is>
+      </c>
+      <c r="F144" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G144" s="5" t="inlineStr">
+        <is>
+          <t>区分票面重复与潜在冲突，避免只按金额或驳回直接放行</t>
+        </is>
+      </c>
+      <c r="H144" s="5" t="inlineStr">
+        <is>
+          <t>R002 → 自动审核结果</t>
+        </is>
+      </c>
+      <c r="I144" s="5" t="inlineStr">
+        <is>
+          <t>T02命中BX-H001；同号不同代码与类型比较</t>
+        </is>
+      </c>
+      <c r="J144" s="5" t="inlineStr">
+        <is>
+          <t>基线190业务/142浏览器；最终225业务/154浏览器通过，含R00235项T01–T30及12项浏览器、原R00122/11；生产独立HTML T02驳回/重审证据/恢复隔离及390px四页通过</t>
+        </is>
+      </c>
+      <c r="K144" s="5" t="inlineStr">
+        <is>
+          <t>只查本地R002库及有效单据，非全局判重或违规认定</t>
+        </is>
+      </c>
+      <c r="L144" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R002-v2验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="88" customHeight="1">
+      <c r="A145" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>v2 / R002 v1</t>
+        </is>
+      </c>
+      <c r="C145" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>R002复核与版本</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>独立人工通过/驳回、复核人原因时间、版本及原始证据保留</t>
+        </is>
+      </c>
+      <c r="F145" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G145" s="5" t="inlineStr">
+        <is>
+          <t>让财务人工判断可追溯，不覆盖自动规则</t>
+        </is>
+      </c>
+      <c r="H145" s="5" t="inlineStr">
+        <is>
+          <t>R002 → 人工复核 / 审核版本选择</t>
+        </is>
+      </c>
+      <c r="I145" s="5" t="inlineStr">
+        <is>
+          <t>T02填写周宁及原因驳回；重审后查看旧版</t>
+        </is>
+      </c>
+      <c r="J145" s="5" t="inlineStr">
+        <is>
+          <t>基线190业务/142浏览器；最终225业务/154浏览器通过，含R00235项T01–T30及12项浏览器、原R00122/11；生产独立HTML T02驳回/重审证据/恢复隔离及390px四页通过</t>
+        </is>
+      </c>
+      <c r="K145" s="5" t="inlineStr">
+        <is>
+          <t>最新待复核可操作；一版本一次，模拟人员无生产鉴权</t>
+        </is>
+      </c>
+      <c r="L145" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R002-v2验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="88" customHeight="1">
+      <c r="A146" s="5" t="n">
+        <v>141</v>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>v2 / R002 v1</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D146" s="5" t="inlineStr">
+        <is>
+          <t>R002模拟发票库</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>五笔种子、号码单号搜索/状态筛选、新增编辑及确认恢复</t>
+        </is>
+      </c>
+      <c r="F146" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G146" s="5" t="inlineStr">
+        <is>
+          <t>提供可维护可复现查重资料，不重置已审核证据</t>
+        </is>
+      </c>
+      <c r="H146" s="5" t="inlineStr">
+        <is>
+          <t>R002 → 模拟历史发票库</t>
+        </is>
+      </c>
+      <c r="I146" s="5" t="inlineStr">
+        <is>
+          <t>改BX-H001代码再审，新版本更新旧证据不变；恢复后保留R001/R002</t>
+        </is>
+      </c>
+      <c r="J146" s="5" t="inlineStr">
+        <is>
+          <t>基线190业务/142浏览器；最终225业务/154浏览器通过，含R00235项T01–T30及12项浏览器、原R00122/11；生产独立HTML T02驳回/重审证据/恢复隔离及390px四页通过</t>
+        </is>
+      </c>
+      <c r="K146" s="5" t="inlineStr">
+        <is>
+          <t>库编辑是模拟操作；恢复只替换历史库</t>
+        </is>
+      </c>
+      <c r="L146" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R002-v2验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="88" customHeight="1">
+      <c r="A147" s="5" t="n">
+        <v>142</v>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>v2 / R002 v1</t>
+        </is>
+      </c>
+      <c r="C147" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>R002数据完整性</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>保存前本地再查重、排除自身、保留最近有效票面、冲突配额失败保护</t>
+        </is>
+      </c>
+      <c r="F147" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G147" s="5" t="inlineStr">
+        <is>
+          <t>防止旧页覆盖、数据错误洗掉有效发票或误把自己判为重复</t>
+        </is>
+      </c>
+      <c r="H147" s="5" t="inlineStr">
+        <is>
+          <t>R002 → 重审 / 模拟历史发票库</t>
+        </is>
+      </c>
+      <c r="I147" s="5" t="inlineStr">
+        <is>
+          <t>重审产生v2，旧结论仍可看；错误资料后有效v1仍入库</t>
+        </is>
+      </c>
+      <c r="J147" s="5" t="inlineStr">
+        <is>
+          <t>基线190业务/142浏览器；最终225业务/154浏览器通过，含R00235项T01–T30及12项浏览器、原R00122/11；生产独立HTML T02驳回/重审证据/恢复隔离及390px四页通过</t>
+        </is>
+      </c>
+      <c r="K147" s="5" t="inlineStr">
+        <is>
+          <t>同单可靠票面绑定，更换票新建；没有服务端原子事务</t>
+        </is>
+      </c>
+      <c r="L147" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R002-v2验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="88" customHeight="1">
+      <c r="A148" s="5" t="n">
+        <v>143</v>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>v2 / R002 v1</t>
+        </is>
+      </c>
+      <c r="C148" s="6" t="n">
+        <v>46319</v>
+      </c>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t>R002交付与验证</t>
+        </is>
+      </c>
+      <c r="E148" s="5" t="inlineStr">
+        <is>
+          <t>三入口独立HTML、R001互链共享复核、v2文档演示复盘和真实自动测试</t>
+        </is>
+      </c>
+      <c r="F148" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G148" s="5" t="inlineStr">
+        <is>
+          <t>交付可运行可解释且兼容原规则的财务作品</t>
+        </is>
+      </c>
+      <c r="H148" s="5" t="inlineStr">
+        <is>
+          <t>README / CHANGELOG / R002验收 / r002.html</t>
+        </is>
+      </c>
+      <c r="I148" s="5" t="inlineStr">
+        <is>
+          <t>在线T02完整驳回，R001 T03超300回归及手机四页</t>
+        </is>
+      </c>
+      <c r="J148" s="5" t="inlineStr">
+        <is>
+          <t>基线190业务/142浏览器；最终225业务/154浏览器通过，含R00235项T01–T30及12项浏览器、原R00122/11；生产独立HTML T02驳回/重审证据/恢复隔离及390px四页通过</t>
+        </is>
+      </c>
+      <c r="K148" s="5" t="inlineStr">
+        <is>
+          <t>不扩展R003或其他模块；没有真实企业提效数据</t>
+        </is>
+      </c>
+      <c r="L148" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R002-v2验收.md</t>
         </is>
       </c>
     </row>
@@ -9915,6 +10300,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L140" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L141" r:id="rId136"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L142" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L143" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L144" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L145" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L146" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L147" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L148" r:id="rId143"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9928,7 +10319,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId138"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId144"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10494,7 +10885,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>R001 v1仅交付独立住宿费审核、15条城市职级制度、整数分/日历、原始结果与独立人工复核及历史标准快照；不扩展其他业务，无真实企业收益或生产鉴权。</t>
+          <t>v2 / R002 v1只新增发票重复风险审核、模拟历史库、独立人工复核及版本证据；保留R001判断和数据。225项业务/154项浏览器通过，不代表跨用户查重、税务验真或真实企业收益。</t>
         </is>
       </c>
     </row>
@@ -10506,7 +10897,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/?v=0.26</t>
+          <t>https://jameyan42.github.io/-/r002.html（R002）；同目录r001.html保留住宿审核，根地址为原轻报。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track R003 delivery in feature history workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$35</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$148</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$154</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H34" headerRowCount="1">
-  <autoFilter ref="A5:H34"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H35" headerRowCount="1">
+  <autoFilter ref="A5:H35"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L148" headerRowCount="1">
-  <autoFilter ref="A5:L148"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L154" headerRowCount="1">
+  <autoFilter ref="A5:L154"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-24  |  已交付 29 个阶段、143 项内容  |  当前功能版本 v2 / R002 v1  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-25  |  已交付 30 个阶段、149 项内容  |  当前功能版本 v3 / R003 v1  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1698,6 +1698,42 @@
       <c r="H34" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/a059d16</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="74" customHeight="1">
+      <c r="A35" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>v3 / R003 v1</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>合同付款条件审核与资金占用分离</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>259项业务/157项浏览器全部通过，R00334项含T01–T30、3项页面流程；生产独立HTML T04驳回/刷新保留、手机四区和R002互链通过；基线12项服务连接失败重启后全通过</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/16d1735</t>
         </is>
       </c>
     </row>
@@ -1737,6 +1773,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId30"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1750,7 +1787,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1762,7 +1799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L148"/>
+  <dimension ref="A1:L154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10153,6 +10190,354 @@
       <c r="L148" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/R002-v2验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="88" customHeight="1">
+      <c r="A149" s="5" t="n">
+        <v>144</v>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>v3 / R003 v1</t>
+        </is>
+      </c>
+      <c r="C149" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>R003结构化合同</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>三种付款模式、四模拟合同和独立付款历史</t>
+        </is>
+      </c>
+      <c r="F149" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G149" s="5" t="inlineStr">
+        <is>
+          <t>将总额、阶段及结算条件配置化</t>
+        </is>
+      </c>
+      <c r="H149" s="5" t="inlineStr">
+        <is>
+          <t>R003 → 数据管理</t>
+        </is>
+      </c>
+      <c r="I149" s="5" t="inlineStr">
+        <is>
+          <t>查看HT-001至004与30/40/30阶段</t>
+        </is>
+      </c>
+      <c r="J149" s="5" t="inlineStr">
+        <is>
+          <t>259项业务/157项浏览器全部通过，R00334项含T01–T30、3项页面流程；生产独立HTML T04驳回/刷新保留、手机四区和R002互链通过；基线12项服务连接失败重启后全通过</t>
+        </is>
+      </c>
+      <c r="K149" s="5" t="inlineStr">
+        <is>
+          <t>不审合同合法性</t>
+        </is>
+      </c>
+      <c r="L149" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R003-v3验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="88" customHeight="1">
+      <c r="A150" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
+        <is>
+          <t>v3 / R003 v1</t>
+        </is>
+      </c>
+      <c r="C150" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D150" s="5" t="inlineStr">
+        <is>
+          <t>R003自动控制</t>
+        </is>
+      </c>
+      <c r="E150" s="5" t="inlineStr">
+        <is>
+          <t>R003-01至09多风险、整数分基点及尾差</t>
+        </is>
+      </c>
+      <c r="F150" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G150" s="5" t="inlineStr">
+        <is>
+          <t>减少重复计算，区分资料错误与付款风险</t>
+        </is>
+      </c>
+      <c r="H150" s="5" t="inlineStr">
+        <is>
+          <t>R003 → 录入 / 自动结果</t>
+        </is>
+      </c>
+      <c r="I150" s="5" t="inlineStr">
+        <is>
+          <t>T04第二阶段35000超5000及缺证据多风险</t>
+        </is>
+      </c>
+      <c r="J150" s="5" t="inlineStr">
+        <is>
+          <t>259项业务/157项浏览器全部通过，R00334项含T01–T30、3项页面流程；生产独立HTML T04驳回/刷新保留、手机四区和R002互链通过；基线12项服务连接失败重启后全通过</t>
+        </is>
+      </c>
+      <c r="K150" s="5" t="inlineStr">
+        <is>
+          <t>无跨账号占用事务</t>
+        </is>
+      </c>
+      <c r="L150" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R003-v3验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="88" customHeight="1">
+      <c r="A151" s="5" t="n">
+        <v>146</v>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>v3 / R003 v1</t>
+        </is>
+      </c>
+      <c r="C151" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>R003付款事实与占用</t>
+        </is>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>已支付/待支付分离、合同阶段结算占用及本单排除</t>
+        </is>
+      </c>
+      <c r="F151" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G151" s="5" t="inlineStr">
+        <is>
+          <t>不将待支付当实际支付，识别潜在超额</t>
+        </is>
+      </c>
+      <c r="H151" s="5" t="inlineStr">
+        <is>
+          <t>R003 → 结果计算与历史付款</t>
+        </is>
+      </c>
+      <c r="I151" s="5" t="inlineStr">
+        <is>
+          <t>T16/T17/T27对照已付与待支付</t>
+        </is>
+      </c>
+      <c r="J151" s="5" t="inlineStr">
+        <is>
+          <t>259项业务/157项浏览器全部通过，R00334项含T01–T30、3项页面流程；生产独立HTML T04驳回/刷新保留、手机四区和R002互链通过；基线12项服务连接失败重启后全通过</t>
+        </is>
+      </c>
+      <c r="K151" s="5" t="inlineStr">
+        <is>
+          <t>审核不自动创建资金流水</t>
+        </is>
+      </c>
+      <c r="L151" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R003-v3验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="88" customHeight="1">
+      <c r="A152" s="5" t="n">
+        <v>147</v>
+      </c>
+      <c r="B152" s="5" t="inlineStr">
+        <is>
+          <t>v3 / R003 v1</t>
+        </is>
+      </c>
+      <c r="C152" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D152" s="5" t="inlineStr">
+        <is>
+          <t>R003版本及人工</t>
+        </is>
+      </c>
+      <c r="E152" s="5" t="inlineStr">
+        <is>
+          <t>同单版本快照、独立人工通过驳回与原结果保留</t>
+        </is>
+      </c>
+      <c r="F152" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G152" s="5" t="inlineStr">
+        <is>
+          <t>保留当时条件和例外判断依据</t>
+        </is>
+      </c>
+      <c r="H152" s="5" t="inlineStr">
+        <is>
+          <t>R003 → 人工复核 / 版本选择</t>
+        </is>
+      </c>
+      <c r="I152" s="5" t="inlineStr">
+        <is>
+          <t>T04驳回，变更证据后重审并查看旧版本</t>
+        </is>
+      </c>
+      <c r="J152" s="5" t="inlineStr">
+        <is>
+          <t>259项业务/157项浏览器全部通过，R00334项含T01–T30、3项页面流程；生产独立HTML T04驳回/刷新保留、手机四区和R002互链通过；基线12项服务连接失败重启后全通过</t>
+        </is>
+      </c>
+      <c r="K152" s="5" t="inlineStr">
+        <is>
+          <t>模拟人员无生产鉴权</t>
+        </is>
+      </c>
+      <c r="L152" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R003-v3验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="88" customHeight="1">
+      <c r="A153" s="5" t="n">
+        <v>148</v>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>v3 / R003 v1</t>
+        </is>
+      </c>
+      <c r="C153" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>R003管理与安全</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>合同付款新增修改、确认恢复、独立键与失败保护</t>
+        </is>
+      </c>
+      <c r="F153" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G153" s="5" t="inlineStr">
+        <is>
+          <t>可维护模拟环境而不删除审核历史及R001/R002</t>
+        </is>
+      </c>
+      <c r="H153" s="5" t="inlineStr">
+        <is>
+          <t>R003 → 模拟合同与付款数据</t>
+        </is>
+      </c>
+      <c r="I153" s="5" t="inlineStr">
+        <is>
+          <t>改交付证据；恢复后历史版本不变</t>
+        </is>
+      </c>
+      <c r="J153" s="5" t="inlineStr">
+        <is>
+          <t>259项业务/157项浏览器全部通过，R00334项含T01–T30、3项页面流程；生产独立HTML T04驳回/刷新保留、手机四区和R002互链通过；基线12项服务连接失败重启后全通过</t>
+        </is>
+      </c>
+      <c r="K153" s="5" t="inlineStr">
+        <is>
+          <t>阶段/证据JSON编辑非图形设计器</t>
+        </is>
+      </c>
+      <c r="L153" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R003-v3验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="88" customHeight="1">
+      <c r="A154" s="5" t="n">
+        <v>149</v>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t>v3 / R003 v1</t>
+        </is>
+      </c>
+      <c r="C154" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D154" s="5" t="inlineStr">
+        <is>
+          <t>R003交付验证</t>
+        </is>
+      </c>
+      <c r="E154" s="5" t="inlineStr">
+        <is>
+          <t>四入口独立网页、T04演示、README/CHANGELOG及验收复盘</t>
+        </is>
+      </c>
+      <c r="F154" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G154" s="5" t="inlineStr">
+        <is>
+          <t>交付能复现与解释财务边界的作品</t>
+        </is>
+      </c>
+      <c r="H154" s="5" t="inlineStr">
+        <is>
+          <t>R003 → r003.html / 文档</t>
+        </is>
+      </c>
+      <c r="I154" s="5" t="inlineStr">
+        <is>
+          <t>在线T04完整演示及手机四区</t>
+        </is>
+      </c>
+      <c r="J154" s="5" t="inlineStr">
+        <is>
+          <t>259项业务/157项浏览器全部通过，R00334项含T01–T30、3项页面流程；生产独立HTML T04驳回/刷新保留、手机四区和R002互链通过；基线12项服务连接失败重启后全通过</t>
+        </is>
+      </c>
+      <c r="K154" s="5" t="inlineStr">
+        <is>
+          <t>无真实访谈或收益数据，不新增R004</t>
+        </is>
+      </c>
+      <c r="L154" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R003-v3验收.md</t>
         </is>
       </c>
     </row>
@@ -10306,6 +10691,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L146" r:id="rId141"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L147" r:id="rId142"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L148" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L149" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L150" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L151" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L152" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L153" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L154" r:id="rId149"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10319,7 +10710,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId144"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId150"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10741,7 +11132,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>记录口径更新于 2026-10-24</t>
+          <t>记录口径更新于 2026-10-25</t>
         </is>
       </c>
     </row>
@@ -10885,7 +11276,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v2 / R002 v1只新增发票重复风险审核、模拟历史库、独立人工复核及版本证据；保留R001判断和数据。225项业务/154项浏览器通过，不代表跨用户查重、税务验真或真实企业收益。</t>
+          <t>v3 / R003 v1新增三模式合同付款条件审核、已支付/待支付分离、独立人工与版本证据、模拟数据管理；259业务/157浏览器通过。无真实付款或跨用户资金占用事务。</t>
         </is>
       </c>
     </row>
@@ -10897,7 +11288,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/r002.html（R002）；同目录r001.html保留住宿审核，根地址为原轻报。</t>
+          <t>https://jameyan42.github.io/-/r003.html（R003）；同目录r001.html/r002.html保留住宿与发票审核，根地址为原轻报。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record local OCR integration and sample verification in feature history
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$36</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$154</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$157</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H35" headerRowCount="1">
-  <autoFilter ref="A5:H35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H36" headerRowCount="1">
+  <autoFilter ref="A5:H36"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L154" headerRowCount="1">
-  <autoFilter ref="A5:L154"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L157" headerRowCount="1">
+  <autoFilter ref="A5:L157"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-25  |  已交付 30 个阶段、149 项内容  |  当前功能版本 v3 / R003 v1  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-25  |  已交付 31 个阶段、152 项内容  |  当前功能版本 OCR本机引擎验证  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1734,6 +1734,42 @@
       <c r="H35" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/16d1735</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="74" customHeight="1">
+      <c r="A36" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>OCR本机引擎验证</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>可选RapidOCR本机接入与真实字段验证</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>259业务测试/23项OCR与PDF票面浏览器通过；本机RapidOCR实际模型推理及浏览器10字段、电子PDF、原识别框、403/400边界验证通过；非任意真实发票准确率结论</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/e25bebc</t>
         </is>
       </c>
     </row>
@@ -1774,6 +1810,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId31"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1787,7 +1824,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId32"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1799,7 +1836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L154"/>
+  <dimension ref="A1:L157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10538,6 +10575,180 @@
       <c r="L154" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/R003-v3验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="88" customHeight="1">
+      <c r="A155" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>OCR本机引擎验证</t>
+        </is>
+      </c>
+      <c r="C155" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>OCR引擎</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>开源调研及RapidOCR ONNX可选本机服务</t>
+        </is>
+      </c>
+      <c r="F155" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G155" s="5" t="inlineStr">
+        <is>
+          <t>比较中文票据适用性，不直接依赖外部演示</t>
+        </is>
+      </c>
+      <c r="H155" s="5" t="inlineStr">
+        <is>
+          <t>services/local_ocr</t>
+        </is>
+      </c>
+      <c r="I155" s="5" t="inlineStr">
+        <is>
+          <t>本机8765打开主应用</t>
+        </is>
+      </c>
+      <c r="J155" s="5" t="inlineStr">
+        <is>
+          <t>259业务测试/23项OCR与PDF票面浏览器通过；本机RapidOCR实际模型推理及浏览器10字段、电子PDF、原识别框、403/400边界验证通过；非任意真实发票准确率结论</t>
+        </is>
+      </c>
+      <c r="K155" s="5" t="inlineStr">
+        <is>
+          <t>GitHub Pages不运行Python，线上未切换</t>
+        </is>
+      </c>
+      <c r="L155" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/services/local_ocr/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="88" customHeight="1">
+      <c r="A156" s="5" t="n">
+        <v>151</v>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>OCR本机引擎验证</t>
+        </is>
+      </c>
+      <c r="C156" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D156" s="5" t="inlineStr">
+        <is>
+          <t>OCR适配</t>
+        </is>
+      </c>
+      <c r="E156" s="5" t="inlineStr">
+        <is>
+          <t>原OCR调用链本机模式、PDF预处理与人工字段确认</t>
+        </is>
+      </c>
+      <c r="F156" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G156" s="5" t="inlineStr">
+        <is>
+          <t>保持旧流程，识别范围只送本机</t>
+        </is>
+      </c>
+      <c r="H156" s="5" t="inlineStr">
+        <is>
+          <t>报销 / 对公票面采集</t>
+        </is>
+      </c>
+      <c r="I156" s="5" t="inlineStr">
+        <is>
+          <t>结构化PNG 10字段、PDF106元、原框268.50元</t>
+        </is>
+      </c>
+      <c r="J156" s="5" t="inlineStr">
+        <is>
+          <t>259业务测试/23项OCR与PDF票面浏览器通过；本机RapidOCR实际模型推理及浏览器10字段、电子PDF、原识别框、403/400边界验证通过；非任意真实发票准确率结论</t>
+        </is>
+      </c>
+      <c r="K156" s="5" t="inlineStr">
+        <is>
+          <t>不含逐行商品/二维码/验真，需脱敏真实样本</t>
+        </is>
+      </c>
+      <c r="L156" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/services/local_ocr/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="88" customHeight="1">
+      <c r="A157" s="5" t="n">
+        <v>152</v>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>OCR本机引擎验证</t>
+        </is>
+      </c>
+      <c r="C157" s="6" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>OCR保护及验证</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>Host/Origin限制、图片上限、单任务锁、无票据日志落盘</t>
+        </is>
+      </c>
+      <c r="F157" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G157" s="5" t="inlineStr">
+        <is>
+          <t>限制本机服务暴露并真实运行模型</t>
+        </is>
+      </c>
+      <c r="H157" s="5" t="inlineStr">
+        <is>
+          <t>本机浏览器验证脚本</t>
+        </is>
+      </c>
+      <c r="I157" s="5" t="inlineStr">
+        <is>
+          <t>跨来源403、坏图片400及同源请求</t>
+        </is>
+      </c>
+      <c r="J157" s="5" t="inlineStr">
+        <is>
+          <t>259业务测试/23项OCR与PDF票面浏览器通过；本机RapidOCR实际模型推理及浏览器10字段、电子PDF、原识别框、403/400边界验证通过；非任意真实发票准确率结论</t>
+        </is>
+      </c>
+      <c r="K157" s="5" t="inlineStr">
+        <is>
+          <t>非生产后端，取消不强杀正在运行的CPU任务</t>
+        </is>
+      </c>
+      <c r="L157" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/services/local_ocr/README.md</t>
         </is>
       </c>
     </row>
@@ -10697,6 +10908,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L152" r:id="rId147"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L153" r:id="rId148"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L154" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L155" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L156" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L157" r:id="rId152"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10710,7 +10924,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId150"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId153"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11276,7 +11490,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>v3 / R003 v1新增三模式合同付款条件审核、已支付/待支付分离、独立人工与版本证据、模拟数据管理；259业务/157浏览器通过。无真实付款或跨用户资金占用事务。</t>
+          <t>新增可选RapidOCR ONNX本机服务，模型与浏览器实测10票面字段及PDF；259业务/23项OCR相关浏览器通过。GitHub Pages仍为原Tesseract，需要脱敏失败样本验证真实版式；不是发票验真。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record S001 integration progress and compatibility limits
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$37</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$157</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$163</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H36" headerRowCount="1">
-  <autoFilter ref="A5:H36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H37" headerRowCount="1">
+  <autoFilter ref="A5:H37"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L157" headerRowCount="1">
-  <autoFilter ref="A5:L157"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L163" headerRowCount="1">
+  <autoFilter ref="A5:L163"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-25  |  已交付 31 个阶段、152 项内容  |  当前功能版本 OCR本机引擎验证  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-30  |  已交付 32 个阶段、158 项内容  |  当前功能版本 S001统一报销审核  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1770,6 +1770,42 @@
       <c r="H36" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/e25bebc</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="74" customHeight="1">
+      <c r="A37" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>S001统一报销审核</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>原轻报内统一报销单与三规则同批审核</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>274业务/164浏览器全通过，含新增15规则/状态与7页面流程；最后7项、构建导出及生产同构链再次通过；原R001/R002/合同R003不改核心</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/8bd1cb2</t>
         </is>
       </c>
     </row>
@@ -1811,6 +1847,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId32"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1824,7 +1861,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId32"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId33"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1836,7 +1873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L157"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10749,6 +10786,354 @@
       <c r="L157" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/services/local_ocr/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="88" customHeight="1">
+      <c r="A158" s="5" t="n">
+        <v>153</v>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>S001统一报销审核</t>
+        </is>
+      </c>
+      <c r="C158" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D158" s="5" t="inlineStr">
+        <is>
+          <t>统一报销对象</t>
+        </is>
+      </c>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>原主系统内草稿/住宿/多发票/稳定编号与列表搜索</t>
+        </is>
+      </c>
+      <c r="F158" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G158" s="5" t="inlineStr">
+        <is>
+          <t>一次录入，不反复切独立规则页面</t>
+        </is>
+      </c>
+      <c r="H158" s="5" t="inlineStr">
+        <is>
+          <t>报销单管理</t>
+        </is>
+      </c>
+      <c r="I158" s="5" t="inlineStr">
+        <is>
+          <t>载入600元住宿例、保存草稿并刷新</t>
+        </is>
+      </c>
+      <c r="J158" s="5" t="inlineStr">
+        <is>
+          <t>274业务/164浏览器全通过，含新增15规则/状态与7页面流程；最后7项、构建导出及生产同构链再次通过；原R001/R002/合同R003不改核心</t>
+        </is>
+      </c>
+      <c r="K158" s="5" t="inlineStr">
+        <is>
+          <t>旧单只读聚合保留原流程，不伪造迁移</t>
+        </is>
+      </c>
+      <c r="L158" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/S001-统一报销审核验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="88" customHeight="1">
+      <c r="A159" s="5" t="n">
+        <v>154</v>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>S001统一报销审核</t>
+        </is>
+      </c>
+      <c r="C159" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>统一规则注册</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>适配原R001/R002、统一状态和多风险/单规则ERROR</t>
+        </is>
+      </c>
+      <c r="F159" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G159" s="5" t="inlineStr">
+        <is>
+          <t>同批看到标准、重复和金额依据</t>
+        </is>
+      </c>
+      <c r="H159" s="5" t="inlineStr">
+        <is>
+          <t>审核详情 / 审核规则</t>
+        </is>
+      </c>
+      <c r="I159" s="5" t="inlineStr">
+        <is>
+          <t>1200申请、800标准、1000重复票同屏三异常</t>
+        </is>
+      </c>
+      <c r="J159" s="5" t="inlineStr">
+        <is>
+          <t>274业务/164浏览器全通过，含新增15规则/状态与7页面流程；最后7项、构建导出及生产同构链再次通过；原R001/R002/合同R003不改核心</t>
+        </is>
+      </c>
+      <c r="K159" s="5" t="inlineStr">
+        <is>
+          <t>历史规则集合快照兼容增量注册，未重写原制度</t>
+        </is>
+      </c>
+      <c r="L159" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/S001-统一报销审核验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="88" customHeight="1">
+      <c r="A160" s="5" t="n">
+        <v>155</v>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>S001统一报销审核</t>
+        </is>
+      </c>
+      <c r="C160" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D160" s="5" t="inlineStr">
+        <is>
+          <t>R003票额支持</t>
+        </is>
+      </c>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>多票整数分合计、超票额BLOCK、部分报销REVIEW</t>
+        </is>
+      </c>
+      <c r="F160" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G160" s="5" t="inlineStr">
+        <is>
+          <t>区别缺票与合理个人承担差额</t>
+        </is>
+      </c>
+      <c r="H160" s="5" t="inlineStr">
+        <is>
+          <t>统一审核R003</t>
+        </is>
+      </c>
+      <c r="I160" s="5" t="inlineStr">
+        <is>
+          <t>400+300支持700；少票200拦截；外币信息不足</t>
+        </is>
+      </c>
+      <c r="J160" s="5" t="inlineStr">
+        <is>
+          <t>274业务/164浏览器全通过，含新增15规则/状态与7页面流程；最后7项、构建导出及生产同构链再次通过；原R001/R002/合同R003不改核心</t>
+        </is>
+      </c>
+      <c r="K160" s="5" t="inlineStr">
+        <is>
+          <t>新内部key隔离，不覆盖既有合同付款R003</t>
+        </is>
+      </c>
+      <c r="L160" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/S001-统一报销审核验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="88" customHeight="1">
+      <c r="A161" s="5" t="n">
+        <v>156</v>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>S001统一报销审核</t>
+        </is>
+      </c>
+      <c r="C161" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>财务与历史</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>独立最终决定、意见、批次、编辑失效和重新审核</t>
+        </is>
+      </c>
+      <c r="F161" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G161" s="5" t="inlineStr">
+        <is>
+          <t>保留自动结论和旧批准，不静默沿用</t>
+        </is>
+      </c>
+      <c r="H161" s="5" t="inlineStr">
+        <is>
+          <t>财务审核 / 审核历史</t>
+        </is>
+      </c>
+      <c r="I161" s="5" t="inlineStr">
+        <is>
+          <t>批准后修改金额回草稿；重审保留全部版本</t>
+        </is>
+      </c>
+      <c r="J161" s="5" t="inlineStr">
+        <is>
+          <t>274业务/164浏览器全通过，含新增15规则/状态与7页面流程；最后7项、构建导出及生产同构链再次通过；原R001/R002/合同R003不改核心</t>
+        </is>
+      </c>
+      <c r="K161" s="5" t="inlineStr">
+        <is>
+          <t>BLOCK/信息不足/ERROR无普通例外授权，模拟身份非鉴权</t>
+        </is>
+      </c>
+      <c r="L161" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/S001-统一报销审核验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="88" customHeight="1">
+      <c r="A162" s="5" t="n">
+        <v>157</v>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>S001统一报销审核</t>
+        </is>
+      </c>
+      <c r="C162" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>票面及原件</t>
+        </is>
+      </c>
+      <c r="E162" s="5" t="inlineStr">
+        <is>
+          <t>复用原附件与图片PDF OCR，保存来源和明细</t>
+        </is>
+      </c>
+      <c r="F162" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G162" s="5" t="inlineStr">
+        <is>
+          <t>减少重复录入并明确候选需人工核对</t>
+        </is>
+      </c>
+      <c r="H162" s="5" t="inlineStr">
+        <is>
+          <t>统一报销表单发票区</t>
+        </is>
+      </c>
+      <c r="I162" s="5" t="inlineStr">
+        <is>
+          <t>原件识别265元并保存刷新、最多5票</t>
+        </is>
+      </c>
+      <c r="J162" s="5" t="inlineStr">
+        <is>
+          <t>274业务/164浏览器全通过，含新增15规则/状态与7页面流程；最后7项、构建导出及生产同构链再次通过；原R001/R002/合同R003不改核心</t>
+        </is>
+      </c>
+      <c r="K162" s="5" t="inlineStr">
+        <is>
+          <t>原件/快照受浏览器容量限制，不验真</t>
+        </is>
+      </c>
+      <c r="L162" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/S001-统一报销审核验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="88" customHeight="1">
+      <c r="A163" s="5" t="n">
+        <v>158</v>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>S001统一报销审核</t>
+        </is>
+      </c>
+      <c r="C163" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>整合交付</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>原网站导航布局、真实端到端及回归、文档和生产验证</t>
+        </is>
+      </c>
+      <c r="F163" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G163" s="5" t="inlineStr">
+        <is>
+          <t>交付连贯可操作的审核流程</t>
+        </is>
+      </c>
+      <c r="H163" s="5" t="inlineStr">
+        <is>
+          <t>/?view=claims</t>
+        </is>
+      </c>
+      <c r="I163" s="5" t="inlineStr">
+        <is>
+          <t>创建→自动审核→财务决定→列表→历史</t>
+        </is>
+      </c>
+      <c r="J163" s="5" t="inlineStr">
+        <is>
+          <t>274业务/164浏览器全通过，含新增15规则/状态与7页面流程；最后7项、构建导出及生产同构链再次通过；原R001/R002/合同R003不改核心</t>
+        </is>
+      </c>
+      <c r="K163" s="5" t="inlineStr">
+        <is>
+          <t>旧预算/付款/消息/全量备份未自动承接新单，无生产数据库</t>
+        </is>
+      </c>
+      <c r="L163" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/S001-统一报销审核验收.md</t>
         </is>
       </c>
     </row>
@@ -10911,6 +11296,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L155" r:id="rId150"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L156" r:id="rId151"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L157" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L158" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L159" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L160" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L161" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L162" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L163" r:id="rId158"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10924,7 +11315,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId153"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId159"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11346,7 +11737,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>记录口径更新于 2026-10-25</t>
+          <t>记录口径更新于 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -11490,7 +11881,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>新增可选RapidOCR ONNX本机服务，模型与浏览器实测10票面字段及PDF；259业务/23项OCR相关浏览器通过。GitHub Pages仍为原Tesseract，需要脱敏失败样本验证真实版式；不是发票验真。</t>
+          <t>S001在原轻报框架内接入统一报销、多票、三规则同批、财务决定及历史失效；274业务/164浏览器通过。旧单保留原流程，旧预算付款未自动接入，不覆盖合同R003。</t>
         </is>
       </c>
     </row>
@@ -11502,7 +11893,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>https://jameyan42.github.io/-/r003.html（R003）；同目录r001.html/r002.html保留住宿与发票审核，根地址为原轻报。</t>
+          <t>https://jameyan42.github.io/-/?view=claims（统一报销）；原工作台及独立规则页面兼容保留。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track R004 implementation and verification in feature workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$38</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$163</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$169</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H37" headerRowCount="1">
-  <autoFilter ref="A5:H37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H38" headerRowCount="1">
+  <autoFilter ref="A5:H38"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L163" headerRowCount="1">
-  <autoFilter ref="A5:L163"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L169" headerRowCount="1">
+  <autoFilter ref="A5:L169"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-30  |  已交付 32 个阶段、158 项内容  |  当前功能版本 S001统一报销审核  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-30  |  已交付 33 个阶段、164 项内容  |  当前功能版本 R004法人抬头税号  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1806,6 +1806,42 @@
       <c r="H37" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/8bd1cb2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="74" customHeight="1">
+      <c r="A38" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>R004法人抬头税号</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>统一报销多法人购买方抬头税号审核</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>293项业务/170项浏览器通过；R00419项含T001–T012与额外边界、6条新增页面；最后13项、独立构建及生产同构法人BLOCK→更正重审→保留旧批次通过</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/f98644b</t>
         </is>
       </c>
     </row>
@@ -1848,6 +1884,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId33"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1861,7 +1898,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId33"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId34"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1873,7 +1910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L163"/>
+  <dimension ref="A1:L169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11134,6 +11171,354 @@
       <c r="L163" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/S001-统一报销审核验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="88" customHeight="1">
+      <c r="A164" s="5" t="n">
+        <v>159</v>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>R004法人抬头税号</t>
+        </is>
+      </c>
+      <c r="C164" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>法人基准</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>三模拟法人、版本/有效期、历史名称及税号授权和票据政策</t>
+        </is>
+      </c>
+      <c r="F164" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G164" s="5" t="inlineStr">
+        <is>
+          <t>以明确法人代替部门或集团名称作为核对基准</t>
+        </is>
+      </c>
+      <c r="H164" s="5" t="inlineStr">
+        <is>
+          <t>统一报销表单 / 审核规则</t>
+        </is>
+      </c>
+      <c r="I164" s="5" t="inlineStr">
+        <is>
+          <t>选择深圳/东莞，查看标准名称税号和带日期别名</t>
+        </is>
+      </c>
+      <c r="J164" s="5" t="inlineStr">
+        <is>
+          <t>293项业务/170项浏览器通过；R00419项含T001–T012与额外边界、6条新增页面；最后13项、独立构建及生产同构法人BLOCK→更正重审→保留旧批次通过</t>
+        </is>
+      </c>
+      <c r="K164" s="5" t="inlineStr">
+        <is>
+          <t>虚构DEMO税号；JSON配置非正式主数据平台</t>
+        </is>
+      </c>
+      <c r="L164" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R004-发票抬头与税号验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="88" customHeight="1">
+      <c r="A165" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>R004法人抬头税号</t>
+        </is>
+      </c>
+      <c r="C165" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>R004逐票审核</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>完整名称税号比较、跨法人及个人抬头拦截、未知名称复核</t>
+        </is>
+      </c>
+      <c r="F165" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G165" s="5" t="inlineStr">
+        <is>
+          <t>不把集团子公司或相似名称当同一法人</t>
+        </is>
+      </c>
+      <c r="H165" s="5" t="inlineStr">
+        <is>
+          <t>统一审核R004</t>
+        </is>
+      </c>
+      <c r="I165" s="5" t="inlineStr">
+        <is>
+          <t>正常PASS、东莞票BLOCK、同税号未知名REVIEW</t>
+        </is>
+      </c>
+      <c r="J165" s="5" t="inlineStr">
+        <is>
+          <t>293项业务/170项浏览器通过；R00419项含T001–T012与额外边界、6条新增页面；最后13项、独立构建及生产同构法人BLOCK→更正重审→保留旧批次通过</t>
+        </is>
+      </c>
+      <c r="K165" s="5" t="inlineStr">
+        <is>
+          <t>无税务联网验真或官方格式校验</t>
+        </is>
+      </c>
+      <c r="L165" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R004-发票抬头与税号验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="88" customHeight="1">
+      <c r="A166" s="5" t="n">
+        <v>161</v>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>R004法人抬头税号</t>
+        </is>
+      </c>
+      <c r="C166" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>识别可靠性</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>核对状态/整体置信度与原票税号是否确为空分开</t>
+        </is>
+      </c>
+      <c r="F166" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G166" s="5" t="inlineStr">
+        <is>
+          <t>避免将OCR漏读直接当作已确认错票</t>
+        </is>
+      </c>
+      <c r="H166" s="5" t="inlineStr">
+        <is>
+          <t>统一发票区 / R004依据</t>
+        </is>
+      </c>
+      <c r="I166" s="5" t="inlineStr">
+        <is>
+          <t>未知空税号信息不足，票面确认空按模拟政策BLOCK</t>
+        </is>
+      </c>
+      <c r="J166" s="5" t="inlineStr">
+        <is>
+          <t>293项业务/170项浏览器通过；R00419项含T001–T012与额外边界、6条新增页面；最后13项、独立构建及生产同构法人BLOCK→更正重审→保留旧批次通过</t>
+        </is>
+      </c>
+      <c r="K166" s="5" t="inlineStr">
+        <is>
+          <t>高整体分数不等于真实字段概率，需人工核对</t>
+        </is>
+      </c>
+      <c r="L166" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R004-发票抬头与税号验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="88" customHeight="1">
+      <c r="A167" s="5" t="n">
+        <v>162</v>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>R004法人抬头税号</t>
+        </is>
+      </c>
+      <c r="C167" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>财务留痕</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>补材料/已核实意见、修改原因及前后值、角色时间记录</t>
+        </is>
+      </c>
+      <c r="F167" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G167" s="5" t="inlineStr">
+        <is>
+          <t>记录人工责任而不覆盖自动结论</t>
+        </is>
+      </c>
+      <c r="H167" s="5" t="inlineStr">
+        <is>
+          <t>财务复核 / 审核历史</t>
+        </is>
+      </c>
+      <c r="I167" s="5" t="inlineStr">
+        <is>
+          <t>记录核查、修改所属公司重审、旧BLOCK保留</t>
+        </is>
+      </c>
+      <c r="J167" s="5" t="inlineStr">
+        <is>
+          <t>293项业务/170项浏览器通过；R00419项含T001–T012与额外边界、6条新增页面；最后13项、独立构建及生产同构法人BLOCK→更正重审→保留旧批次通过</t>
+        </is>
+      </c>
+      <c r="K167" s="5" t="inlineStr">
+        <is>
+          <t>BLOCK无普通例外放行，前端模拟身份非生产授权</t>
+        </is>
+      </c>
+      <c r="L167" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R004-发票抬头与税号验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="88" customHeight="1">
+      <c r="A168" s="5" t="n">
+        <v>163</v>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>R004法人抬头税号</t>
+        </is>
+      </c>
+      <c r="C168" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D168" s="5" t="inlineStr">
+        <is>
+          <t>版本兼容</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>配置快照、旧三规则读取和新四规则同批</t>
+        </is>
+      </c>
+      <c r="F168" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G168" s="5" t="inlineStr">
+        <is>
+          <t>更新配置不追改旧记录，R001–R003核心保留</t>
+        </is>
+      </c>
+      <c r="H168" s="5" t="inlineStr">
+        <is>
+          <t>审核批次 / 配置版本</t>
+        </is>
+      </c>
+      <c r="I168" s="5" t="inlineStr">
+        <is>
+          <t>配置改版本后新审用新值、旧结果仍可重放</t>
+        </is>
+      </c>
+      <c r="J168" s="5" t="inlineStr">
+        <is>
+          <t>293项业务/170项浏览器通过；R00419项含T001–T012与额外边界、6条新增页面；最后13项、独立构建及生产同构法人BLOCK→更正重审→保留旧批次通过</t>
+        </is>
+      </c>
+      <c r="K168" s="5" t="inlineStr">
+        <is>
+          <t>特殊票R004NA不豁免其他规则</t>
+        </is>
+      </c>
+      <c r="L168" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R004-发票抬头与税号验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="88" customHeight="1">
+      <c r="A169" s="5" t="n">
+        <v>164</v>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>R004法人抬头税号</t>
+        </is>
+      </c>
+      <c r="C169" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>交付与验证</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>R004产品复盘、测试、文字安全和原网站集成</t>
+        </is>
+      </c>
+      <c r="F169" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G169" s="5" t="inlineStr">
+        <is>
+          <t>交付可解释且有实测依据的单规则增量</t>
+        </is>
+      </c>
+      <c r="H169" s="5" t="inlineStr">
+        <is>
+          <t>R004_PRODUCT_DESIGN_NOTES / 验收</t>
+        </is>
+      </c>
+      <c r="I169" s="5" t="inlineStr">
+        <is>
+          <t>一次执行四异常、手机逐票可读、配置注入不执行</t>
+        </is>
+      </c>
+      <c r="J169" s="5" t="inlineStr">
+        <is>
+          <t>293项业务/170项浏览器通过；R00419项含T001–T012与额外边界、6条新增页面；最后13项、独立构建及生产同构法人BLOCK→更正重审→保留旧批次通过</t>
+        </is>
+      </c>
+      <c r="K169" s="5" t="inlineStr">
+        <is>
+          <t>无新增OCR/银行/ERP/AI模块或新依赖</t>
+        </is>
+      </c>
+      <c r="L169" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R004-发票抬头与税号验收.md</t>
         </is>
       </c>
     </row>
@@ -11302,6 +11687,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L161" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L162" r:id="rId157"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L163" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L164" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L165" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L166" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L167" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L168" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L169" r:id="rId164"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11315,7 +11706,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId159"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId165"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11881,7 +12272,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>S001在原轻报框架内接入统一报销、多票、三规则同批、财务决定及历史失效；274业务/164浏览器通过。旧单保留原流程，旧预算付款未自动接入，不覆盖合同R003。</t>
+          <t>R004接入S001：法人/历史名称及税号/票据政策、逐票结果、OCR可信区分和变更核查留痕；293业务/170浏览器通过。非官方验真、前端身份非生产鉴权，无新引擎或独立R004页。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record R005 stage and refresh feature history workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$39</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$169</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$173</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H38" headerRowCount="1">
-  <autoFilter ref="A5:H38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H39" headerRowCount="1">
+  <autoFilter ref="A5:H39"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L169" headerRowCount="1">
-  <autoFilter ref="A5:L169"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L173" headerRowCount="1">
+  <autoFilter ref="A5:L173"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-30  |  已交付 33 个阶段、164 项内容  |  当前功能版本 R004法人抬头税号  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-30  |  已交付 34 个阶段、168 项内容  |  当前功能版本 R005费用科目匹配  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1842,6 +1842,42 @@
       <c r="H38" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/f98644b</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="74" customHeight="1">
+      <c r="A39" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>R005费用科目匹配</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>统一费用预核算与法人科目映射审核</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>311项业务/175项固定版本浏览器通过；R00518项单元含T001–T012与5条页面流程；最终52项统一规则、构建及生产同构更正科目/批准/刷新留史通过</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/249cbd1</t>
         </is>
       </c>
     </row>
@@ -1885,6 +1921,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId34"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1898,7 +1935,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId34"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId35"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1910,7 +1947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L169"/>
+  <dimension ref="A1:L173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11519,6 +11556,238 @@
       <c r="L169" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/R004-发票抬头与税号验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="88" customHeight="1">
+      <c r="A170" s="5" t="n">
+        <v>165</v>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
+        <is>
+          <t>R005费用科目匹配</t>
+        </is>
+      </c>
+      <c r="C170" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D170" s="5" t="inlineStr">
+        <is>
+          <t>核算制度</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>法人/集团科目映射、多个允许科目、生效期及冲突处理</t>
+        </is>
+      </c>
+      <c r="F170" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G170" s="5" t="inlineStr">
+        <is>
+          <t>规则驱动推荐，避免错用主体及单默认科目</t>
+        </is>
+      </c>
+      <c r="H170" s="5" t="inlineStr">
+        <is>
+          <t>审核规则 / 报销单</t>
+        </is>
+      </c>
+      <c r="I170" s="5" t="inlineStr">
+        <is>
+          <t>深圳住宿6602.01、东莞6602.11、培训6602.05</t>
+        </is>
+      </c>
+      <c r="J170" s="5" t="inlineStr">
+        <is>
+          <t>311项业务/175项固定版本浏览器通过；R00518项单元含T001–T012与5条页面流程；最终52项统一规则、构建及生产同构更正科目/批准/刷新留史通过</t>
+        </is>
+      </c>
+      <c r="K170" s="5" t="inlineStr">
+        <is>
+          <t>仅模拟制度，复杂事项不强制费用化</t>
+        </is>
+      </c>
+      <c r="L170" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R005-费用科目匹配验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="88" customHeight="1">
+      <c r="A171" s="5" t="n">
+        <v>166</v>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>R005费用科目匹配</t>
+        </is>
+      </c>
+      <c r="C171" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>员工与财务</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>推荐与财务确认分离、明确业务阶段及科目异常</t>
+        </is>
+      </c>
+      <c r="F171" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G171" s="5" t="inlineStr">
+        <is>
+          <t>员工不强制填科目，财务修正后重审</t>
+        </is>
+      </c>
+      <c r="H171" s="5" t="inlineStr">
+        <is>
+          <t>报销单管理 / 财务审核</t>
+        </is>
+      </c>
+      <c r="I171" s="5" t="inlineStr">
+        <is>
+          <t>员工待确认、错科目BLOCK、修正PASS</t>
+        </is>
+      </c>
+      <c r="J171" s="5" t="inlineStr">
+        <is>
+          <t>311项业务/175项固定版本浏览器通过；R00518项单元含T001–T012与5条页面流程；最终52项统一规则、构建及生产同构更正科目/批准/刷新留史通过</t>
+        </is>
+      </c>
+      <c r="K171" s="5" t="inlineStr">
+        <is>
+          <t>模拟角色非生产鉴权，无总账凭证</t>
+        </is>
+      </c>
+      <c r="L171" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R005-费用科目匹配验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="88" customHeight="1">
+      <c r="A172" s="5" t="n">
+        <v>167</v>
+      </c>
+      <c r="B172" s="5" t="inlineStr">
+        <is>
+          <t>R005费用科目匹配</t>
+        </is>
+      </c>
+      <c r="C172" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D172" s="5" t="inlineStr">
+        <is>
+          <t>历史证据</t>
+        </is>
+      </c>
+      <c r="E172" s="5" t="inlineStr">
+        <is>
+          <t>科目制度版本及输入快照、修改前后值和旧批次兼容</t>
+        </is>
+      </c>
+      <c r="F172" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G172" s="5" t="inlineStr">
+        <is>
+          <t>不覆盖历史，不沿用失效批准</t>
+        </is>
+      </c>
+      <c r="H172" s="5" t="inlineStr">
+        <is>
+          <t>审核历史 / 审核规则</t>
+        </is>
+      </c>
+      <c r="I172" s="5" t="inlineStr">
+        <is>
+          <t>配置变更和科目更正后比较旧新批次</t>
+        </is>
+      </c>
+      <c r="J172" s="5" t="inlineStr">
+        <is>
+          <t>311项业务/175项固定版本浏览器通过；R00518项单元含T001–T012与5条页面流程；最终52项统一规则、构建及生产同构更正科目/批准/刷新留史通过</t>
+        </is>
+      </c>
+      <c r="K172" s="5" t="inlineStr">
+        <is>
+          <t>无服务端防篡改和授权例外流程</t>
+        </is>
+      </c>
+      <c r="L172" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R005-费用科目匹配验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="88" customHeight="1">
+      <c r="A173" s="5" t="n">
+        <v>168</v>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>R005费用科目匹配</t>
+        </is>
+      </c>
+      <c r="C173" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>交付与验证</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>五异常集成回归、业务解释及14道面试追问</t>
+        </is>
+      </c>
+      <c r="F173" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G173" s="5" t="inlineStr">
+        <is>
+          <t>用实际规则和测试展示产品判断</t>
+        </is>
+      </c>
+      <c r="H173" s="5" t="inlineStr">
+        <is>
+          <t>R005_BUSINESS_RULES / PRODUCT_INTERVIEW / 验收</t>
+        </is>
+      </c>
+      <c r="I173" s="5" t="inlineStr">
+        <is>
+          <t>五条规则一次输出，再走完整财务修正链</t>
+        </is>
+      </c>
+      <c r="J173" s="5" t="inlineStr">
+        <is>
+          <t>311项业务/175项固定版本浏览器通过；R00518项单元含T001–T012与5条页面流程；最终52项统一规则、构建及生产同构更正科目/批准/刷新留史通过</t>
+        </is>
+      </c>
+      <c r="K173" s="5" t="inlineStr">
+        <is>
+          <t>无外部AI服务、新依赖、独立R005网页或真实企业收益证明</t>
+        </is>
+      </c>
+      <c r="L173" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R005-费用科目匹配验收.md</t>
         </is>
       </c>
     </row>
@@ -11693,6 +11962,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L167" r:id="rId162"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L168" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L169" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L170" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L171" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L172" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L173" r:id="rId168"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11706,7 +11979,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId165"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId169"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12272,7 +12545,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>R004接入S001：法人/历史名称及税号/票据政策、逐票结果、OCR可信区分和变更核查留痕；293业务/170浏览器通过。非官方验真、前端身份非生产鉴权，无新引擎或独立R004页。</t>
+          <t>R005接入S001：法人/集团科目映射、允许集合/期限/冲突、员工推荐与财务确认分离、版本和更正留痕；311业务/175浏览器通过。非正式记账、前端身份非生产鉴权，无新依赖或独立R005页。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record R006 stage and refresh feature history workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$39</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$173</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$177</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H39" headerRowCount="1">
-  <autoFilter ref="A5:H39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H40" headerRowCount="1">
+  <autoFilter ref="A5:H40"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L173" headerRowCount="1">
-  <autoFilter ref="A5:L173"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L177" headerRowCount="1">
+  <autoFilter ref="A5:L177"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-30  |  已交付 34 个阶段、168 项内容  |  当前功能版本 R005费用科目匹配  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-30  |  已交付 35 个阶段、172 项内容  |  当前功能版本 R006审批附件完整性  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1878,6 +1878,42 @@
       <c r="H39" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/249cbd1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="74" customHeight="1">
+      <c r="A40" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>R006审批附件完整性</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>统一具名业务审批与附件完整性审核</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>335项业务/184项浏览器最终全通过；R00624项规则含T001–T016、9项页面流程；构建导出及生产同构1500元缺节点/缺文件→补正重提→两人审批→六规则PASS→财务批准→刷新历史通过</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/3405c54</t>
         </is>
       </c>
     </row>
@@ -1922,6 +1958,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId35"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1935,7 +1972,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId35"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId36"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1947,7 +1984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L173"/>
+  <dimension ref="A1:L177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11788,6 +11825,238 @@
       <c r="L173" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/R005-费用科目匹配验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="88" customHeight="1">
+      <c r="A174" s="5" t="n">
+        <v>169</v>
+      </c>
+      <c r="B174" s="5" t="inlineStr">
+        <is>
+          <t>R006审批附件完整性</t>
+        </is>
+      </c>
+      <c r="C174" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D174" s="5" t="inlineStr">
+        <is>
+          <t>审批与授权</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>法人金额政策、具名顺序审批、职责分离及驳回退回</t>
+        </is>
+      </c>
+      <c r="F174" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G174" s="5" t="inlineStr">
+        <is>
+          <t>识别缺节点与越权，区分正常等待</t>
+        </is>
+      </c>
+      <c r="H174" s="5" t="inlineStr">
+        <is>
+          <t>报销详情 / 财务审核</t>
+        </is>
+      </c>
+      <c r="I174" s="5" t="inlineStr">
+        <is>
+          <t>深圳1500元主管赵航→负责人许明</t>
+        </is>
+      </c>
+      <c r="J174" s="5" t="inlineStr">
+        <is>
+          <t>335项业务/184项浏览器最终全通过；R00624项规则含T001–T016、9项页面流程；构建导出及生产同构1500元缺节点/缺文件→补正重提→两人审批→六规则PASS→财务批准→刷新历史通过</t>
+        </is>
+      </c>
+      <c r="K174" s="5" t="inlineStr">
+        <is>
+          <t>模拟组织授权，无真实身份/BPM/签名</t>
+        </is>
+      </c>
+      <c r="L174" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R006-审批附件完整性验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="88" customHeight="1">
+      <c r="A175" s="5" t="n">
+        <v>170</v>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>R006审批附件完整性</t>
+        </is>
+      </c>
+      <c r="C175" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>报销材料</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>真实文件分类、逐票/多票PDF关联、人工核实及出差申请替代</t>
+        </is>
+      </c>
+      <c r="F175" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G175" s="5" t="inlineStr">
+        <is>
+          <t>不将票面字段或文件标签当作有效材料</t>
+        </is>
+      </c>
+      <c r="H175" s="5" t="inlineStr">
+        <is>
+          <t>报销单编辑 / R006-B</t>
+        </is>
+      </c>
+      <c r="I175" s="5" t="inlineStr">
+        <is>
+          <t>原件缺失→上传关联→待核实→明确人工核实</t>
+        </is>
+      </c>
+      <c r="J175" s="5" t="inlineStr">
+        <is>
+          <t>335项业务/184项浏览器最终全通过；R00624项规则含T001–T016、9项页面流程；构建导出及生产同构1500元缺节点/缺文件→补正重提→两人审批→六规则PASS→财务批准→刷新历史通过</t>
+        </is>
+      </c>
+      <c r="K175" s="5" t="inlineStr">
+        <is>
+          <t>基础格式/保存检查非票据验真或内容识别</t>
+        </is>
+      </c>
+      <c r="L175" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R006-审批附件完整性验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="88" customHeight="1">
+      <c r="A176" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>R006审批附件完整性</t>
+        </is>
+      </c>
+      <c r="C176" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D176" s="5" t="inlineStr">
+        <is>
+          <t>历史与内控</t>
+        </is>
+      </c>
+      <c r="E176" s="5" t="inlineStr">
+        <is>
+          <t>单据版本绑定、政策组织快照、金额/附件操作与新批准门槛</t>
+        </is>
+      </c>
+      <c r="F176" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G176" s="5" t="inlineStr">
+        <is>
+          <t>旧结果保留，资料变化须重新审批，历史未执行不补通过</t>
+        </is>
+      </c>
+      <c r="H176" s="5" t="inlineStr">
+        <is>
+          <t>审核历史 / 规则配置</t>
+        </is>
+      </c>
+      <c r="I176" s="5" t="inlineStr">
+        <is>
+          <t>审批800后改1500或删文件，旧审批不覆盖新版本</t>
+        </is>
+      </c>
+      <c r="J176" s="5" t="inlineStr">
+        <is>
+          <t>335项业务/184项浏览器最终全通过；R00624项规则含T001–T016、9项页面流程；构建导出及生产同构1500元缺节点/缺文件→补正重提→两人审批→六规则PASS→财务批准→刷新历史通过</t>
+        </is>
+      </c>
+      <c r="K176" s="5" t="inlineStr">
+        <is>
+          <t>本地演示日志非防篡改，全字段变更保守重审</t>
+        </is>
+      </c>
+      <c r="L176" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R006-审批附件完整性验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="88" customHeight="1">
+      <c r="A177" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>R006审批附件完整性</t>
+        </is>
+      </c>
+      <c r="C177" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="D177" s="5" t="inlineStr">
+        <is>
+          <t>交付与验证</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>六规则异常共存、完整链路及规则/面试/演示文档</t>
+        </is>
+      </c>
+      <c r="F177" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G177" s="5" t="inlineStr">
+        <is>
+          <t>以实际流程验证产品内控边界</t>
+        </is>
+      </c>
+      <c r="H177" s="5" t="inlineStr">
+        <is>
+          <t>R006_BUSINESS_RULES / PRODUCT_INTERVIEW / 验收</t>
+        </is>
+      </c>
+      <c r="I177" s="5" t="inlineStr">
+        <is>
+          <t>旧五规则可读、新批准先重审；手机可用</t>
+        </is>
+      </c>
+      <c r="J177" s="5" t="inlineStr">
+        <is>
+          <t>335项业务/184项浏览器最终全通过；R00624项规则含T001–T016、9项页面流程；构建导出及生产同构1500元缺节点/缺文件→补正重提→两人审批→六规则PASS→财务批准→刷新历史通过</t>
+        </is>
+      </c>
+      <c r="K177" s="5" t="inlineStr">
+        <is>
+          <t>无新依赖、独立R006页、银行付款或真实企业收益</t>
+        </is>
+      </c>
+      <c r="L177" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R006-审批附件完整性验收.md</t>
         </is>
       </c>
     </row>
@@ -11966,6 +12235,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L171" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L172" r:id="rId167"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L173" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L174" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L175" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId172"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11979,7 +12252,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId169"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId173"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12545,7 +12818,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>R005接入S001：法人/集团科目映射、允许集合/期限/冲突、员工推荐与财务确认分离、版本和更正留痕；311业务/175浏览器通过。非正式记账、前端身份非生产鉴权，无新依赖或独立R005页。</t>
+          <t>R006接入S001：法人金额政策、具名/顺序/职责分离、材料逐票关联与内容待核实、版本化审批及操作留痕；335业务/184浏览器通过。非生产鉴权、验真或防篡改，无新依赖或独立R006页。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record R007 stage and refresh feature history workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$41</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$177</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$181</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H40" headerRowCount="1">
-  <autoFilter ref="A5:H40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H41" headerRowCount="1">
+  <autoFilter ref="A5:H41"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L177" headerRowCount="1">
-  <autoFilter ref="A5:L177"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L181" headerRowCount="1">
+  <autoFilter ref="A5:L181"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-30  |  已交付 35 个阶段、172 项内容  |  当前功能版本 R006审批附件完整性  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-31  |  已交付 36 个阶段、176 项内容  |  当前功能版本 R007预算额度控制  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1914,6 +1914,42 @@
       <c r="H40" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/3405c54</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="74" customHeight="1">
+      <c r="A41" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>R007预算额度控制</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>统一预算生命周期、事件流水与具名超额授权</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>365项业务/193项全量浏览器通过；最后预算15项、统一规则106项补测通过；R00730项含T001–T022、9条页面，最终构建及生产同构超500→额外授权→财务批准→一次结转/负余额/历史通过</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/5cc6fb4</t>
         </is>
       </c>
     </row>
@@ -1959,6 +1995,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId36"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1972,7 +2009,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId36"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1984,7 +2021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L177"/>
+  <dimension ref="A1:L181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12057,6 +12094,238 @@
       <c r="L177" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/R006-审批附件完整性验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="88" customHeight="1">
+      <c r="A178" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="B178" s="5" t="inlineStr">
+        <is>
+          <t>R007预算额度控制</t>
+        </is>
+      </c>
+      <c r="C178" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D178" s="5" t="inlineStr">
+        <is>
+          <t>预算政策与审核</t>
+        </is>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>法人部门费用类型发生月、HARD/SOFT/WARNING及整数分余额</t>
+        </is>
+      </c>
+      <c r="F178" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G178" s="5" t="inlineStr">
+        <is>
+          <t>规则可配置，不把未设预算当无限</t>
+        </is>
+      </c>
+      <c r="H178" s="5" t="inlineStr">
+        <is>
+          <t>预算管理 / 报销单 / R007</t>
+        </is>
+      </c>
+      <c r="I178" s="5" t="inlineStr">
+        <is>
+          <t>10000-6000-2000可用2000，2500超500</t>
+        </is>
+      </c>
+      <c r="J178" s="5" t="inlineStr">
+        <is>
+          <t>365项业务/193项全量浏览器通过；最后预算15项、统一规则106项补测通过；R00730项含T001–T022、9条页面，最终构建及生产同构超500→额外授权→财务批准→一次结转/负余额/历史通过</t>
+        </is>
+      </c>
+      <c r="K178" s="5" t="inlineStr">
+        <is>
+          <t>单预算归属、人民币、跨月需确认</t>
+        </is>
+      </c>
+      <c r="L178" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R007-费用预算与额度验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="88" customHeight="1">
+      <c r="A179" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>R007预算额度控制</t>
+        </is>
+      </c>
+      <c r="C179" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D179" s="5" t="inlineStr">
+        <is>
+          <t>预算生命周期</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>提交预占、在途差额、驳回撤销释放、财务结转及幂等事件</t>
+        </is>
+      </c>
+      <c r="F179" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G179" s="5" t="inlineStr">
+        <is>
+          <t>不重复扣减，已使用不能直接改/撤</t>
+        </is>
+      </c>
+      <c r="H179" s="5" t="inlineStr">
+        <is>
+          <t>报销详情 / 预算流水</t>
+        </is>
+      </c>
+      <c r="I179" s="5" t="inlineStr">
+        <is>
+          <t>800改1200只调400，预占转已使用不再减一次</t>
+        </is>
+      </c>
+      <c r="J179" s="5" t="inlineStr">
+        <is>
+          <t>365项业务/193项全量浏览器通过；最后预算15项、统一规则106项补测通过；R00730项含T001–T022、9条页面，最终构建及生产同构超500→额外授权→财务批准→一次结转/负余额/历史通过</t>
+        </is>
+      </c>
+      <c r="K179" s="5" t="inlineStr">
+        <is>
+          <t>本地存储非多人事务或防篡改，正式冲销尚无</t>
+        </is>
+      </c>
+      <c r="L179" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R007-费用预算与额度验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="88" customHeight="1">
+      <c r="A180" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="B180" s="5" t="inlineStr">
+        <is>
+          <t>R007预算额度控制</t>
+        </is>
+      </c>
+      <c r="C180" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D180" s="5" t="inlineStr">
+        <is>
+          <t>审批联动与证据</t>
+        </is>
+      </c>
+      <c r="E180" s="5" t="inlineStr">
+        <is>
+          <t>具名预算负责人第三节点、在途补授权、批准时实时预算复查</t>
+        </is>
+      </c>
+      <c r="F180" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G180" s="5" t="inlineStr">
+        <is>
+          <t>普通意见不能绕过超额授权，保留金额风险</t>
+        </is>
+      </c>
+      <c r="H180" s="5" t="inlineStr">
+        <is>
+          <t>R006 / 财务最终复核 / 审核历史</t>
+        </is>
+      </c>
+      <c r="I180" s="5" t="inlineStr">
+        <is>
+          <t>授权后R006PASS、R007仍REVIEW，财务独立批准</t>
+        </is>
+      </c>
+      <c r="J180" s="5" t="inlineStr">
+        <is>
+          <t>365项业务/193项全量浏览器通过；最后预算15项、统一规则106项补测通过；R00730项含T001–T022、9条页面，最终构建及生产同构超500→额外授权→财务批准→一次结转/负余额/历史通过</t>
+        </is>
+      </c>
+      <c r="K180" s="5" t="inlineStr">
+        <is>
+          <t>旧预算及未登记历史不自动迁移，不伪造已使用</t>
+        </is>
+      </c>
+      <c r="L180" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R007-费用预算与额度验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="88" customHeight="1">
+      <c r="A181" s="5" t="n">
+        <v>176</v>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>R007预算额度控制</t>
+        </is>
+      </c>
+      <c r="C181" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D181" s="5" t="inlineStr">
+        <is>
+          <t>交付与验证</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>预算筛选配置看板、显式期初模拟、精度与终态保护及演示文档</t>
+        </is>
+      </c>
+      <c r="F181" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G181" s="5" t="inlineStr">
+        <is>
+          <t>在同一网站演示完整预算控制</t>
+        </is>
+      </c>
+      <c r="H181" s="5" t="inlineStr">
+        <is>
+          <t>R007业务规则 / 面试 / 演示 / 验收</t>
+        </is>
+      </c>
+      <c r="I181" s="5" t="inlineStr">
+        <is>
+          <t>主案例、正常案例、驳回释放；手机及极大分位验证</t>
+        </is>
+      </c>
+      <c r="J181" s="5" t="inlineStr">
+        <is>
+          <t>365项业务/193项全量浏览器通过；最后预算15项、统一规则106项补测通过；R00730项含T001–T022、9条页面，最终构建及生产同构超500→额外授权→财务批准→一次结转/负余额/历史通过</t>
+        </is>
+      </c>
+      <c r="K181" s="5" t="inlineStr">
+        <is>
+          <t>无新网站/依赖、银行、总账、预测AI或真实企业收益</t>
+        </is>
+      </c>
+      <c r="L181" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R007-费用预算与额度验收.md</t>
         </is>
       </c>
     </row>
@@ -12239,6 +12508,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L175" r:id="rId170"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId171"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId176"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12252,7 +12525,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId173"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId177"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12674,7 +12947,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>记录口径更新于 2026-10-30</t>
+          <t>记录口径更新于 2026-10-31</t>
         </is>
       </c>
     </row>
@@ -12818,7 +13091,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>R006接入S001：法人金额政策、具名/顺序/职责分离、材料逐票关联与内容待核实、版本化审批及操作留痕；335业务/184浏览器通过。非生产鉴权、验真或防篡改，无新依赖或独立R006页。</t>
+          <t>R007接入S001：法人/部门/费用/月预算、三模式、精确预占释放结转、R006具名额外授权及流水/最终复查证据；365业务/193浏览器通过，最后15预算及106统一规则补测通过。无独立网站/新依赖；非生产事务或多人并发。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record R008 delivery and refresh feature history workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$42</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$181</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$186</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H41" headerRowCount="1">
-  <autoFilter ref="A5:H41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H42" headerRowCount="1">
+  <autoFilter ref="A5:H42"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L181" headerRowCount="1">
-  <autoFilter ref="A5:L181"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L186" headerRowCount="1">
+  <autoFilter ref="A5:L186"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-31  |  已交付 36 个阶段、176 项内容  |  当前功能版本 R007预算额度控制  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-31  |  已交付 37 个阶段、181 项内容  |  当前功能版本 R008规则配置中心  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1950,6 +1950,42 @@
       <c r="H41" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/5cc6fb4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="74" customHeight="1">
+      <c r="A42" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>R008规则配置中心</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>统一规则草稿、真实模拟、版本发布与多法人追溯</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>397项业务/203项全量浏览器通过；最终R00810条页面补测及生产同构400→450、旧快照、零预算/审批副作用、390px验证通过；R00832项模型用例覆盖T001–T025。</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/db067c8</t>
         </is>
       </c>
     </row>
@@ -1996,6 +2032,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId37"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2009,7 +2046,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId38"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2021,7 +2058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L181"/>
+  <dimension ref="A1:L186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12326,6 +12363,296 @@
       <c r="L181" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/R007-费用预算与额度验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="88" customHeight="1">
+      <c r="A182" s="5" t="n">
+        <v>177</v>
+      </c>
+      <c r="B182" s="5" t="inlineStr">
+        <is>
+          <t>R008规则配置中心</t>
+        </is>
+      </c>
+      <c r="C182" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D182" s="5" t="inlineStr">
+        <is>
+          <t>统一规则管理</t>
+        </is>
+      </c>
+      <c r="E182" s="5" t="inlineStr">
+        <is>
+          <t>七规则列表、中文参数、集团/法人、业务日期和未来生效</t>
+        </is>
+      </c>
+      <c r="F182" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G182" s="5" t="inlineStr">
+        <is>
+          <t>财务可在明确范围维护制度</t>
+        </is>
+      </c>
+      <c r="H182" s="5" t="inlineStr">
+        <is>
+          <t>审核规则 / 规则管理中心</t>
+        </is>
+      </c>
+      <c r="I182" s="5" t="inlineStr">
+        <is>
+          <t>显式导入现有配置，复制草稿不影响正式规则</t>
+        </is>
+      </c>
+      <c r="J182" s="5" t="inlineStr">
+        <is>
+          <t>397项业务/203项全量浏览器通过；最终R00810条页面补测及生产同构400→450、旧快照、零预算/审批副作用、390px验证通过；R00832项模型用例覆盖T001–T025。</t>
+        </is>
+      </c>
+      <c r="K182" s="5" t="inlineStr">
+        <is>
+          <t>新增城市/复杂政策行用结构化参数，非任意脚本</t>
+        </is>
+      </c>
+      <c r="L182" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R008-规则管理中心验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="88" customHeight="1">
+      <c r="A183" s="5" t="n">
+        <v>178</v>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>R008规则配置中心</t>
+        </is>
+      </c>
+      <c r="C183" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D183" s="5" t="inlineStr">
+        <is>
+          <t>真实策略接入</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>R001–R007标准、查重处理、部分报销、票种、科目、审批附件与预算策略</t>
+        </is>
+      </c>
+      <c r="F183" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G183" s="5" t="inlineStr">
+        <is>
+          <t>页面参数真实影响同一引擎，无独立工具</t>
+        </is>
+      </c>
+      <c r="H183" s="5" t="inlineStr">
+        <is>
+          <t>同一报销单 / 七规则报告</t>
+        </is>
+      </c>
+      <c r="I183" s="5" t="inlineStr">
+        <is>
+          <t>400→450使430申请从超30转通过；不同法人450/350</t>
+        </is>
+      </c>
+      <c r="J183" s="5" t="inlineStr">
+        <is>
+          <t>397项业务/203项全量浏览器通过；最终R00810条页面补测及生产同构400→450、旧快照、零预算/审批副作用、390px验证通过；R00832项模型用例覆盖T001–T025。</t>
+        </is>
+      </c>
+      <c r="K183" s="5" t="inlineStr">
+        <is>
+          <t>唯一标识/精度/币种不开放；无票特批尚无</t>
+        </is>
+      </c>
+      <c r="L183" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R008-规则管理中心验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="88" customHeight="1">
+      <c r="A184" s="5" t="n">
+        <v>179</v>
+      </c>
+      <c r="B184" s="5" t="inlineStr">
+        <is>
+          <t>R008规则配置中心</t>
+        </is>
+      </c>
+      <c r="C184" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D184" s="5" t="inlineStr">
+        <is>
+          <t>发布与恢复</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>校验、真实新旧模拟、二次确认、版本差异、复制历史回滚和草稿归档</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G184" s="5" t="inlineStr">
+        <is>
+          <t>降低错误制度直接影响业务的风险</t>
+        </is>
+      </c>
+      <c r="H184" s="5" t="inlineStr">
+        <is>
+          <t>规则详情 / 模拟 / 版本历史</t>
+        </is>
+      </c>
+      <c r="I184" s="5" t="inlineStr">
+        <is>
+          <t>先模拟再发布；未来策略不提前接管；旧版不可覆盖</t>
+        </is>
+      </c>
+      <c r="J184" s="5" t="inlineStr">
+        <is>
+          <t>397项业务/203项全量浏览器通过；最终R00810条页面补测及生产同构400→450、旧快照、零预算/审批副作用、390px验证通过；R00832项模型用例覆盖T001–T025。</t>
+        </is>
+      </c>
+      <c r="K184" s="5" t="inlineStr">
+        <is>
+          <t>本地演示权限、无发布会签和后端事务</t>
+        </is>
+      </c>
+      <c r="L184" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R008-规则管理中心验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="88" customHeight="1">
+      <c r="A185" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>R008规则配置中心</t>
+        </is>
+      </c>
+      <c r="C185" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>追溯与内控</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>原历史快照、在途R006锁定、R007策略流水分离、故障保存及追加日志</t>
+        </is>
+      </c>
+      <c r="F185" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t>保留旧依据，模拟不消耗预算</t>
+        </is>
+      </c>
+      <c r="H185" s="5" t="inlineStr">
+        <is>
+          <t>审核历史 / 预算 / 配置日志</t>
+        </is>
+      </c>
+      <c r="I185" s="5" t="inlineStr">
+        <is>
+          <t>旧430单保持超30；预算85%时80→90预警不同但流水不变</t>
+        </is>
+      </c>
+      <c r="J185" s="5" t="inlineStr">
+        <is>
+          <t>397项业务/203项全量浏览器通过；最终R00810条页面补测及生产同构400→450、旧快照、零预算/审批副作用、390px验证通过；R00832项模型用例覆盖T001–T025。</t>
+        </is>
+      </c>
+      <c r="K185" s="5" t="inlineStr">
+        <is>
+          <t>日志可被本地用户修改；无正式冲销或完整备份恢复</t>
+        </is>
+      </c>
+      <c r="L185" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R008-规则管理中心验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="88" customHeight="1">
+      <c r="A186" s="5" t="n">
+        <v>181</v>
+      </c>
+      <c r="B186" s="5" t="inlineStr">
+        <is>
+          <t>R008规则配置中心</t>
+        </is>
+      </c>
+      <c r="C186" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D186" s="5" t="inlineStr">
+        <is>
+          <t>产品交付与验证</t>
+        </is>
+      </c>
+      <c r="E186" s="5" t="inlineStr">
+        <is>
+          <t>技术检查、产品需求、14道面试问答、演示、验收及功能Excel</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G186" s="5" t="inlineStr">
+        <is>
+          <t>支持完整演示和连续项目复盘</t>
+        </is>
+      </c>
+      <c r="H186" s="5" t="inlineStr">
+        <is>
+          <t>R008文档 / 同一主网站</t>
+        </is>
+      </c>
+      <c r="I186" s="5" t="inlineStr">
+        <is>
+          <t>完整新单→七规则→材料具名审批→财务批准→一次预算结转</t>
+        </is>
+      </c>
+      <c r="J186" s="5" t="inlineStr">
+        <is>
+          <t>397项业务/203项全量浏览器通过；最终R00810条页面补测及生产同构400→450、旧快照、零预算/审批副作用、390px验证通过；R00832项模型用例覆盖T001–T025。</t>
+        </is>
+      </c>
+      <c r="K186" s="5" t="inlineStr">
+        <is>
+          <t>无新增依赖、外部AI或虚构企业收益；非200人正式上线</t>
+        </is>
+      </c>
+      <c r="L186" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R008-规则管理中心验收.md</t>
         </is>
       </c>
     </row>
@@ -12512,6 +12839,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId174"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId175"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L184" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L185" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L186" r:id="rId181"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12525,7 +12857,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId177"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId182"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12624,7 +12956,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>多法人与预算维度扩展评估</t>
+          <t>预算多费用明细与项目维度评估</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -12634,12 +12966,12 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>已完成单企业部门/月独立预算和新增硬控，尚无多法人、项目/费用类型预算及并发控制</t>
+          <t>R007已完成法人/部门/费用类型/月预算及事件流水，尚无单据多预算分摊、项目维度或后端并发事务</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>按真实任务反馈评估法人/项目/类型归属和跨主体口径，再设计后端预算事务</t>
+          <t>依据试点需求评估费用行分摊、项目主数据和后端占用事务</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -12649,7 +12981,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>v0.26仅交付单企业部门/月度；今天先演练与答辩，扩展未计为已完成</t>
+          <t>R007真实额度控制及R008策略版本已交付；多预算分摊与正式多人事务不计为已完成</t>
         </is>
       </c>
     </row>
@@ -12824,7 +13156,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>规则适用范围与核对策略评估</t>
+          <t>部门项目多层规则与授权豁免评估</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -12834,7 +13166,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>已交付逐项核对及差旅城市/人员职级制度，尚无按组织部门的通用制度适用范围或豁免机制</t>
+          <t>R008已完成集团/法人完整配置、模拟发布与历史快照；尚无部门/项目多层继承或无票授权豁免</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -12849,7 +13181,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>v0.25完成逐项核对、v0.28完成差旅城市职级制度；通用组织适用与豁免尚未实现</t>
+          <t>保留R008两层优先级与原内控；新范围和豁免须先明确授权责任及冲突规则，不把核查意见作为豁免</t>
         </is>
       </c>
     </row>
@@ -13091,7 +13423,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>R007接入S001：法人/部门/费用/月预算、三模式、精确预占释放结转、R006具名额外授权及流水/最终复查证据；365业务/193浏览器通过，最后15预算及106统一规则补测通过。无独立网站/新依赖；非生产事务或多人并发。</t>
+          <t>R008接入原七规则：集团/法人完整制度、草稿校验/真实模拟/二次发布、未来生效、历史快照、在途锁定及预算策略分离；397业务/203全量浏览器通过，最后10项R008与导出网页同构验证通过。无新网站或依赖；非生产授权、事务或防篡改。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record R009 demo delivery and pending real model integration
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,11 +14,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$43</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$186</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$191</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'使用与维护'!$A$5:$B$17</definedName>
   </definedNames>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H42" headerRowCount="1">
-  <autoFilter ref="A5:H42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H43" headerRowCount="1">
+  <autoFilter ref="A5:H43"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L186" headerRowCount="1">
-  <autoFilter ref="A5:L186"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L191" headerRowCount="1">
+  <autoFilter ref="A5:L191"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -264,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H12" headerRowCount="1">
-  <autoFilter ref="A5:H12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Roadmap" displayName="Roadmap" ref="A5:H13" headerRowCount="1">
+  <autoFilter ref="A5:H13"/>
   <tableColumns count="8">
     <tableColumn id="1" name="顺序"/>
     <tableColumn id="2" name="优先级"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-31  |  已交付 37 个阶段、181 项内容  |  当前功能版本 R008规则配置中心  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-31  |  已交付 38 个阶段、186 项内容  |  当前功能版本 R009辅助分析演示  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -1986,6 +1986,42 @@
       <c r="H42" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/db067c8</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="74" customHeight="1">
+      <c r="A43" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>R009辅助分析演示</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>本地辅助分析、证据与人工反馈闭环（非真实模型）</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>433项业务/214项全量浏览器通过；最后R00911项页面复测及静态/-/产物验证通过，财务JSON不变、零预算/审批副作用、无外部分析请求。仅演示；真实模型未接入/未评测。</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/931463d</t>
         </is>
       </c>
     </row>
@@ -2033,6 +2069,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId38"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2046,7 +2083,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId38"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2058,7 +2095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L186"/>
+  <dimension ref="A1:L191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12653,6 +12690,296 @@
       <c r="L186" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/R008-规则管理中心验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="88" customHeight="1">
+      <c r="A187" s="5" t="n">
+        <v>182</v>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>R009辅助分析演示</t>
+        </is>
+      </c>
+      <c r="C187" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D187" s="5" t="inlineStr">
+        <is>
+          <t>脱敏上下文与证据</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>当前单据版本/七规则批次白名单、原文与真实制度引用、结构和数值校验</t>
+        </is>
+      </c>
+      <c r="F187" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
+          <t>保护依据及财务控制边界</t>
+        </is>
+      </c>
+      <c r="H187" s="5" t="inlineStr">
+        <is>
+          <t>原报销详情 / 辅助分析</t>
+        </is>
+      </c>
+      <c r="I187" s="5" t="inlineStr">
+        <is>
+          <t>虚构第12条制度、无依据准确率/原文和工具操作被拒绝</t>
+        </is>
+      </c>
+      <c r="J187" s="5" t="inlineStr">
+        <is>
+          <t>433项业务/214项全量浏览器通过；最后R00911项页面复测及静态/-/产物验证通过，财务JSON不变、零预算/审批副作用、无外部分析请求。仅演示；真实模型未接入/未评测。</t>
+        </is>
+      </c>
+      <c r="K187" s="5" t="inlineStr">
+        <is>
+          <t>证据存在不保证任意语义正确；仅模拟或脱敏资料</t>
+        </is>
+      </c>
+      <c r="L187" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R009-AI辅助分析验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="88" customHeight="1">
+      <c r="A188" s="5" t="n">
+        <v>183</v>
+      </c>
+      <c r="B188" s="5" t="inlineStr">
+        <is>
+          <t>R009辅助分析演示</t>
+        </is>
+      </c>
+      <c r="C188" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D188" s="5" t="inlineStr">
+        <is>
+          <t>本地演示分析</t>
+        </is>
+      </c>
+      <c r="E188" s="5" t="inlineStr">
+        <is>
+          <t>个人用途、模糊说明、个人延住与显式虚构比较样本，原异常单独汇总</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G188" s="5" t="inlineStr">
+        <is>
+          <t>演示辅助建议如何协助财务核实</t>
+        </is>
+      </c>
+      <c r="H188" s="5" t="inlineStr">
+        <is>
+          <t>同一单据七规则之后</t>
+        </is>
+      </c>
+      <c r="I188" s="5" t="inlineStr">
+        <is>
+          <t>3晚800个人延住需核水单；2晚不推断已报第三晚；非住宿不取遗留明细</t>
+        </is>
+      </c>
+      <c r="J188" s="5" t="inlineStr">
+        <is>
+          <t>433项业务/214项全量浏览器通过；最后R00911项页面复测及静态/-/产物验证通过，财务JSON不变、零预算/审批副作用、无外部分析请求。仅演示；真实模型未接入/未评测。</t>
+        </is>
+      </c>
+      <c r="K188" s="5" t="inlineStr">
+        <is>
+          <t>关键词/预设模板，未调用大模型，不宣称模型识别准确率</t>
+        </is>
+      </c>
+      <c r="L188" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R009-AI辅助分析验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="88" customHeight="1">
+      <c r="A189" s="5" t="n">
+        <v>184</v>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>R009辅助分析演示</t>
+        </is>
+      </c>
+      <c r="C189" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D189" s="5" t="inlineStr">
+        <is>
+          <t>人工反馈与统计</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>有效/误报/待补/忽略/未复核、人工独立发现、最后标签分母及关联原财务处理</t>
+        </is>
+      </c>
+      <c r="F189" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G189" s="5" t="inlineStr">
+        <is>
+          <t>形成可审查反馈，不自动训练或改规则</t>
+        </is>
+      </c>
+      <c r="H189" s="5" t="inlineStr">
+        <is>
+          <t>风险卡片 / 分析历史 / 财务工作台统计</t>
+        </is>
+      </c>
+      <c r="I189" s="5" t="inlineStr">
+        <is>
+          <t>误报反馈追加，人工发现不计AI命中，无完整真值不算漏报率</t>
+        </is>
+      </c>
+      <c r="J189" s="5" t="inlineStr">
+        <is>
+          <t>433项业务/214项全量浏览器通过；最后R00911项页面复测及静态/-/产物验证通过，财务JSON不变、零预算/审批副作用、无外部分析请求。仅演示；真实模型未接入/未评测。</t>
+        </is>
+      </c>
+      <c r="K189" s="5" t="inlineStr">
+        <is>
+          <t>重复/过期批次均计提示统计；无真实成本/效率收益</t>
+        </is>
+      </c>
+      <c r="L189" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R009-AI辅助分析验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="88" customHeight="1">
+      <c r="A190" s="5" t="n">
+        <v>185</v>
+      </c>
+      <c r="B190" s="5" t="inlineStr">
+        <is>
+          <t>R009辅助分析演示</t>
+        </is>
+      </c>
+      <c r="C190" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D190" s="5" t="inlineStr">
+        <is>
+          <t>执行与设置生命周期</t>
+        </is>
+      </c>
+      <c r="E190" s="5" t="inlineStr">
+        <is>
+          <t>异步、缓存复用、追加重跑、过期、取消超时中断及保存重试，R008同页AI设置版本</t>
+        </is>
+      </c>
+      <c r="F190" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G190" s="5" t="inlineStr">
+        <is>
+          <t>AI故障不阻断原规则或财务审核</t>
+        </is>
+      </c>
+      <c r="H190" s="5" t="inlineStr">
+        <is>
+          <t>原详情 / R008内AI设置扩展</t>
+        </is>
+      </c>
+      <c r="I190" s="5" t="inlineStr">
+        <is>
+          <t>超时仍可完成真实原财务批准与一次预算结转；保存失败不清财务意见</t>
+        </is>
+      </c>
+      <c r="J190" s="5" t="inlineStr">
+        <is>
+          <t>433项业务/214项全量浏览器通过；最后R00911项页面复测及静态/-/产物验证通过，财务JSON不变、零预算/审批副作用、无外部分析请求。仅演示；真实模型未接入/未评测。</t>
+        </is>
+      </c>
+      <c r="K190" s="5" t="inlineStr">
+        <is>
+          <t>独立AI记录非第二套报销；浏览器权限/并发/备份仍非生产</t>
+        </is>
+      </c>
+      <c r="L190" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R009-AI辅助分析验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="88" customHeight="1">
+      <c r="A191" s="5" t="n">
+        <v>186</v>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>R009辅助分析演示</t>
+        </is>
+      </c>
+      <c r="C191" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>演示与交付验证</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>技术现状、产品需求、15道问答、五类演示、设计预期标签、验收与Excel</t>
+        </is>
+      </c>
+      <c r="F191" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>清楚区分演示产品闭环与待接入的真实AI</t>
+        </is>
+      </c>
+      <c r="H191" s="5" t="inlineStr">
+        <is>
+          <t>R009四份交付文档 / 既有主网站</t>
+        </is>
+      </c>
+      <c r="I191" s="5" t="inlineStr">
+        <is>
+          <t>完整七规则→演示风险→证据→反馈→历史，失败不动财务对象</t>
+        </is>
+      </c>
+      <c r="J191" s="5" t="inlineStr">
+        <is>
+          <t>433项业务/214项全量浏览器通过；最后R00911项页面复测及静态/-/产物验证通过，财务JSON不变、零预算/审批副作用、无外部分析请求。仅演示；真实模型未接入/未评测。</t>
+        </is>
+      </c>
+      <c r="K191" s="5" t="inlineStr">
+        <is>
+          <t>真实模型服务端、供应商/费用/外发授权及独立财务评测未完成</t>
+        </is>
+      </c>
+      <c r="L191" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/R009-AI辅助分析验收.md</t>
         </is>
       </c>
     </row>
@@ -12844,6 +13171,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L184" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L185" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L186" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L187" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L188" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L189" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L190" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L191" r:id="rId186"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12857,7 +13189,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId182"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId187"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12869,7 +13201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13222,6 +13554,46 @@
       <c r="H12" s="5" t="inlineStr">
         <is>
           <t>新账号权限、费用或真实财务资料必须按既有授权边界单独确认；本轮仅完成差旅规则，无正式企业上线承诺</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="100" customHeight="1">
+      <c r="A13" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>R009真实模型服务端接入与独立财务评估</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>尚未接入</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>R009目前只有明确标注的本地演示模板及反馈闭环，没有真实提供商、服务端或独立裁定的模型效果数据</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>服务端保密/授权/脱敏确认/超时限流用量、提供商保留策略及真实模型输出评测；不开放审批工具</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>先用虚构独立样本验证接口、证据和失败隔离；明确费用与外发范围授权，真实身份/数据权限和独立财务标注后才评估真实业务试点</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>真实账号权限、费用或真实财务资料必须按既有授权边界确认；不把本地故障模拟或模板测试当真实模型评测</t>
         </is>
       </c>
     </row>
@@ -13423,7 +13795,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>R008接入原七规则：集团/法人完整制度、草稿校验/真实模拟/二次发布、未来生效、历史快照、在途锁定及预算策略分离；397业务/203全量浏览器通过，最后10项R008与导出网页同构验证通过。无新网站或依赖；非生产授权、事务或防篡改。</t>
+          <t>R009本地演示接入原系统：脱敏上下文/证据校验、预设风险/原规则解释、人工反馈及统计、追加历史/过期、超时和保存故障隔离、R008内AI设置版本。433业务/214全量浏览器及最后11项R009、静态产物验证通过。真实大模型尚未接入，不写识别率/成本/效率成果。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record R010 evidence and update ordered feature workbook
</commit_message>
<xml_diff>
--- a/deliverables/qingbao-feature-history.xlsx
+++ b/deliverables/qingbao-feature-history.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'阶段总览'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'阶段总览'!$A$5:$H$44</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'历史新增明细'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$191</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'历史新增明细'!$A$5:$L$196</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'下一步计划'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'下一步计划'!$A$5:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'使用与维护'!$1:$5</definedName>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H43" headerRowCount="1">
-  <autoFilter ref="A5:H43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StageOverview" displayName="StageOverview" ref="A5:H44" headerRowCount="1">
+  <autoFilter ref="A5:H44"/>
   <tableColumns count="8">
     <tableColumn id="1" name="阶段顺序"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -243,8 +243,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L191" headerRowCount="1">
-  <autoFilter ref="A5:L191"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FeatureHistory" displayName="FeatureHistory" ref="A5:L196" headerRowCount="1">
+  <autoFilter ref="A5:L196"/>
   <tableColumns count="12">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="版本/阶段"/>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -611,7 +611,7 @@
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>更新：2026-10-31  |  已交付 38 个阶段、186 项内容  |  当前功能版本 R009辅助分析演示  |  后续计划不计入已完成</t>
+          <t>更新：2026-10-31  |  已交付 39 个阶段、191 项内容  |  当前功能版本 R010开源发票识别  |  后续计划不计入已完成</t>
         </is>
       </c>
     </row>
@@ -2022,6 +2022,42 @@
       <c r="H43" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/commit/931463d</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="74" customHeight="1">
+      <c r="A44" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>R010开源发票识别</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>开源CPU识别、PDF文字层及原表单核对闭环</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>448项业务、214项既有浏览器、4项实际本机OCR浏览器、8项Python传输保护通过；12份虚构样票逐字段/耗时实测，静态/-/PDF及Tesseract通过。非真实发票准确率。</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/commit/2757347</t>
         </is>
       </c>
     </row>
@@ -2070,6 +2106,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId39"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2083,7 +2120,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId40"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2095,7 +2132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L191"/>
+  <dimension ref="A1:L196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12980,6 +13017,296 @@
       <c r="L191" s="8" t="inlineStr">
         <is>
           <t>https://github.com/Jameyan42/-/blob/main/docs/R009-AI辅助分析验收.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="88" customHeight="1">
+      <c r="A192" s="5" t="n">
+        <v>187</v>
+      </c>
+      <c r="B192" s="5" t="inlineStr">
+        <is>
+          <t>R010开源发票识别</t>
+        </is>
+      </c>
+      <c r="C192" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D192" s="5" t="inlineStr">
+        <is>
+          <t>开源选型与本机服务</t>
+        </is>
+      </c>
+      <c r="E192" s="5" t="inlineStr">
+        <is>
+          <t>三项指定开源项目调研、RapidOCR/Paddle模型CPU集成和安全本机接口</t>
+        </is>
+      </c>
+      <c r="F192" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G192" s="5" t="inlineStr">
+        <is>
+          <t>复用成熟模型且无需付费外发</t>
+        </is>
+      </c>
+      <c r="H192" s="5" t="inlineStr">
+        <is>
+          <t>既有主网站统一报销单 / 本机127.0.0.1:8766</t>
+        </is>
+      </c>
+      <c r="I192" s="5" t="inlineStr">
+        <is>
+          <t>运行8766本机服务，查看实际引擎及健康状态</t>
+        </is>
+      </c>
+      <c r="J192" s="5" t="inlineStr">
+        <is>
+          <t>448项业务、214项既有浏览器、4项实际本机OCR浏览器、8项Python传输保护通过；12份虚构样票逐字段/耗时实测，静态/-/PDF及Tesseract通过。非真实发票准确率。</t>
+        </is>
+      </c>
+      <c r="K192" s="5" t="inlineStr">
+        <is>
+          <t>仅合成样票，真实脱敏票准确率/Windows实机未验证；Pages仅浏览器后备；Paddle3原生权重源403；不等于税务验真或正式企业上线</t>
+        </is>
+      </c>
+      <c r="L192" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/r010/TEST_REPORT.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="88" customHeight="1">
+      <c r="A193" s="5" t="n">
+        <v>188</v>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>R010开源发票识别</t>
+        </is>
+      </c>
+      <c r="C193" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>PDF与结构化识别</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>文字层优先、扫描件OCR、票号日期买卖方税号及净额税额合计项目</t>
+        </is>
+      </c>
+      <c r="F193" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="inlineStr">
+        <is>
+          <t>减少重复录入，缺失不补零不倒推</t>
+        </is>
+      </c>
+      <c r="H193" s="5" t="inlineStr">
+        <is>
+          <t>既有主网站统一报销单 / 本机127.0.0.1:8766</t>
+        </is>
+      </c>
+      <c r="I193" s="5" t="inlineStr">
+        <is>
+          <t>文字PDF零模型请求，扫描件走实际模型，查看逐字段JSON</t>
+        </is>
+      </c>
+      <c r="J193" s="5" t="inlineStr">
+        <is>
+          <t>448项业务、214项既有浏览器、4项实际本机OCR浏览器、8项Python传输保护通过；12份虚构样票逐字段/耗时实测，静态/-/PDF及Tesseract通过。非真实发票准确率。</t>
+        </is>
+      </c>
+      <c r="K193" s="5" t="inlineStr">
+        <is>
+          <t>仅合成样票，真实脱敏票准确率/Windows实机未验证；Pages仅浏览器后备；Paddle3原生权重源403；不等于税务验真或正式企业上线</t>
+        </is>
+      </c>
+      <c r="L193" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/r010/TEST_REPORT.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="88" customHeight="1">
+      <c r="A194" s="5" t="n">
+        <v>189</v>
+      </c>
+      <c r="B194" s="5" t="inlineStr">
+        <is>
+          <t>R010开源发票识别</t>
+        </is>
+      </c>
+      <c r="C194" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D194" s="5" t="inlineStr">
+        <is>
+          <t>票面人工核对</t>
+        </is>
+      </c>
+      <c r="E194" s="5" t="inlineStr">
+        <is>
+          <t>原始识别/原件哈希/人工修正和确认快照、置信度提示</t>
+        </is>
+      </c>
+      <c r="F194" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G194" s="5" t="inlineStr">
+        <is>
+          <t>方便财务对照原件并保留来源</t>
+        </is>
+      </c>
+      <c r="H194" s="5" t="inlineStr">
+        <is>
+          <t>既有主网站统一报销单 / 本机127.0.0.1:8766</t>
+        </is>
+      </c>
+      <c r="I194" s="5" t="inlineStr">
+        <is>
+          <t>1060修正1061，保存刷新查看两种值与时间</t>
+        </is>
+      </c>
+      <c r="J194" s="5" t="inlineStr">
+        <is>
+          <t>448项业务、214项既有浏览器、4项实际本机OCR浏览器、8项Python传输保护通过；12份虚构样票逐字段/耗时实测，静态/-/PDF及Tesseract通过。非真实发票准确率。</t>
+        </is>
+      </c>
+      <c r="K194" s="5" t="inlineStr">
+        <is>
+          <t>仅合成样票，真实脱敏票准确率/Windows实机未验证；Pages仅浏览器后备；Paddle3原生权重源403；不等于税务验真或正式企业上线</t>
+        </is>
+      </c>
+      <c r="L194" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/r010/TEST_REPORT.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="88" customHeight="1">
+      <c r="A195" s="5" t="n">
+        <v>190</v>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>R010开源发票识别</t>
+        </is>
+      </c>
+      <c r="C195" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D195" s="5" t="inlineStr">
+        <is>
+          <t>既有审核联动</t>
+        </is>
+      </c>
+      <c r="E195" s="5" t="inlineStr">
+        <is>
+          <t>识别及票面编辑后自动调用R002/R003/R004预审</t>
+        </is>
+      </c>
+      <c r="F195" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G195" s="5" t="inlineStr">
+        <is>
+          <t>沿用已有规则、正式审批和预算保护</t>
+        </is>
+      </c>
+      <c r="H195" s="5" t="inlineStr">
+        <is>
+          <t>既有主网站统一报销单 / 本机127.0.0.1:8766</t>
+        </is>
+      </c>
+      <c r="I195" s="5" t="inlineStr">
+        <is>
+          <t>相同两票重复提醒，金额差异及抬头不足明确提示</t>
+        </is>
+      </c>
+      <c r="J195" s="5" t="inlineStr">
+        <is>
+          <t>448项业务、214项既有浏览器、4项实际本机OCR浏览器、8项Python传输保护通过；12份虚构样票逐字段/耗时实测，静态/-/PDF及Tesseract通过。非真实发票准确率。</t>
+        </is>
+      </c>
+      <c r="K195" s="5" t="inlineStr">
+        <is>
+          <t>仅合成样票，真实脱敏票准确率/Windows实机未验证；Pages仅浏览器后备；Paddle3原生权重源403；不等于税务验真或正式企业上线</t>
+        </is>
+      </c>
+      <c r="L195" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/r010/TEST_REPORT.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="88" customHeight="1">
+      <c r="A196" s="5" t="n">
+        <v>191</v>
+      </c>
+      <c r="B196" s="5" t="inlineStr">
+        <is>
+          <t>R010开源发票识别</t>
+        </is>
+      </c>
+      <c r="C196" s="6" t="n">
+        <v>46326</v>
+      </c>
+      <c r="D196" s="5" t="inlineStr">
+        <is>
+          <t>验证与交付</t>
+        </is>
+      </c>
+      <c r="E196" s="5" t="inlineStr">
+        <is>
+          <t>12份虚构样票、逐字段CSV/JSON、实际页面测试、启动说明和Excel</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="G196" s="5" t="inlineStr">
+        <is>
+          <t>交付可复核证据，明确真实准确率与部署边界</t>
+        </is>
+      </c>
+      <c r="H196" s="5" t="inlineStr">
+        <is>
+          <t>既有主网站统一报销单 / 本机127.0.0.1:8766</t>
+        </is>
+      </c>
+      <c r="I196" s="5" t="inlineStr">
+        <is>
+          <t>查看选型/验收/样票报告，区分在线后备和本机PP-OCR</t>
+        </is>
+      </c>
+      <c r="J196" s="5" t="inlineStr">
+        <is>
+          <t>448项业务、214项既有浏览器、4项实际本机OCR浏览器、8项Python传输保护通过；12份虚构样票逐字段/耗时实测，静态/-/PDF及Tesseract通过。非真实发票准确率。</t>
+        </is>
+      </c>
+      <c r="K196" s="5" t="inlineStr">
+        <is>
+          <t>仅合成样票，真实脱敏票准确率/Windows实机未验证；Pages仅浏览器后备；Paddle3原生权重源403；不等于税务验真或正式企业上线</t>
+        </is>
+      </c>
+      <c r="L196" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Jameyan42/-/blob/main/docs/r010/TEST_REPORT.md</t>
         </is>
       </c>
     </row>
@@ -13176,6 +13503,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L189" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L190" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L191" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L192" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L193" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L194" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L195" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L196" r:id="rId191"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13189,7 +13521,7 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId187"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId192"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>